<commit_message>
script: inattentional-blindness (build blocked 2026-10-12, not scheduled)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P6Jtw3xpFhoxQhHQCSJPDP
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -2895,7 +2895,11 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K27" s="10" t="n"/>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>inattentional-blindness</t>
+        </is>
+      </c>
       <c r="L27" s="11" t="n"/>
       <c r="M27" s="5">
         <f>IF(L27="","",TEXT(L27,"ddd"))</f>
@@ -2904,7 +2908,11 @@
       <c r="N27" s="10" t="n"/>
       <c r="O27" s="10" t="n"/>
       <c r="P27" s="10" t="n"/>
-      <c r="Q27" s="10" t="n"/>
+      <c r="Q27" s="10" t="inlineStr">
+        <is>
+          <t>Simons &amp; Chabris 1999, Perception 28(9):1059-1074, doi:10.1068/p281059; gorilla condition 56% missed / 44% noticed (overall 46% missed, incl. umbrella woman).</t>
+        </is>
+      </c>
       <c r="R27" s="10" t="n"/>
       <c r="S27" s="12" t="n"/>
       <c r="T27" s="10" t="n"/>
@@ -2945,7 +2953,11 @@
         <f>IF(N(AC27)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC27&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC27&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN27" s="10" t="n"/>
+      <c r="AN27" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-12: script.json written and verified; build blocked (run could not execute repo build scripts), not scheduled. Status left at Idea so the next run builds it.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="5" t="n">

</xml_diff>

<commit_message>
Visual styles: 15 looks adapted from lemo-opuscar (MIT), assigned per idea in the tracker
- _looks.ts: grounds, palettes, OFL fonts, text treatments, title lock-ups, crowd/avatar styling, chrome
- template plates render in the script's look; tracker gets a Visual style column, Looks sheet and Summary block
- runbook: scripts carry no + look; weekly review compares and tunes looks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -4,7 +4,8 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -66,7 +67,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="33">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +77,156 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF303030"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0A0A0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF4D12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F7F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2A5CB3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F1E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB2182B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAE9E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE30613"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1E7D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8417F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4EEE2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF48B0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF18336B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6453A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B0906"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B0C10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB7F34A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6A4BD8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD23F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2C14E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4572E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B1714"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2A52A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBF5E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2725B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2B1D4F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD447"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F2EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC8363A"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,6 +282,36 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -231,6 +412,11 @@
     <comment ref="I4" authorId="0" shapeId="0">
       <text>
         <t>Blue = filled in by the daily pipeline (you can edit too). Black = formulas. Priority: lowest number with Status 'Idea' is made next — renumber to reorder.</t>
+      </text>
+    </comment>
+    <comment ref="AO5" authorId="0" shapeId="0">
+      <text>
+        <t>The look this Short is built in (see the Looks sheet). Change it before the idea is made to switch styles; the daily pipeline copies it into the script.</t>
       </text>
     </comment>
   </commentList>
@@ -451,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AN105"/>
+  <dimension ref="A2:AO105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -494,6 +680,7 @@
     <col width="12" customWidth="1" min="38" max="38"/>
     <col width="11" customWidth="1" min="39" max="39"/>
     <col width="50" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -558,6 +745,11 @@
           <t>LEARNING</t>
         </is>
       </c>
+      <c r="AO4" s="9" t="inlineStr">
+        <is>
+          <t>STYLE</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -758,6 +950,11 @@
       <c r="AN5" s="8" t="inlineStr">
         <is>
           <t>Lesson / notes</t>
+        </is>
+      </c>
+      <c r="AO5" s="8" t="inlineStr">
+        <is>
+          <t>Visual style</t>
         </is>
       </c>
     </row>
@@ -885,6 +1082,11 @@
           <t>Pilot: 16:9 horizontal, YouTube only — not comparable with the vertical Shorts.</t>
         </is>
       </c>
+      <c r="AO6" s="10" t="inlineStr">
+        <is>
+          <t>pixel-lab</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="5" t="n">
@@ -982,6 +1184,11 @@
         <v/>
       </c>
       <c r="AN7" s="10" t="n"/>
+      <c r="AO7" s="10" t="inlineStr">
+        <is>
+          <t>keynote</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="5" t="n">
@@ -1079,6 +1286,11 @@
         <v/>
       </c>
       <c r="AN8" s="10" t="n"/>
+      <c r="AO8" s="10" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -1176,6 +1388,11 @@
         <v/>
       </c>
       <c r="AN9" s="10" t="n"/>
+      <c r="AO9" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -1273,6 +1490,11 @@
         <v/>
       </c>
       <c r="AN10" s="10" t="n"/>
+      <c r="AO10" s="10" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -1370,6 +1592,11 @@
         <v/>
       </c>
       <c r="AN11" s="10" t="n"/>
+      <c r="AO11" s="10" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -1467,6 +1694,11 @@
         <v/>
       </c>
       <c r="AN12" s="10" t="n"/>
+      <c r="AO12" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -1564,6 +1796,11 @@
         <v/>
       </c>
       <c r="AN13" s="10" t="n"/>
+      <c r="AO13" s="10" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="5" t="n">
@@ -1661,6 +1898,11 @@
         <v/>
       </c>
       <c r="AN14" s="10" t="n"/>
+      <c r="AO14" s="10" t="inlineStr">
+        <is>
+          <t>keynote</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -1758,6 +2000,11 @@
         <v/>
       </c>
       <c r="AN15" s="10" t="n"/>
+      <c r="AO15" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -1879,6 +2126,11 @@
         <v/>
       </c>
       <c r="AN16" s="10" t="n"/>
+      <c r="AO16" s="10" t="inlineStr">
+        <is>
+          <t>pixel-lab</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="5" t="n">
@@ -1976,6 +2228,11 @@
         <v/>
       </c>
       <c r="AN17" s="10" t="n"/>
+      <c r="AO17" s="10" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -2073,6 +2330,11 @@
         <v/>
       </c>
       <c r="AN18" s="10" t="n"/>
+      <c r="AO18" s="10" t="inlineStr">
+        <is>
+          <t>pixel-quest</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="5" t="n">
@@ -2170,6 +2432,11 @@
         <v/>
       </c>
       <c r="AN19" s="10" t="n"/>
+      <c r="AO19" s="10" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -2267,6 +2534,11 @@
         <v/>
       </c>
       <c r="AN20" s="10" t="n"/>
+      <c r="AO20" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -2364,6 +2636,11 @@
         <v/>
       </c>
       <c r="AN21" s="10" t="n"/>
+      <c r="AO21" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="5" t="n">
@@ -2461,6 +2738,11 @@
         <v/>
       </c>
       <c r="AN22" s="10" t="n"/>
+      <c r="AO22" s="10" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="5" t="n">
@@ -2558,6 +2840,11 @@
         <v/>
       </c>
       <c r="AN23" s="10" t="n"/>
+      <c r="AO23" s="10" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="5" t="n">
@@ -2655,6 +2942,11 @@
         <v/>
       </c>
       <c r="AN24" s="10" t="n"/>
+      <c r="AO24" s="10" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="5" t="n">
@@ -2752,6 +3044,11 @@
         <v/>
       </c>
       <c r="AN25" s="10" t="n"/>
+      <c r="AO25" s="10" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="5" t="n">
@@ -2849,6 +3146,11 @@
         <v/>
       </c>
       <c r="AN26" s="10" t="n"/>
+      <c r="AO26" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" s="5" t="n">
@@ -2970,6 +3272,11 @@
         <v/>
       </c>
       <c r="AN27" s="10" t="n"/>
+      <c r="AO27" s="10" t="inlineStr">
+        <is>
+          <t>pixel-lab</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="5" t="n">
@@ -3067,6 +3374,11 @@
         <v/>
       </c>
       <c r="AN28" s="10" t="n"/>
+      <c r="AO28" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="5" t="n">
@@ -3164,6 +3476,11 @@
         <v/>
       </c>
       <c r="AN29" s="10" t="n"/>
+      <c r="AO29" s="10" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="5" t="n">
@@ -3261,6 +3578,11 @@
         <v/>
       </c>
       <c r="AN30" s="10" t="n"/>
+      <c r="AO30" s="10" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" s="5" t="n">
@@ -3358,6 +3680,11 @@
         <v/>
       </c>
       <c r="AN31" s="10" t="n"/>
+      <c r="AO31" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="5" t="n">
@@ -3455,6 +3782,11 @@
         <v/>
       </c>
       <c r="AN32" s="10" t="n"/>
+      <c r="AO32" s="10" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" s="5" t="n">
@@ -3552,6 +3884,11 @@
         <v/>
       </c>
       <c r="AN33" s="10" t="n"/>
+      <c r="AO33" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="5" t="n">
@@ -3649,6 +3986,11 @@
         <v/>
       </c>
       <c r="AN34" s="10" t="n"/>
+      <c r="AO34" s="10" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="60" customHeight="1">
       <c r="A35" s="5" t="n">
@@ -3746,6 +4088,11 @@
         <v/>
       </c>
       <c r="AN35" s="10" t="n"/>
+      <c r="AO35" s="10" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="60" customHeight="1">
       <c r="A36" s="5" t="n">
@@ -3843,6 +4190,11 @@
         <v/>
       </c>
       <c r="AN36" s="10" t="n"/>
+      <c r="AO36" s="10" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="5" t="n">
@@ -3940,6 +4292,11 @@
         <v/>
       </c>
       <c r="AN37" s="10" t="n"/>
+      <c r="AO37" s="10" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="5" t="n">
@@ -4037,6 +4394,11 @@
         <v/>
       </c>
       <c r="AN38" s="10" t="n"/>
+      <c r="AO38" s="10" t="inlineStr">
+        <is>
+          <t>pixel-quest</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="5" t="n">
@@ -4134,6 +4496,11 @@
         <v/>
       </c>
       <c r="AN39" s="10" t="n"/>
+      <c r="AO39" s="10" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="60" customHeight="1">
       <c r="A40" s="5" t="n">
@@ -4231,6 +4598,11 @@
         <v/>
       </c>
       <c r="AN40" s="10" t="n"/>
+      <c r="AO40" s="10" t="inlineStr">
+        <is>
+          <t>pixel-quest</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="60" customHeight="1">
       <c r="A41" s="5" t="n">
@@ -4328,6 +4700,11 @@
         <v/>
       </c>
       <c r="AN41" s="10" t="n"/>
+      <c r="AO41" s="10" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="5" t="n">
@@ -4425,6 +4802,11 @@
         <v/>
       </c>
       <c r="AN42" s="10" t="n"/>
+      <c r="AO42" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="5" t="n">
@@ -4522,6 +4904,11 @@
         <v/>
       </c>
       <c r="AN43" s="10" t="n"/>
+      <c r="AO43" s="10" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="5" t="n">
@@ -4619,6 +5006,11 @@
         <v/>
       </c>
       <c r="AN44" s="10" t="n"/>
+      <c r="AO44" s="10" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="60" customHeight="1">
       <c r="A45" s="5" t="n">
@@ -4716,6 +5108,11 @@
         <v/>
       </c>
       <c r="AN45" s="10" t="n"/>
+      <c r="AO45" s="10" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="5" t="n">
@@ -4813,6 +5210,11 @@
         <v/>
       </c>
       <c r="AN46" s="10" t="n"/>
+      <c r="AO46" s="10" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="60" customHeight="1">
       <c r="A47" s="5" t="n">
@@ -4910,6 +5312,11 @@
         <v/>
       </c>
       <c r="AN47" s="10" t="n"/>
+      <c r="AO47" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="60" customHeight="1">
       <c r="A48" s="5" t="n">
@@ -5007,6 +5414,11 @@
         <v/>
       </c>
       <c r="AN48" s="10" t="n"/>
+      <c r="AO48" s="10" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="60" customHeight="1">
       <c r="A49" s="5" t="n">
@@ -5104,6 +5516,11 @@
         <v/>
       </c>
       <c r="AN49" s="10" t="n"/>
+      <c r="AO49" s="10" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="5" t="n">
@@ -5201,6 +5618,11 @@
         <v/>
       </c>
       <c r="AN50" s="10" t="n"/>
+      <c r="AO50" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="60" customHeight="1">
       <c r="A51" s="5" t="n">
@@ -5298,6 +5720,11 @@
         <v/>
       </c>
       <c r="AN51" s="10" t="n"/>
+      <c r="AO51" s="10" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="5" t="n">
@@ -5395,6 +5822,11 @@
         <v/>
       </c>
       <c r="AN52" s="10" t="n"/>
+      <c r="AO52" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="60" customHeight="1">
       <c r="A53" s="5" t="n">
@@ -5492,6 +5924,11 @@
         <v/>
       </c>
       <c r="AN53" s="10" t="n"/>
+      <c r="AO53" s="10" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="60" customHeight="1">
       <c r="A54" s="5" t="n">
@@ -5589,6 +6026,11 @@
         <v/>
       </c>
       <c r="AN54" s="10" t="n"/>
+      <c r="AO54" s="10" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="60" customHeight="1">
       <c r="A55" s="5" t="n">
@@ -5686,6 +6128,11 @@
         <v/>
       </c>
       <c r="AN55" s="10" t="n"/>
+      <c r="AO55" s="10" t="inlineStr">
+        <is>
+          <t>keynote</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="60" customHeight="1">
       <c r="A56" s="5" t="n">
@@ -5783,6 +6230,11 @@
         <v/>
       </c>
       <c r="AN56" s="10" t="n"/>
+      <c r="AO56" s="10" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="60" customHeight="1">
       <c r="A57" s="5" t="n">
@@ -5880,6 +6332,11 @@
         <v/>
       </c>
       <c r="AN57" s="10" t="n"/>
+      <c r="AO57" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="60" customHeight="1">
       <c r="A58" s="5" t="n">
@@ -5977,6 +6434,11 @@
         <v/>
       </c>
       <c r="AN58" s="10" t="n"/>
+      <c r="AO58" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="60" customHeight="1">
       <c r="A59" s="5" t="n">
@@ -6074,6 +6536,11 @@
         <v/>
       </c>
       <c r="AN59" s="10" t="n"/>
+      <c r="AO59" s="10" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="60" customHeight="1">
       <c r="A60" s="5" t="n">
@@ -6171,6 +6638,11 @@
         <v/>
       </c>
       <c r="AN60" s="10" t="n"/>
+      <c r="AO60" s="10" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="60" customHeight="1">
       <c r="A61" s="5" t="n">
@@ -6268,6 +6740,11 @@
         <v/>
       </c>
       <c r="AN61" s="10" t="n"/>
+      <c r="AO61" s="10" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="60" customHeight="1">
       <c r="A62" s="5" t="n">
@@ -6365,6 +6842,11 @@
         <v/>
       </c>
       <c r="AN62" s="10" t="n"/>
+      <c r="AO62" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="60" customHeight="1">
       <c r="A63" s="5" t="n">
@@ -6462,6 +6944,11 @@
         <v/>
       </c>
       <c r="AN63" s="10" t="n"/>
+      <c r="AO63" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="60" customHeight="1">
       <c r="A64" s="5" t="n">
@@ -6559,6 +7046,11 @@
         <v/>
       </c>
       <c r="AN64" s="10" t="n"/>
+      <c r="AO64" s="10" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="60" customHeight="1">
       <c r="A65" s="5" t="n">
@@ -6656,6 +7148,11 @@
         <v/>
       </c>
       <c r="AN65" s="10" t="n"/>
+      <c r="AO65" s="10" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="60" customHeight="1">
       <c r="A66" s="5" t="n">
@@ -6753,6 +7250,11 @@
         <v/>
       </c>
       <c r="AN66" s="10" t="n"/>
+      <c r="AO66" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="60" customHeight="1">
       <c r="A67" s="5" t="n">
@@ -6850,6 +7352,11 @@
         <v/>
       </c>
       <c r="AN67" s="10" t="n"/>
+      <c r="AO67" s="10" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="5" t="n">
@@ -6947,6 +7454,11 @@
         <v/>
       </c>
       <c r="AN68" s="10" t="n"/>
+      <c r="AO68" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="5" t="n">
@@ -7044,6 +7556,11 @@
         <v/>
       </c>
       <c r="AN69" s="10" t="n"/>
+      <c r="AO69" s="10" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="5" t="n">
@@ -7141,6 +7658,11 @@
         <v/>
       </c>
       <c r="AN70" s="10" t="n"/>
+      <c r="AO70" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="60" customHeight="1">
       <c r="A71" s="5" t="n">
@@ -7238,6 +7760,11 @@
         <v/>
       </c>
       <c r="AN71" s="10" t="n"/>
+      <c r="AO71" s="10" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="60" customHeight="1">
       <c r="A72" s="5" t="n">
@@ -7335,6 +7862,11 @@
         <v/>
       </c>
       <c r="AN72" s="10" t="n"/>
+      <c r="AO72" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="60" customHeight="1">
       <c r="A73" s="5" t="n">
@@ -7432,6 +7964,11 @@
         <v/>
       </c>
       <c r="AN73" s="10" t="n"/>
+      <c r="AO73" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="60" customHeight="1">
       <c r="A74" s="5" t="n">
@@ -7529,6 +8066,11 @@
         <v/>
       </c>
       <c r="AN74" s="10" t="n"/>
+      <c r="AO74" s="10" t="inlineStr">
+        <is>
+          <t>pixel-quest</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="60" customHeight="1">
       <c r="A75" s="5" t="n">
@@ -7626,6 +8168,11 @@
         <v/>
       </c>
       <c r="AN75" s="10" t="n"/>
+      <c r="AO75" s="10" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="60" customHeight="1">
       <c r="A76" s="5" t="n">
@@ -7723,6 +8270,11 @@
         <v/>
       </c>
       <c r="AN76" s="10" t="n"/>
+      <c r="AO76" s="10" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="60" customHeight="1">
       <c r="A77" s="5" t="n">
@@ -7820,6 +8372,11 @@
         <v/>
       </c>
       <c r="AN77" s="10" t="n"/>
+      <c r="AO77" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="60" customHeight="1">
       <c r="A78" s="5" t="n">
@@ -7917,6 +8474,11 @@
         <v/>
       </c>
       <c r="AN78" s="10" t="n"/>
+      <c r="AO78" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="60" customHeight="1">
       <c r="A79" s="5" t="n">
@@ -8014,6 +8576,11 @@
         <v/>
       </c>
       <c r="AN79" s="10" t="n"/>
+      <c r="AO79" s="10" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="60" customHeight="1">
       <c r="A80" s="5" t="n">
@@ -8111,6 +8678,11 @@
         <v/>
       </c>
       <c r="AN80" s="10" t="n"/>
+      <c r="AO80" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="60" customHeight="1">
       <c r="A81" s="5" t="n">
@@ -8208,6 +8780,11 @@
         <v/>
       </c>
       <c r="AN81" s="10" t="n"/>
+      <c r="AO81" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="60" customHeight="1">
       <c r="A82" s="5" t="n">
@@ -8305,6 +8882,11 @@
         <v/>
       </c>
       <c r="AN82" s="10" t="n"/>
+      <c r="AO82" s="10" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="60" customHeight="1">
       <c r="A83" s="5" t="n">
@@ -8402,6 +8984,11 @@
         <v/>
       </c>
       <c r="AN83" s="10" t="n"/>
+      <c r="AO83" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="60" customHeight="1">
       <c r="A84" s="5" t="n">
@@ -8499,6 +9086,11 @@
         <v/>
       </c>
       <c r="AN84" s="10" t="n"/>
+      <c r="AO84" s="10" t="inlineStr">
+        <is>
+          <t>pixel-quest</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="60" customHeight="1">
       <c r="A85" s="5" t="n">
@@ -8596,6 +9188,11 @@
         <v/>
       </c>
       <c r="AN85" s="10" t="n"/>
+      <c r="AO85" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="60" customHeight="1">
       <c r="A86" s="5" t="n">
@@ -8693,6 +9290,11 @@
         <v/>
       </c>
       <c r="AN86" s="10" t="n"/>
+      <c r="AO86" s="10" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="60" customHeight="1">
       <c r="A87" s="5" t="n">
@@ -8790,6 +9392,11 @@
         <v/>
       </c>
       <c r="AN87" s="10" t="n"/>
+      <c r="AO87" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="60" customHeight="1">
       <c r="A88" s="5" t="n">
@@ -8887,6 +9494,11 @@
         <v/>
       </c>
       <c r="AN88" s="10" t="n"/>
+      <c r="AO88" s="10" t="inlineStr">
+        <is>
+          <t>keynote</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="60" customHeight="1">
       <c r="A89" s="5" t="n">
@@ -8984,6 +9596,11 @@
         <v/>
       </c>
       <c r="AN89" s="10" t="n"/>
+      <c r="AO89" s="10" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="60" customHeight="1">
       <c r="A90" s="5" t="n">
@@ -9081,6 +9698,11 @@
         <v/>
       </c>
       <c r="AN90" s="10" t="n"/>
+      <c r="AO90" s="10" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="60" customHeight="1">
       <c r="A91" s="5" t="n">
@@ -9178,6 +9800,11 @@
         <v/>
       </c>
       <c r="AN91" s="10" t="n"/>
+      <c r="AO91" s="10" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="60" customHeight="1">
       <c r="A92" s="5" t="n">
@@ -9275,6 +9902,11 @@
         <v/>
       </c>
       <c r="AN92" s="10" t="n"/>
+      <c r="AO92" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="60" customHeight="1">
       <c r="A93" s="5" t="n">
@@ -9372,6 +10004,11 @@
         <v/>
       </c>
       <c r="AN93" s="10" t="n"/>
+      <c r="AO93" s="10" t="inlineStr">
+        <is>
+          <t>keynote</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="60" customHeight="1">
       <c r="A94" s="5" t="n">
@@ -9469,6 +10106,11 @@
         <v/>
       </c>
       <c r="AN94" s="10" t="n"/>
+      <c r="AO94" s="10" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="60" customHeight="1">
       <c r="A95" s="5" t="n">
@@ -9566,6 +10208,11 @@
         <v/>
       </c>
       <c r="AN95" s="10" t="n"/>
+      <c r="AO95" s="10" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="60" customHeight="1">
       <c r="A96" s="5" t="n">
@@ -9663,6 +10310,11 @@
         <v/>
       </c>
       <c r="AN96" s="10" t="n"/>
+      <c r="AO96" s="10" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="60" customHeight="1">
       <c r="A97" s="5" t="n">
@@ -9760,6 +10412,11 @@
         <v/>
       </c>
       <c r="AN97" s="10" t="n"/>
+      <c r="AO97" s="10" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="60" customHeight="1">
       <c r="A98" s="5" t="n">
@@ -9857,6 +10514,11 @@
         <v/>
       </c>
       <c r="AN98" s="10" t="n"/>
+      <c r="AO98" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="60" customHeight="1">
       <c r="A99" s="5" t="n">
@@ -9954,6 +10616,11 @@
         <v/>
       </c>
       <c r="AN99" s="10" t="n"/>
+      <c r="AO99" s="10" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="60" customHeight="1">
       <c r="A100" s="5" t="n">
@@ -10051,6 +10718,11 @@
         <v/>
       </c>
       <c r="AN100" s="10" t="n"/>
+      <c r="AO100" s="10" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="60" customHeight="1">
       <c r="A101" s="5" t="n">
@@ -10148,6 +10820,11 @@
         <v/>
       </c>
       <c r="AN101" s="10" t="n"/>
+      <c r="AO101" s="10" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="60" customHeight="1">
       <c r="A102" s="5" t="n">
@@ -10245,6 +10922,11 @@
         <v/>
       </c>
       <c r="AN102" s="10" t="n"/>
+      <c r="AO102" s="10" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="60" customHeight="1">
       <c r="A103" s="5" t="n">
@@ -10342,6 +11024,11 @@
         <v/>
       </c>
       <c r="AN103" s="10" t="n"/>
+      <c r="AO103" s="10" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="60" customHeight="1">
       <c r="A104" s="5" t="n">
@@ -10439,6 +11126,11 @@
         <v/>
       </c>
       <c r="AN104" s="10" t="n"/>
+      <c r="AO104" s="10" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="60" customHeight="1">
       <c r="A105" s="5" t="n">
@@ -10536,6 +11228,11 @@
         <v/>
       </c>
       <c r="AN105" s="10" t="n"/>
+      <c r="AO105" s="10" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="AM6:AM105">
@@ -10546,12 +11243,15 @@
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="H6:H105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Idea,Researching,Scripted,Scheduled,Published,Vetoed,Failed,Filming,Editing"</formula1>
     </dataValidation>
     <dataValidation sqref="J6:J105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Strong,Weak"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AO6:AO105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Looks!$A$5:$A$19</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10568,7 +11268,501 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Visual styles</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Each Short is built in one look. Looks adapt palettes, type and conventions of the lemo-opuscar film styles (LemoLab, MIT licence, github.com/lemomo-ai/lemo-opuscar) to the vertical psychology template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Look id</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Adapted from</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Best for</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Ideas assigned</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Ground</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Accent</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>pixel-lab</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Pixel Lab (house look)</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>— (Motion as Code house style)</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Default; social/being-watched ideas</t>
+        </is>
+      </c>
+      <c r="E5" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="20" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Whiteboard Explainer</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Learning, study techniques, step-by-step how-tos</t>
+        </is>
+      </c>
+      <c r="E6" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="22" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Data Storytelling</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>dataviz</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Ideas whose punch is a number or chart; stats and sampling</t>
+        </is>
+      </c>
+      <c r="E7" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="23" t="n"/>
+      <c r="G7" s="24" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Swiss Motion Graphics</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>swiss-motion</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Decisions, wording, prices, crisp single-rule ideas</t>
+        </is>
+      </c>
+      <c r="E8" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="26" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Halftone Dossier</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>halftone-dossier</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Classic experiments as 'case files', myths on trial</t>
+        </is>
+      </c>
+      <c r="E9" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="28" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Risograph Print</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>risograph</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Light, warm, everyday social ideas</t>
+        </is>
+      </c>
+      <c r="E10" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="29" t="n"/>
+      <c r="G10" s="30" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Blueprint</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Systems and mechanisms: habits, friction, how the brain is 'built'</t>
+        </is>
+      </c>
+      <c r="E11" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="31" t="n"/>
+      <c r="G11" s="32" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>ASCII / CRT Terminal</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>ascii-crt</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Screens, feeds, notifications, attention online</t>
+        </is>
+      </c>
+      <c r="E12" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="33" t="n"/>
+      <c r="G12" s="34" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>keynote</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Dark Tech Keynote</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>dark-keynote</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Tech/consumer psychology, product and choice design</t>
+        </is>
+      </c>
+      <c r="E13" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="36" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Game Show Flat</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Quizzes, rewards, competitions, playful demos</t>
+        </is>
+      </c>
+      <c r="E14" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="37" t="n"/>
+      <c r="G14" s="38" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Mid-century Cartoon</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>midcentury-toon</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Practical 'how to' tips, everyday routines</t>
+        </is>
+      </c>
+      <c r="E15" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="39" t="n"/>
+      <c r="G15" s="40" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>60s Spy Titles</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>spy-titles</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Hidden thoughts, secrets, things people miss or conceal</t>
+        </is>
+      </c>
+      <c r="E16" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="41" t="n"/>
+      <c r="G16" s="42" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Crayon Picture Book</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>crayon-book</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Gentle emotional topics, self-kindness</t>
+        </is>
+      </c>
+      <c r="E17" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="43" t="n"/>
+      <c r="G17" s="44" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>pixel-quest</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>16-bit Pixel RPG</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>pixel-rpg</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Progress, levelling up, motivation, practice</t>
+        </is>
+      </c>
+      <c r="E18" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="45" t="n"/>
+      <c r="G18" s="46" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>One-line Drawing</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Introspective identity, memory and self-image ideas</t>
+        </is>
+      </c>
+      <c r="E19" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="47" t="n"/>
+      <c r="G19" s="48" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -10593,6 +11787,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -10895,6 +12090,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -10981,6 +12177,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -11202,6 +12399,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
@@ -11285,6 +12483,443 @@
       </c>
       <c r="F31" s="17">
         <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$J$6:$J$105,$A31,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Visual style</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Avg views d7</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Avg retention d7</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Avg engagement d7</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Avg views d30</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>pixel-lab</t>
+        </is>
+      </c>
+      <c r="B34" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C34" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D34" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E34" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>whiteboard</t>
+        </is>
+      </c>
+      <c r="B35" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C35" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D35" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E35" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>data-story</t>
+        </is>
+      </c>
+      <c r="B36" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C36" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D36" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E36" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>swiss</t>
+        </is>
+      </c>
+      <c r="B37" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C37" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D37" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E37" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>dossier</t>
+        </is>
+      </c>
+      <c r="B38" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C38" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D38" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E38" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>riso</t>
+        </is>
+      </c>
+      <c r="B39" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C39" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D39" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E39" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F39" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>blueprint</t>
+        </is>
+      </c>
+      <c r="B40" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C40" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D40" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E40" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F40" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
+      <c r="B41" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C41" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D41" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E41" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>keynote</t>
+        </is>
+      </c>
+      <c r="B42" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C42" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D42" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E42" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F42" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>game-show</t>
+        </is>
+      </c>
+      <c r="B43" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C43" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D43" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E43" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F43" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>cartoon-50s</t>
+        </is>
+      </c>
+      <c r="B44" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C44" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D44" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>spy-noir</t>
+        </is>
+      </c>
+      <c r="B45" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C45" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D45" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E45" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F45" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>crayon</t>
+        </is>
+      </c>
+      <c r="B46" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C46" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D46" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E46" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>pixel-quest</t>
+        </is>
+      </c>
+      <c r="B47" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C47" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D47" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E47" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>one-line</t>
+        </is>
+      </c>
+      <c r="B48" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <v/>
+      </c>
+      <c r="C48" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D48" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E48" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
CI pipeline: GitHub Actions build + Buffer scheduling (scripts written ahead by Claude)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -11294,6 +11294,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -11353,7 +11354,7 @@
         </is>
       </c>
       <c r="E5" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A5)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A5)</f>
         <v/>
       </c>
       <c r="F5" s="19" t="n"/>
@@ -11381,7 +11382,7 @@
         </is>
       </c>
       <c r="E6" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A6)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A6)</f>
         <v/>
       </c>
       <c r="F6" s="21" t="n"/>
@@ -11409,7 +11410,7 @@
         </is>
       </c>
       <c r="E7" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A7)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A7)</f>
         <v/>
       </c>
       <c r="F7" s="23" t="n"/>
@@ -11437,7 +11438,7 @@
         </is>
       </c>
       <c r="E8" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A8)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A8)</f>
         <v/>
       </c>
       <c r="F8" s="25" t="n"/>
@@ -11465,7 +11466,7 @@
         </is>
       </c>
       <c r="E9" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A9)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A9)</f>
         <v/>
       </c>
       <c r="F9" s="27" t="n"/>
@@ -11493,7 +11494,7 @@
         </is>
       </c>
       <c r="E10" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A10)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A10)</f>
         <v/>
       </c>
       <c r="F10" s="29" t="n"/>
@@ -11521,7 +11522,7 @@
         </is>
       </c>
       <c r="E11" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A11)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A11)</f>
         <v/>
       </c>
       <c r="F11" s="31" t="n"/>
@@ -11549,7 +11550,7 @@
         </is>
       </c>
       <c r="E12" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A12)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A12)</f>
         <v/>
       </c>
       <c r="F12" s="33" t="n"/>
@@ -11577,7 +11578,7 @@
         </is>
       </c>
       <c r="E13" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A13)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A13)</f>
         <v/>
       </c>
       <c r="F13" s="35" t="n"/>
@@ -11605,7 +11606,7 @@
         </is>
       </c>
       <c r="E14" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A14)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A14)</f>
         <v/>
       </c>
       <c r="F14" s="37" t="n"/>
@@ -11633,7 +11634,7 @@
         </is>
       </c>
       <c r="E15" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A15)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A15)</f>
         <v/>
       </c>
       <c r="F15" s="39" t="n"/>
@@ -11661,7 +11662,7 @@
         </is>
       </c>
       <c r="E16" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A16)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A16)</f>
         <v/>
       </c>
       <c r="F16" s="41" t="n"/>
@@ -11689,7 +11690,7 @@
         </is>
       </c>
       <c r="E17" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A17)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A17)</f>
         <v/>
       </c>
       <c r="F17" s="43" t="n"/>
@@ -11717,7 +11718,7 @@
         </is>
       </c>
       <c r="E18" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A18)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A18)</f>
         <v/>
       </c>
       <c r="F18" s="45" t="n"/>
@@ -11745,7 +11746,7 @@
         </is>
       </c>
       <c r="E19" s="16">
-        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$105,A19)</f>
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A19)</f>
         <v/>
       </c>
       <c r="F19" s="47" t="n"/>
@@ -11827,23 +11828,23 @@
         </is>
       </c>
       <c r="B5" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A5,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A5,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C5" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A5,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A5,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D5" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A5,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A5,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E5" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A5,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A5,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F5" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A5,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A5,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -11854,23 +11855,23 @@
         </is>
       </c>
       <c r="B6" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A6,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A6,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C6" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A6,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A6,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D6" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A6,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A6,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E6" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A6,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A6,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F6" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A6,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A6,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -11881,23 +11882,23 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A7,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A7,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C7" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A7,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A7,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D7" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A7,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A7,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E7" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A7,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A7,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F7" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A7,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A7,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -11908,23 +11909,23 @@
         </is>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A8,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A8,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C8" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A8,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A8,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A8,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A8,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E8" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A8,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A8,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F8" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A8,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A8,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -11935,23 +11936,23 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A9,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A9,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C9" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A9,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A9,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A9,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A9,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E9" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A9,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A9,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F9" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A9,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A9,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -11962,23 +11963,23 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A10,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A10,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C10" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A10,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A10,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D10" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A10,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A10,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E10" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A10,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A10,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F10" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A10,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A10,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -11989,23 +11990,23 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A11,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A11,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C11" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A11,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A11,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D11" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A11,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A11,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E11" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A11,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A11,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F11" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A11,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A11,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12016,23 +12017,23 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A12,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A12,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C12" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A12,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A12,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D12" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A12,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A12,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E12" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A12,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A12,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F12" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A12,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A12,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12043,23 +12044,23 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A13,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A13,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C13" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A13,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A13,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D13" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A13,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A13,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E13" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A13,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A13,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F13" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A13,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A13,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12070,23 +12071,23 @@
         </is>
       </c>
       <c r="B14" s="16">
-        <f>COUNTIFS('Shorts ideas'!$B$6:$B$105,$A14,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$B$6:$B$400,$A14,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C14" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$B$6:$B$105,$A14,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$B$6:$B$400,$A14,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D14" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$B$6:$B$105,$A14,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$B$6:$B$400,$A14,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E14" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$B$6:$B$105,$A14,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$B$6:$B$400,$A14,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F14" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$B$6:$B$105,$A14,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$B$6:$B$400,$A14,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12130,23 +12131,23 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>COUNTIFS('Shorts ideas'!$N$6:$N$105,$A17,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$N$6:$N$400,$A17,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C17" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$N$6:$N$105,$A17,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$N$6:$N$400,$A17,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D17" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$N$6:$N$105,$A17,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$N$6:$N$400,$A17,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E17" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$N$6:$N$105,$A17,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$N$6:$N$400,$A17,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F17" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$N$6:$N$105,$A17,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$N$6:$N$400,$A17,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12157,23 +12158,23 @@
         </is>
       </c>
       <c r="B18" s="16">
-        <f>COUNTIFS('Shorts ideas'!$N$6:$N$105,$A18,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$N$6:$N$400,$A18,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C18" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$N$6:$N$105,$A18,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$N$6:$N$400,$A18,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D18" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$N$6:$N$105,$A18,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$N$6:$N$400,$A18,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E18" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$N$6:$N$105,$A18,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$N$6:$N$400,$A18,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F18" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$N$6:$N$105,$A18,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$N$6:$N$400,$A18,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12217,23 +12218,23 @@
         </is>
       </c>
       <c r="B21" s="16">
-        <f>COUNTIFS('Shorts ideas'!$M$6:$M$105,$A21,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$M$6:$M$400,$A21,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C21" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$M$6:$M$105,$A21,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$M$6:$M$400,$A21,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D21" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$M$6:$M$105,$A21,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$M$6:$M$400,$A21,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E21" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$M$6:$M$105,$A21,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$M$6:$M$400,$A21,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F21" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$M$6:$M$105,$A21,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$M$6:$M$400,$A21,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12244,23 +12245,23 @@
         </is>
       </c>
       <c r="B22" s="16">
-        <f>COUNTIFS('Shorts ideas'!$M$6:$M$105,$A22,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$M$6:$M$400,$A22,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C22" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$M$6:$M$105,$A22,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$M$6:$M$400,$A22,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D22" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$M$6:$M$105,$A22,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$M$6:$M$400,$A22,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E22" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$M$6:$M$105,$A22,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$M$6:$M$400,$A22,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F22" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$M$6:$M$105,$A22,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$M$6:$M$400,$A22,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12271,23 +12272,23 @@
         </is>
       </c>
       <c r="B23" s="16">
-        <f>COUNTIFS('Shorts ideas'!$M$6:$M$105,$A23,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$M$6:$M$400,$A23,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C23" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$M$6:$M$105,$A23,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$M$6:$M$400,$A23,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D23" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$M$6:$M$105,$A23,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$M$6:$M$400,$A23,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E23" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$M$6:$M$105,$A23,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$M$6:$M$400,$A23,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F23" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$M$6:$M$105,$A23,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$M$6:$M$400,$A23,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12298,23 +12299,23 @@
         </is>
       </c>
       <c r="B24" s="16">
-        <f>COUNTIFS('Shorts ideas'!$M$6:$M$105,$A24,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$M$6:$M$400,$A24,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C24" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$M$6:$M$105,$A24,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$M$6:$M$400,$A24,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D24" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$M$6:$M$105,$A24,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$M$6:$M$400,$A24,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E24" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$M$6:$M$105,$A24,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$M$6:$M$400,$A24,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F24" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$M$6:$M$105,$A24,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$M$6:$M$400,$A24,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12325,23 +12326,23 @@
         </is>
       </c>
       <c r="B25" s="16">
-        <f>COUNTIFS('Shorts ideas'!$M$6:$M$105,$A25,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$M$6:$M$400,$A25,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C25" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$M$6:$M$105,$A25,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$M$6:$M$400,$A25,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D25" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$M$6:$M$105,$A25,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$M$6:$M$400,$A25,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E25" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$M$6:$M$105,$A25,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$M$6:$M$400,$A25,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F25" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$M$6:$M$105,$A25,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$M$6:$M$400,$A25,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12352,23 +12353,23 @@
         </is>
       </c>
       <c r="B26" s="16">
-        <f>COUNTIFS('Shorts ideas'!$M$6:$M$105,$A26,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$M$6:$M$400,$A26,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C26" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$M$6:$M$105,$A26,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$M$6:$M$400,$A26,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D26" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$M$6:$M$105,$A26,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$M$6:$M$400,$A26,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E26" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$M$6:$M$105,$A26,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$M$6:$M$400,$A26,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F26" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$M$6:$M$105,$A26,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$M$6:$M$400,$A26,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12379,23 +12380,23 @@
         </is>
       </c>
       <c r="B27" s="16">
-        <f>COUNTIFS('Shorts ideas'!$M$6:$M$105,$A27,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$M$6:$M$400,$A27,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C27" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$M$6:$M$105,$A27,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$M$6:$M$400,$A27,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D27" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$M$6:$M$105,$A27,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$M$6:$M$400,$A27,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E27" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$M$6:$M$105,$A27,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$M$6:$M$400,$A27,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F27" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$M$6:$M$105,$A27,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$M$6:$M$400,$A27,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12439,23 +12440,23 @@
         </is>
       </c>
       <c r="B30" s="16">
-        <f>COUNTIFS('Shorts ideas'!$J$6:$J$105,$A30,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$J$6:$J$400,$A30,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C30" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$J$6:$J$105,$A30,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$J$6:$J$400,$A30,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D30" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$J$6:$J$105,$A30,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$J$6:$J$400,$A30,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E30" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$J$6:$J$105,$A30,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$J$6:$J$400,$A30,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F30" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$J$6:$J$105,$A30,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$J$6:$J$400,$A30,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12466,26 +12467,27 @@
         </is>
       </c>
       <c r="B31" s="16">
-        <f>COUNTIFS('Shorts ideas'!$J$6:$J$105,$A31,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$J$6:$J$400,$A31,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C31" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$J$6:$J$105,$A31,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$J$6:$J$400,$A31,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D31" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$J$6:$J$105,$A31,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$J$6:$J$400,$A31,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E31" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$J$6:$J$105,$A31,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$J$6:$J$400,$A31,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F31" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$J$6:$J$105,$A31,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
-        <v/>
-      </c>
-    </row>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$J$6:$J$400,$A31,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
@@ -12525,23 +12527,23 @@
         </is>
       </c>
       <c r="B34" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A34,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C34" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A34,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D34" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A34,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E34" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A34,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F34" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A34,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A34,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12552,23 +12554,23 @@
         </is>
       </c>
       <c r="B35" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A35,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C35" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A35,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D35" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A35,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E35" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A35,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F35" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A35,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A35,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12579,23 +12581,23 @@
         </is>
       </c>
       <c r="B36" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A36,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C36" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A36,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D36" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A36,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E36" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A36,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F36" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A36,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A36,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12606,23 +12608,23 @@
         </is>
       </c>
       <c r="B37" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A37,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C37" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A37,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D37" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A37,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E37" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A37,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F37" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A37,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A37,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12633,23 +12635,23 @@
         </is>
       </c>
       <c r="B38" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A38,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C38" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A38,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D38" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A38,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E38" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A38,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F38" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A38,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A38,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12660,23 +12662,23 @@
         </is>
       </c>
       <c r="B39" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A39,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C39" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A39,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D39" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A39,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E39" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A39,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F39" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A39,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A39,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12687,23 +12689,23 @@
         </is>
       </c>
       <c r="B40" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A40,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C40" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A40,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D40" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A40,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E40" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A40,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F40" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A40,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A40,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12714,23 +12716,23 @@
         </is>
       </c>
       <c r="B41" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A41,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C41" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A41,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D41" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A41,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E41" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A41,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F41" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A41,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A41,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12741,23 +12743,23 @@
         </is>
       </c>
       <c r="B42" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A42,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C42" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A42,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D42" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A42,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E42" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A42,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F42" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A42,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A42,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12768,23 +12770,23 @@
         </is>
       </c>
       <c r="B43" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A43,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C43" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A43,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D43" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A43,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E43" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A43,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F43" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A43,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A43,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12795,23 +12797,23 @@
         </is>
       </c>
       <c r="B44" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A44,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C44" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A44,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D44" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A44,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E44" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A44,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F44" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A44,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A44,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12822,23 +12824,23 @@
         </is>
       </c>
       <c r="B45" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A45,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C45" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A45,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D45" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A45,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E45" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A45,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F45" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A45,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A45,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12849,23 +12851,23 @@
         </is>
       </c>
       <c r="B46" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A46,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C46" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A46,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D46" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A46,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E46" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A46,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F46" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A46,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A46,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12876,23 +12878,23 @@
         </is>
       </c>
       <c r="B47" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A47,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C47" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A47,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D47" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A47,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E47" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A47,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F47" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A47,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A47,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>
@@ -12903,23 +12905,23 @@
         </is>
       </c>
       <c r="B48" s="16">
-        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$H$6:$H$105,"Published")</f>
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A48,'Shorts ideas'!$H$6:$H$400,"Published")</f>
         <v/>
       </c>
       <c r="C48" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$AC$6:$AC$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A48,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="D48" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$U$6:$U$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A48,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="E48" s="18">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$AD$6:$AD$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A48,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
         <v/>
       </c>
       <c r="F48" s="17">
-        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$105,'Shorts ideas'!$AO$6:$AO$105,$A48,'Shorts ideas'!$AL$6:$AL$105,"&gt;0"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A48,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Ted type 1 for the next 10 videos: CI illustration picker, 2 scripts converted, runbook rules
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Looks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4662,7 +4662,7 @@
       <c r="P40" s="10" t="n"/>
       <c r="Q40" s="10" t="inlineStr">
         <is>
-          <t>Read &amp; van Leeuwen 1998, OBHDP 76(2):189-205; n=200 Amsterdam employees; all groups chose more unhealthy snacks immediately than in advance (paper PDF)</t>
+          <t>Read &amp; van Leeuwen (1998), Organizational Behavior and Human Decision Processes 76(2)</t>
         </is>
       </c>
       <c r="R40" s="10" t="n"/>
@@ -4708,7 +4708,7 @@
       <c r="AN40" s="10" t="n"/>
       <c r="AO40" s="10" t="inlineStr">
         <is>
-          <t>pixel-quest</t>
+          <t>ted1</t>
         </is>
       </c>
     </row>
@@ -5514,7 +5514,7 @@
       <c r="P48" s="10" t="n"/>
       <c r="Q48" s="10" t="inlineStr">
         <is>
-          <t>Jamieson et al. 2010, JESP 46(1):208-212; actual GRE math M=770 vs 705.7 (n=28) (Harvard DASH)</t>
+          <t>Brooks (2014), Journal of Experimental Psychology: General 143(3)</t>
         </is>
       </c>
       <c r="R48" s="10" t="n"/>
@@ -5560,7 +5560,7 @@
       <c r="AN48" s="10" t="n"/>
       <c r="AO48" s="10" t="inlineStr">
         <is>
-          <t>riso</t>
+          <t>ted1</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11515,7 @@
       <formula1>"Strong,Weak"</formula1>
     </dataValidation>
     <dataValidation sqref="AO6:AO105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Looks!$A$5:$A$19</formula1>
+      <formula1>=Looks!$A$5:$A$20</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11532,7 +11532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12015,6 +12015,34 @@
       <c r="F19" s="47" t="n"/>
       <c r="G19" s="48" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>ted1</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Ted type 1 (card montage)</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>@mindunderglass-style tips channel</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Faceless tip lists: Lottie illustration per line, deep male narrator</t>
+        </is>
+      </c>
+      <c r="E20" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="47" t="n"/>
+      <c r="G20" s="48" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12026,7 +12054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -12051,6 +12079,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12353,6 +12382,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -12439,6 +12469,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -12660,6 +12691,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
@@ -12746,6 +12778,7 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
@@ -13180,6 +13213,33 @@
       </c>
       <c r="F48" s="17">
         <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A48,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>ted1</t>
+        </is>
+      </c>
+      <c r="B49" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A49,'Shorts ideas'!$H$6:$H$400,"Published")</f>
+        <v/>
+      </c>
+      <c r="C49" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A49,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D49" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A49,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A49,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A49,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Long-form Ted type 1: landscape layout, chunked CI build, thumbnail, chapters, Buffer YouTube; first script
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -4,8 +4,9 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -65,6 +66,11 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="33">
@@ -242,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -312,6 +318,8 @@
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -11532,6 +11540,359 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="49" t="inlineStr">
+        <is>
+          <t>Long-form videos (Ted type 1, 16:9, YouTube) — twice a week</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Built by the "Long-form" GitHub workflow (Mon &amp; Thu) for posting Tue &amp; Fri. Status: Idea → Scripted → Scheduled → Published | Vetoed | Failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Angle / hook</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Post date</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Title used</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Length (min)</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>YT views d7</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>YT avg view (s) d7</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>YT retention d7</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>YT likes d7</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>YT views d30</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>Lesson / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Liking &amp; influence</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>7 psychology tricks that make people like you (and why they work)</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>seven-tricks-liked</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>7 Psychology Tricks That Make People Like You (Backed by Research)</t>
+        </is>
+      </c>
+      <c r="L5" s="50">
+        <f>IF(OR(K5="",N(I5)=0),"",K5/(I5*60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Cognitive biases</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>8 ways your brain lies to you every day</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="50">
+        <f>IF(OR(K6="",N(I6)=0),"",K6/(I6*60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>How to study smarter: 6 techniques backed by research</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" s="50">
+        <f>IF(OR(K7="",N(I7)=0),"",K7/(I7*60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Habits</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>The psychology of habits: why you can't stop (and how to)</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" s="50">
+        <f>IF(OR(K8="",N(I8)=0),"",K8/(I8*60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Social pressure</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Why good people go along with bad things: conformity, obedience and the bystander effect</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="50">
+        <f>IF(OR(K9="",N(I9)=0),"",K9/(I9*60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Persuasion defense</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Manipulation tactics people use on you, and how to spot them</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="50">
+        <f>IF(OR(K10="",N(I10)=0),"",K10/(I10*60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Memory hacks that actually work, according to science</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" s="50">
+        <f>IF(OR(K11="",N(I11)=0),"",K11/(I11*60))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Procrastination</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Why you procrastinate (it's not laziness) and what fixes it</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" s="50">
+        <f>IF(OR(K12="",N(I12)=0),"",K12/(I12*60))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D5:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Idea,Scripted,Scheduled,Published,Vetoed,Failed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -12048,7 +12409,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12079,7 +12440,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12382,7 +12742,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -12469,7 +12828,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -12691,7 +13049,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
@@ -12778,7 +13135,6 @@
         <v/>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Name the Claude Design style 'Ted type 2' (ted2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Long form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Looks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11531,7 +11531,7 @@
       <formula1>"Strong,Weak"</formula1>
     </dataValidation>
     <dataValidation sqref="AO6:AO105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Looks!$A$5:$A$20</formula1>
+      <formula1>=Looks!$A$5:$A$21</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11901,7 +11901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12412,6 +12412,34 @@
       <c r="F20" s="47" t="n"/>
       <c r="G20" s="48" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Ted type 2 (Claude Design style)</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Shivam's Claude Design 'Rename Your Nerves Short'</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Faceless tips: drawn SVG scene per line, kinetic emphasis captions, deep narrator</t>
+        </is>
+      </c>
+      <c r="E21" s="16">
+        <f>COUNTIF('Shorts ideas'!$AO$6:$AO$400,A21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="47" t="n"/>
+      <c r="G21" s="48" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12423,7 +12451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -12448,6 +12476,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12750,6 +12779,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -12836,6 +12866,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -13057,6 +13088,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
@@ -13143,6 +13175,7 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
@@ -13604,6 +13637,33 @@
       </c>
       <c r="F49" s="17">
         <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A49,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="B50" s="16">
+        <f>COUNTIFS('Shorts ideas'!$AO$6:$AO$400,$A50,'Shorts ideas'!$H$6:$H$400,"Published")</f>
+        <v/>
+      </c>
+      <c r="C50" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AC$6:$AC$400,'Shorts ideas'!$AO$6:$AO$400,$A50,'Shorts ideas'!$AC$6:$AC$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="D50" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$U$6:$U$400,'Shorts ideas'!$AO$6:$AO$400,$A50,'Shorts ideas'!$U$6:$U$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="E50" s="18">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AD$6:$AD$400,'Shorts ideas'!$AO$6:$AO$400,$A50,'Shorts ideas'!$AD$6:$AD$400,"&gt;0"),"")</f>
+        <v/>
+      </c>
+      <c r="F50" s="17">
+        <f>IFERROR(AVERAGEIFS('Shorts ideas'!$AL$6:$AL$400,'Shorts ideas'!$AO$6:$AO$400,$A50,'Shorts ideas'!$AL$6:$AL$400,"&gt;0"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Open Loops: Shivam's Claude Design Short, voiced (Ash/Nova) with a calm bed; prebuilt format
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AO105"/>
+  <dimension ref="A2:AO106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11514,6 +11514,112 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Memory and learning</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Open loops (Zeigarnik effect)</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>Nova, my brain won't let me sleep.</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>Unfinished tasks stay active in memory (Zeigarnik 1927); writing the next step quiets them (Masicampo &amp; Baumeister 2011).</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Nova dialogue: Ash and robot Nova in a low-poly night room</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I106" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="J106" s="10" t="n"/>
+      <c r="K106" s="10" t="inlineStr">
+        <is>
+          <t>open-loops</t>
+        </is>
+      </c>
+      <c r="L106" s="11" t="n"/>
+      <c r="M106" s="5">
+        <f>IF(L106="","",TEXT(L106,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N106" s="10" t="n"/>
+      <c r="O106" s="10" t="n"/>
+      <c r="P106" s="10" t="n"/>
+      <c r="Q106" s="10" t="inlineStr">
+        <is>
+          <t>Zeigarnik 1927, Psychologische Forschung 9:1-85; Masicampo &amp; Baumeister 2011, JPSP 101(4):667-683</t>
+        </is>
+      </c>
+      <c r="R106" s="10" t="n"/>
+      <c r="S106" s="12" t="n"/>
+      <c r="T106" s="10" t="n"/>
+      <c r="U106" s="13">
+        <f>IF(OR(T106="",N(O106)=0),"",T106/O106)</f>
+        <v/>
+      </c>
+      <c r="V106" s="10" t="n"/>
+      <c r="W106" s="10" t="n"/>
+      <c r="X106" s="10" t="n"/>
+      <c r="Y106" s="12" t="n"/>
+      <c r="Z106" s="10" t="n"/>
+      <c r="AA106" s="12" t="n"/>
+      <c r="AB106" s="10" t="n"/>
+      <c r="AC106" s="14">
+        <f>IF(COUNT(S106,Y106,AA106)=0,"",SUM(S106,Y106,AA106))</f>
+        <v/>
+      </c>
+      <c r="AD106" s="13">
+        <f>IF(N(AC106)=0,"",SUM(V106,W106,X106,Z106,AB106)/AC106)</f>
+        <v/>
+      </c>
+      <c r="AE106" s="12" t="n"/>
+      <c r="AF106" s="12" t="n"/>
+      <c r="AG106" s="12" t="n"/>
+      <c r="AH106" s="14">
+        <f>IF(COUNT(AE106,AF106,AG106)=0,"",SUM(AE106,AF106,AG106))</f>
+        <v/>
+      </c>
+      <c r="AI106" s="12" t="n"/>
+      <c r="AJ106" s="12" t="n"/>
+      <c r="AK106" s="12" t="n"/>
+      <c r="AL106" s="14">
+        <f>IF(COUNT(AI106,AJ106,AK106)=0,"",SUM(AI106,AJ106,AK106))</f>
+        <v/>
+      </c>
+      <c r="AM106" s="5">
+        <f>IF(N(AC106)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC106&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC106&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN106" s="10" t="n"/>
+      <c r="AO106" s="10" t="inlineStr">
+        <is>
+          <t>nova</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="AM6:AM105">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -11524,13 +11630,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Idea,Researching,Scripted,Scheduled,Published,Vetoed,Failed,Filming,Editing"</formula1>
     </dataValidation>
-    <dataValidation sqref="J6:J105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J6:J106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Strong,Weak"</formula1>
     </dataValidation>
-    <dataValidation sqref="AO6:AO105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AO6:AO106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Looks!$A$5:$A$21</formula1>
     </dataValidation>
   </dataValidations>
@@ -12476,7 +12582,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12779,7 +12884,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -12866,7 +12970,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -13088,7 +13191,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
@@ -13175,7 +13277,6 @@
         <v/>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scripts: 12 new (+ present-bias converted to Ted type 2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GJ5FsYUZJGoj11ggYnd2tt
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Long form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Looks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I8" s="10" t="n">
@@ -1267,16 +1267,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K8" s="10" t="n"/>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>anchoring</t>
+        </is>
+      </c>
       <c r="L8" s="11" t="n"/>
       <c r="M8" s="5">
         <f>IF(L8="","",TEXT(L8,"ddd"))</f>
         <v/>
       </c>
-      <c r="N8" s="10" t="n"/>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O8" s="10" t="n"/>
       <c r="P8" s="10" t="n"/>
-      <c r="Q8" s="10" t="n"/>
+      <c r="Q8" s="10" t="inlineStr">
+        <is>
+          <t>Tversky &amp; Kahneman 1974, Science 185(4157):1124-1131; wheel 10 vs 65 -&gt; median 25% vs 45% African UN members</t>
+        </is>
+      </c>
       <c r="R8" s="10" t="n"/>
       <c r="S8" s="12" t="n"/>
       <c r="T8" s="10" t="n"/>
@@ -1320,7 +1332,7 @@
       <c r="AN8" s="10" t="n"/>
       <c r="AO8" s="10" t="inlineStr">
         <is>
-          <t>swiss</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2336,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I18" s="10" t="n">
@@ -2335,16 +2347,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K18" s="10" t="n"/>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>spacing-effect</t>
+        </is>
+      </c>
       <c r="L18" s="11" t="n"/>
       <c r="M18" s="5">
         <f>IF(L18="","",TEXT(L18,"ddd"))</f>
         <v/>
       </c>
-      <c r="N18" s="10" t="n"/>
+      <c r="N18" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O18" s="10" t="n"/>
       <c r="P18" s="10" t="n"/>
-      <c r="Q18" s="10" t="n"/>
+      <c r="Q18" s="10" t="inlineStr">
+        <is>
+          <t>Cepeda et al. 2006, Psychological Bulletin 132(3):354-380; 317 experiments/184 articles, spaced &gt; massed recall</t>
+        </is>
+      </c>
       <c r="R18" s="10" t="n"/>
       <c r="S18" s="12" t="n"/>
       <c r="T18" s="10" t="n"/>
@@ -2388,7 +2412,7 @@
       <c r="AN18" s="10" t="n"/>
       <c r="AO18" s="10" t="inlineStr">
         <is>
-          <t>pixel-quest</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3620,7 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I30" s="10" t="n">
@@ -3607,16 +3631,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K30" s="10" t="n"/>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t>cocktail-party</t>
+        </is>
+      </c>
       <c r="L30" s="11" t="n"/>
       <c r="M30" s="5">
         <f>IF(L30="","",TEXT(L30,"ddd"))</f>
         <v/>
       </c>
-      <c r="N30" s="10" t="n"/>
+      <c r="N30" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O30" s="10" t="n"/>
       <c r="P30" s="10" t="n"/>
-      <c r="Q30" s="10" t="n"/>
+      <c r="Q30" s="10" t="inlineStr">
+        <is>
+          <t>Moray 1959, QJEP 11(1):56-60; words repeated 35x in rejected ear not recalled, ~1/3 noticed own name (cf. Wood &amp; Cowan 1995)</t>
+        </is>
+      </c>
       <c r="R30" s="10" t="n"/>
       <c r="S30" s="12" t="n"/>
       <c r="T30" s="10" t="n"/>
@@ -3660,7 +3696,7 @@
       <c r="AN30" s="10" t="n"/>
       <c r="AO30" s="10" t="inlineStr">
         <is>
-          <t>riso</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4752,7 @@
       <c r="AN40" s="10" t="n"/>
       <c r="AO40" s="10" t="inlineStr">
         <is>
-          <t>ted1</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4790,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I41" s="10" t="n">
@@ -4765,16 +4801,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K41" s="10" t="n"/>
+      <c r="K41" s="10" t="inlineStr">
+        <is>
+          <t>procrastination-feelings</t>
+        </is>
+      </c>
       <c r="L41" s="11" t="n"/>
       <c r="M41" s="5">
         <f>IF(L41="","",TEXT(L41,"ddd"))</f>
         <v/>
       </c>
-      <c r="N41" s="10" t="n"/>
+      <c r="N41" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O41" s="10" t="n"/>
       <c r="P41" s="10" t="n"/>
-      <c r="Q41" s="10" t="n"/>
+      <c r="Q41" s="10" t="inlineStr">
+        <is>
+          <t>Tice &amp; Baumeister 1997, Psychological Science 8(6):454-458; less stress early, more stress/illness late, lower grades; Sirois &amp; Pychyl 2013 mood repair</t>
+        </is>
+      </c>
       <c r="R41" s="10" t="n"/>
       <c r="S41" s="12" t="n"/>
       <c r="T41" s="10" t="n"/>
@@ -4818,7 +4866,7 @@
       <c r="AN41" s="10" t="n"/>
       <c r="AO41" s="10" t="inlineStr">
         <is>
-          <t>crayon</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5968,7 @@
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I52" s="10" t="n">
@@ -5931,16 +5979,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K52" s="10" t="n"/>
+      <c r="K52" s="10" t="inlineStr">
+        <is>
+          <t>suppression</t>
+        </is>
+      </c>
       <c r="L52" s="11" t="n"/>
       <c r="M52" s="5">
         <f>IF(L52="","",TEXT(L52,"ddd"))</f>
         <v/>
       </c>
-      <c r="N52" s="10" t="n"/>
+      <c r="N52" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O52" s="10" t="n"/>
       <c r="P52" s="10" t="n"/>
-      <c r="Q52" s="10" t="n"/>
+      <c r="Q52" s="10" t="inlineStr">
+        <is>
+          <t>Butler et al. 2003, Emotion 3(1):48-67; suppression raised partners' blood pressure, lowered rapport/affiliation</t>
+        </is>
+      </c>
       <c r="R52" s="10" t="n"/>
       <c r="S52" s="12" t="n"/>
       <c r="T52" s="10" t="n"/>
@@ -5984,7 +6044,7 @@
       <c r="AN52" s="10" t="n"/>
       <c r="AO52" s="10" t="inlineStr">
         <is>
-          <t>spy-noir</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -7168,7 +7228,7 @@
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I64" s="10" t="n">
@@ -7179,16 +7239,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K64" s="10" t="n"/>
+      <c r="K64" s="10" t="inlineStr">
+        <is>
+          <t>mere-exposure</t>
+        </is>
+      </c>
       <c r="L64" s="11" t="n"/>
       <c r="M64" s="5">
         <f>IF(L64="","",TEXT(L64,"ddd"))</f>
         <v/>
       </c>
-      <c r="N64" s="10" t="n"/>
+      <c r="N64" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O64" s="10" t="n"/>
       <c r="P64" s="10" t="n"/>
-      <c r="Q64" s="10" t="n"/>
+      <c r="Q64" s="10" t="inlineStr">
+        <is>
+          <t>Moreland &amp; Beach 1992, J Exp Social Psych 28(3):255-276; women attended 0/5/10/15 lectures, rated more attractive/likeable with more exposure</t>
+        </is>
+      </c>
       <c r="R64" s="10" t="n"/>
       <c r="S64" s="12" t="n"/>
       <c r="T64" s="10" t="n"/>
@@ -7232,7 +7304,7 @@
       <c r="AN64" s="10" t="n"/>
       <c r="AO64" s="10" t="inlineStr">
         <is>
-          <t>riso</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7570,7 @@
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I67" s="10" t="n">
@@ -7509,16 +7581,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K67" s="10" t="n"/>
+      <c r="K67" s="10" t="inlineStr">
+        <is>
+          <t>informational-influence</t>
+        </is>
+      </c>
       <c r="L67" s="11" t="n"/>
       <c r="M67" s="5">
         <f>IF(L67="","",TEXT(L67,"ddd"))</f>
         <v/>
       </c>
-      <c r="N67" s="10" t="n"/>
+      <c r="N67" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O67" s="10" t="n"/>
       <c r="P67" s="10" t="n"/>
-      <c r="Q67" s="10" t="n"/>
+      <c r="Q67" s="10" t="inlineStr">
+        <is>
+          <t>Sherif 1935, Archives of Psychology 27(187); autokinetic effect, group estimates converge and persist when tested alone</t>
+        </is>
+      </c>
       <c r="R67" s="10" t="n"/>
       <c r="S67" s="12" t="n"/>
       <c r="T67" s="10" t="n"/>
@@ -7562,7 +7646,7 @@
       <c r="AN67" s="10" t="n"/>
       <c r="AO67" s="10" t="inlineStr">
         <is>
-          <t>data-story</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -7600,7 +7684,7 @@
       </c>
       <c r="H68" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I68" s="10" t="n">
@@ -7611,16 +7695,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K68" s="10" t="n"/>
+      <c r="K68" s="10" t="inlineStr">
+        <is>
+          <t>normative-influence</t>
+        </is>
+      </c>
       <c r="L68" s="11" t="n"/>
       <c r="M68" s="5">
         <f>IF(L68="","",TEXT(L68,"ddd"))</f>
         <v/>
       </c>
-      <c r="N68" s="10" t="n"/>
+      <c r="N68" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O68" s="10" t="n"/>
       <c r="P68" s="10" t="n"/>
-      <c r="Q68" s="10" t="n"/>
+      <c r="Q68" s="10" t="inlineStr">
+        <is>
+          <t>Asch 1956, Psychological Monographs 70(9); written private answers cut conformity sharply (cf. Deutsch &amp; Gerard 1955)</t>
+        </is>
+      </c>
       <c r="R68" s="10" t="n"/>
       <c r="S68" s="12" t="n"/>
       <c r="T68" s="10" t="n"/>
@@ -7664,7 +7760,7 @@
       <c r="AN68" s="10" t="n"/>
       <c r="AO68" s="10" t="inlineStr">
         <is>
-          <t>game-show</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8638,7 @@
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I77" s="10" t="n">
@@ -8553,16 +8649,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K77" s="10" t="n"/>
+      <c r="K77" s="10" t="inlineStr">
+        <is>
+          <t>better-than-average</t>
+        </is>
+      </c>
       <c r="L77" s="11" t="n"/>
       <c r="M77" s="5">
         <f>IF(L77="","",TEXT(L77,"ddd"))</f>
         <v/>
       </c>
-      <c r="N77" s="10" t="n"/>
+      <c r="N77" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O77" s="10" t="n"/>
       <c r="P77" s="10" t="n"/>
-      <c r="Q77" s="10" t="n"/>
+      <c r="Q77" s="10" t="inlineStr">
+        <is>
+          <t>Svenson 1981, Acta Psychologica 47(2):143-148; 93% US / 69% Swedish students rated driving skill above median</t>
+        </is>
+      </c>
       <c r="R77" s="10" t="n"/>
       <c r="S77" s="12" t="n"/>
       <c r="T77" s="10" t="n"/>
@@ -8606,7 +8714,7 @@
       <c r="AN77" s="10" t="n"/>
       <c r="AO77" s="10" t="inlineStr">
         <is>
-          <t>game-show</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -8644,7 +8752,7 @@
       </c>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I78" s="10" t="n">
@@ -8655,16 +8763,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K78" s="10" t="n"/>
+      <c r="K78" s="10" t="inlineStr">
+        <is>
+          <t>impostor-feelings</t>
+        </is>
+      </c>
       <c r="L78" s="11" t="n"/>
       <c r="M78" s="5">
         <f>IF(L78="","",TEXT(L78,"ddd"))</f>
         <v/>
       </c>
-      <c r="N78" s="10" t="n"/>
+      <c r="N78" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O78" s="10" t="n"/>
       <c r="P78" s="10" t="n"/>
-      <c r="Q78" s="10" t="n"/>
+      <c r="Q78" s="10" t="inlineStr">
+        <is>
+          <t>Clance &amp; Imes 1978, Psychotherapy 15(3):241-247 (150+ high-achieving women); Bravata et al. 2020 JGIM review, 62 studies, 9-82%</t>
+        </is>
+      </c>
       <c r="R78" s="10" t="n"/>
       <c r="S78" s="12" t="n"/>
       <c r="T78" s="10" t="n"/>
@@ -8708,7 +8828,7 @@
       <c r="AN78" s="10" t="n"/>
       <c r="AO78" s="10" t="inlineStr">
         <is>
-          <t>spy-noir</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -9688,7 +9808,7 @@
       </c>
       <c r="H88" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I88" s="10" t="n">
@@ -9699,16 +9819,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K88" s="10" t="n"/>
+      <c r="K88" s="10" t="inlineStr">
+        <is>
+          <t>likes-feedback</t>
+        </is>
+      </c>
       <c r="L88" s="11" t="n"/>
       <c r="M88" s="5">
         <f>IF(L88="","",TEXT(L88,"ddd"))</f>
         <v/>
       </c>
-      <c r="N88" s="10" t="n"/>
+      <c r="N88" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O88" s="10" t="n"/>
       <c r="P88" s="10" t="n"/>
-      <c r="Q88" s="10" t="n"/>
+      <c r="Q88" s="10" t="inlineStr">
+        <is>
+          <t>Sherman et al. 2016, Psychological Science 27(7):1027-1035; n=32 teens 13-18, many-like photos liked more, NAcc activity for own photos with many likes</t>
+        </is>
+      </c>
       <c r="R88" s="10" t="n"/>
       <c r="S88" s="12" t="n"/>
       <c r="T88" s="10" t="n"/>
@@ -9752,7 +9884,7 @@
       <c r="AN88" s="10" t="n"/>
       <c r="AO88" s="10" t="inlineStr">
         <is>
-          <t>keynote</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -10630,7 +10762,7 @@
       </c>
       <c r="H97" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I97" s="10" t="n">
@@ -10641,16 +10773,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K97" s="10" t="n"/>
+      <c r="K97" s="10" t="inlineStr">
+        <is>
+          <t>left-right-brain-myth</t>
+        </is>
+      </c>
       <c r="L97" s="11" t="n"/>
       <c r="M97" s="5">
         <f>IF(L97="","",TEXT(L97,"ddd"))</f>
         <v/>
       </c>
-      <c r="N97" s="10" t="n"/>
+      <c r="N97" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O97" s="10" t="n"/>
       <c r="P97" s="10" t="n"/>
-      <c r="Q97" s="10" t="n"/>
+      <c r="Q97" s="10" t="inlineStr">
+        <is>
+          <t>Nielsen et al. 2013, PLOS ONE 8(8):e71275; 1,011 people aged 7-29, no whole-brain left/right dominance</t>
+        </is>
+      </c>
       <c r="R97" s="10" t="n"/>
       <c r="S97" s="12" t="n"/>
       <c r="T97" s="10" t="n"/>
@@ -10694,7 +10838,7 @@
       <c r="AN97" s="10" t="n"/>
       <c r="AO97" s="10" t="inlineStr">
         <is>
-          <t>blueprint</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scripts: 12 more Ted type 2; 8-bit avatar posts cancelled (Vetoed); runbook: Ted type 2 only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GJ5FsYUZJGoj11ggYnd2tt
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I7" s="10" t="n">
@@ -1215,7 +1215,11 @@
         <f>IF(N(AC7)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC7&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC7&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN7" s="10" t="n"/>
+      <c r="AN7" s="10" t="inlineStr">
+        <is>
+          <t>Cancelled in Buffer 2026-10-15 before posting: Shivam retired the 8-bit avatar format (Ted type 2 only)</t>
+        </is>
+      </c>
       <c r="AO7" s="10" t="inlineStr">
         <is>
           <t>keynote</t>
@@ -1370,7 +1374,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I9" s="10" t="n">
@@ -1381,16 +1385,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K9" s="10" t="n"/>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>availability-heuristic</t>
+        </is>
+      </c>
       <c r="L9" s="11" t="n"/>
       <c r="M9" s="5">
         <f>IF(L9="","",TEXT(L9,"ddd"))</f>
         <v/>
       </c>
-      <c r="N9" s="10" t="n"/>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O9" s="10" t="n"/>
       <c r="P9" s="10" t="n"/>
-      <c r="Q9" s="10" t="n"/>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Lichtenstein, Slovic et al. 1978, JEP:HLM 4(6):551-578; 41 causes of death, dramatic over-, common underestimated; Tversky &amp; Kahneman 1973</t>
+        </is>
+      </c>
       <c r="R9" s="10" t="n"/>
       <c r="S9" s="12" t="n"/>
       <c r="T9" s="10" t="n"/>
@@ -1434,7 +1450,7 @@
       <c r="AN9" s="10" t="n"/>
       <c r="AO9" s="10" t="inlineStr">
         <is>
-          <t>dossier</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1488,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I10" s="10" t="n">
@@ -1483,16 +1499,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K10" s="10" t="n"/>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>sunk-cost</t>
+        </is>
+      </c>
       <c r="L10" s="11" t="n"/>
       <c r="M10" s="5">
         <f>IF(L10="","",TEXT(L10,"ddd"))</f>
         <v/>
       </c>
-      <c r="N10" s="10" t="n"/>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O10" s="10" t="n"/>
       <c r="P10" s="10" t="n"/>
-      <c r="Q10" s="10" t="n"/>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>Arkes &amp; Blumer 1985, OBHDP 35(1):124-140; ski trip 00 Michigan vs 0 Wisconsin, 54% (33/61) chose Michigan</t>
+        </is>
+      </c>
       <c r="R10" s="10" t="n"/>
       <c r="S10" s="12" t="n"/>
       <c r="T10" s="10" t="n"/>
@@ -1536,7 +1564,7 @@
       <c r="AN10" s="10" t="n"/>
       <c r="AO10" s="10" t="inlineStr">
         <is>
-          <t>cartoon-50s</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2238,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I17" s="10" t="n">
@@ -2295,7 +2323,11 @@
         <f>IF(N(AC17)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC17&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC17&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN17" s="10" t="n"/>
+      <c r="AN17" s="10" t="inlineStr">
+        <is>
+          <t>Cancelled in Buffer 2026-10-15 before posting: Shivam retired the 8-bit avatar format (Ted type 2 only)</t>
+        </is>
+      </c>
       <c r="AO17" s="10" t="inlineStr">
         <is>
           <t>whiteboard</t>
@@ -2450,7 +2482,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I19" s="10" t="n">
@@ -2461,16 +2493,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K19" s="10" t="n"/>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>interleaving</t>
+        </is>
+      </c>
       <c r="L19" s="11" t="n"/>
       <c r="M19" s="5">
         <f>IF(L19="","",TEXT(L19,"ddd"))</f>
         <v/>
       </c>
-      <c r="N19" s="10" t="n"/>
+      <c r="N19" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O19" s="10" t="n"/>
       <c r="P19" s="10" t="n"/>
-      <c r="Q19" s="10" t="n"/>
+      <c r="Q19" s="10" t="inlineStr">
+        <is>
+          <t>Rohrer &amp; Taylor 2007, Instructional Science 35:481-498; practice 89% blocked vs 60% mixed; test 1 wk later 63% mixed vs 20% blocked</t>
+        </is>
+      </c>
       <c r="R19" s="10" t="n"/>
       <c r="S19" s="12" t="n"/>
       <c r="T19" s="10" t="n"/>
@@ -2514,7 +2558,7 @@
       <c r="AN19" s="10" t="n"/>
       <c r="AO19" s="10" t="inlineStr">
         <is>
-          <t>blueprint</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2596,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I20" s="10" t="n">
@@ -2563,16 +2607,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K20" s="10" t="n"/>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>memory-rebuilds</t>
+        </is>
+      </c>
       <c r="L20" s="11" t="n"/>
       <c r="M20" s="5">
         <f>IF(L20="","",TEXT(L20,"ddd"))</f>
         <v/>
       </c>
-      <c r="N20" s="10" t="n"/>
+      <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O20" s="10" t="n"/>
       <c r="P20" s="10" t="n"/>
-      <c r="Q20" s="10" t="n"/>
+      <c r="Q20" s="10" t="inlineStr">
+        <is>
+          <t>Loftus &amp; Palmer 1974, JVLVB 13(5):585-589; smashed 40.5 mph vs hit 34.0; broken glass 32% vs 14%</t>
+        </is>
+      </c>
       <c r="R20" s="10" t="n"/>
       <c r="S20" s="12" t="n"/>
       <c r="T20" s="10" t="n"/>
@@ -2616,7 +2672,7 @@
       <c r="AN20" s="10" t="n"/>
       <c r="AO20" s="10" t="inlineStr">
         <is>
-          <t>one-line</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -3494,7 +3550,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I29" s="10" t="n">
@@ -3579,7 +3635,11 @@
         <f>IF(N(AC29)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC29&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC29&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN29" s="10" t="n"/>
+      <c r="AN29" s="10" t="inlineStr">
+        <is>
+          <t>Cancelled in Buffer 2026-10-15 before posting: Shivam retired the 8-bit avatar format (Ted type 2 only)</t>
+        </is>
+      </c>
       <c r="AO29" s="10" t="inlineStr">
         <is>
           <t>terminal</t>
@@ -4904,7 +4964,7 @@
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I42" s="10" t="n">
@@ -4915,16 +4975,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K42" s="10" t="n"/>
+      <c r="K42" s="10" t="inlineStr">
+        <is>
+          <t>immediate-rewards</t>
+        </is>
+      </c>
       <c r="L42" s="11" t="n"/>
       <c r="M42" s="5">
         <f>IF(L42="","",TEXT(L42,"ddd"))</f>
         <v/>
       </c>
-      <c r="N42" s="10" t="n"/>
+      <c r="N42" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O42" s="10" t="n"/>
       <c r="P42" s="10" t="n"/>
-      <c r="Q42" s="10" t="n"/>
+      <c r="Q42" s="10" t="inlineStr">
+        <is>
+          <t>Woolley &amp; Fishbach 2018, JPSP 114(6):877-890; immediate vs delayed rewards increase interest/persistence after reward ends</t>
+        </is>
+      </c>
       <c r="R42" s="10" t="n"/>
       <c r="S42" s="12" t="n"/>
       <c r="T42" s="10" t="n"/>
@@ -4968,7 +5040,7 @@
       <c r="AN42" s="10" t="n"/>
       <c r="AO42" s="10" t="inlineStr">
         <is>
-          <t>game-show</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -7798,7 +7870,7 @@
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I69" s="10" t="n">
@@ -7809,16 +7881,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K69" s="10" t="n"/>
+      <c r="K69" s="10" t="inlineStr">
+        <is>
+          <t>social-proof</t>
+        </is>
+      </c>
       <c r="L69" s="11" t="n"/>
       <c r="M69" s="5">
         <f>IF(L69="","",TEXT(L69,"ddd"))</f>
         <v/>
       </c>
-      <c r="N69" s="10" t="n"/>
+      <c r="N69" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O69" s="10" t="n"/>
       <c r="P69" s="10" t="n"/>
-      <c r="Q69" s="10" t="n"/>
+      <c r="Q69" s="10" t="inlineStr">
+        <is>
+          <t>Goldstein, Cialdini &amp; Griskevicius 2008, J Consumer Research 35(3):472-482; towel reuse 35% standard, 44% descriptive norm, 49% same-room norm</t>
+        </is>
+      </c>
       <c r="R69" s="10" t="n"/>
       <c r="S69" s="12" t="n"/>
       <c r="T69" s="10" t="n"/>
@@ -7862,7 +7946,7 @@
       <c r="AN69" s="10" t="n"/>
       <c r="AO69" s="10" t="inlineStr">
         <is>
-          <t>riso</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -7900,7 +7984,7 @@
       </c>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I70" s="10" t="n">
@@ -7911,16 +7995,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K70" s="10" t="n"/>
+      <c r="K70" s="10" t="inlineStr">
+        <is>
+          <t>bystander-effect</t>
+        </is>
+      </c>
       <c r="L70" s="11" t="n"/>
       <c r="M70" s="5">
         <f>IF(L70="","",TEXT(L70,"ddd"))</f>
         <v/>
       </c>
-      <c r="N70" s="10" t="n"/>
+      <c r="N70" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O70" s="10" t="n"/>
       <c r="P70" s="10" t="n"/>
-      <c r="Q70" s="10" t="n"/>
+      <c r="Q70" s="10" t="inlineStr">
+        <is>
+          <t>Darley &amp; Latane 1968, JPSP 8(4):377-383; alone 85% helped before seizure ended vs 31% with four others</t>
+        </is>
+      </c>
       <c r="R70" s="10" t="n"/>
       <c r="S70" s="12" t="n"/>
       <c r="T70" s="10" t="n"/>
@@ -7964,7 +8060,7 @@
       <c r="AN70" s="10" t="n"/>
       <c r="AO70" s="10" t="inlineStr">
         <is>
-          <t>dossier</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -9922,7 +10018,7 @@
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I89" s="10" t="n">
@@ -9933,16 +10029,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K89" s="10" t="n"/>
+      <c r="K89" s="10" t="inlineStr">
+        <is>
+          <t>highlight-reel</t>
+        </is>
+      </c>
       <c r="L89" s="11" t="n"/>
       <c r="M89" s="5">
         <f>IF(L89="","",TEXT(L89,"ddd"))</f>
         <v/>
       </c>
-      <c r="N89" s="10" t="n"/>
+      <c r="N89" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O89" s="10" t="n"/>
       <c r="P89" s="10" t="n"/>
-      <c r="Q89" s="10" t="n"/>
+      <c r="Q89" s="10" t="inlineStr">
+        <is>
+          <t>Jordan et al. 2011, PSPB 37(1):120-135; peers' negative emotions underestimated, positive overestimated; linked to loneliness, lower life satisfaction</t>
+        </is>
+      </c>
       <c r="R89" s="10" t="n"/>
       <c r="S89" s="12" t="n"/>
       <c r="T89" s="10" t="n"/>
@@ -9986,7 +10094,7 @@
       <c r="AN89" s="10" t="n"/>
       <c r="AO89" s="10" t="inlineStr">
         <is>
-          <t>riso</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -10024,7 +10132,7 @@
       </c>
       <c r="H90" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I90" s="10" t="n">
@@ -10035,16 +10143,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K90" s="10" t="n"/>
+      <c r="K90" s="10" t="inlineStr">
+        <is>
+          <t>fomo</t>
+        </is>
+      </c>
       <c r="L90" s="11" t="n"/>
       <c r="M90" s="5">
         <f>IF(L90="","",TEXT(L90,"ddd"))</f>
         <v/>
       </c>
-      <c r="N90" s="10" t="n"/>
+      <c r="N90" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O90" s="10" t="n"/>
       <c r="P90" s="10" t="n"/>
-      <c r="Q90" s="10" t="n"/>
+      <c r="Q90" s="10" t="inlineStr">
+        <is>
+          <t>Przybylski et al. 2013, Computers in Human Behavior 29(4):1841-1848; FOMO correlates w/ lower mood &amp; life satisfaction, social media in lectures/driving</t>
+        </is>
+      </c>
       <c r="R90" s="10" t="n"/>
       <c r="S90" s="12" t="n"/>
       <c r="T90" s="10" t="n"/>
@@ -10088,7 +10208,7 @@
       <c r="AN90" s="10" t="n"/>
       <c r="AO90" s="10" t="inlineStr">
         <is>
-          <t>terminal</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -10126,7 +10246,7 @@
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I91" s="10" t="n">
@@ -10137,16 +10257,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K91" s="10" t="n"/>
+      <c r="K91" s="10" t="inlineStr">
+        <is>
+          <t>loss-framing</t>
+        </is>
+      </c>
       <c r="L91" s="11" t="n"/>
       <c r="M91" s="5">
         <f>IF(L91="","",TEXT(L91,"ddd"))</f>
         <v/>
       </c>
-      <c r="N91" s="10" t="n"/>
+      <c r="N91" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O91" s="10" t="n"/>
       <c r="P91" s="10" t="n"/>
-      <c r="Q91" s="10" t="n"/>
+      <c r="Q91" s="10" t="inlineStr">
+        <is>
+          <t>Tversky &amp; Kahneman 1981, Science 211(4481):453-458; 200 saved 72% vs 400 die 22%</t>
+        </is>
+      </c>
       <c r="R91" s="10" t="n"/>
       <c r="S91" s="12" t="n"/>
       <c r="T91" s="10" t="n"/>
@@ -10190,7 +10322,7 @@
       <c r="AN91" s="10" t="n"/>
       <c r="AO91" s="10" t="inlineStr">
         <is>
-          <t>swiss</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10768,7 @@
       </c>
       <c r="H96" s="5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I96" s="10" t="n">
@@ -10721,7 +10853,11 @@
         <f>IF(N(AC96)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC96&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC96&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN96" s="10" t="n"/>
+      <c r="AN96" s="10" t="inlineStr">
+        <is>
+          <t>Cancelled in Buffer 2026-10-15 before posting: Shivam retired the 8-bit avatar format (Ted type 2 only)</t>
+        </is>
+      </c>
       <c r="AO96" s="10" t="inlineStr">
         <is>
           <t>whiteboard</t>
@@ -10876,7 +11012,7 @@
       </c>
       <c r="H98" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I98" s="10" t="n">
@@ -10887,16 +11023,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K98" s="10" t="n"/>
+      <c r="K98" s="10" t="inlineStr">
+        <is>
+          <t>ten-percent-myth</t>
+        </is>
+      </c>
       <c r="L98" s="11" t="n"/>
       <c r="M98" s="5">
         <f>IF(L98="","",TEXT(L98,"ddd"))</f>
         <v/>
       </c>
-      <c r="N98" s="10" t="n"/>
+      <c r="N98" s="10" t="inlineStr">
+        <is>
+          <t>thoughts</t>
+        </is>
+      </c>
       <c r="O98" s="10" t="n"/>
       <c r="P98" s="10" t="n"/>
-      <c r="Q98" s="10" t="n"/>
+      <c r="Q98" s="10" t="inlineStr">
+        <is>
+          <t>Beyerstein 1999, in Mind Myths (Della Sala ed.); imaging shows activity across all regions; brain ~2% body weight, ~20% energy</t>
+        </is>
+      </c>
       <c r="R98" s="10" t="n"/>
       <c r="S98" s="12" t="n"/>
       <c r="T98" s="10" t="n"/>
@@ -10940,7 +11088,7 @@
       <c r="AN98" s="10" t="n"/>
       <c r="AO98" s="10" t="inlineStr">
         <is>
-          <t>dossier</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>
@@ -10978,7 +11126,7 @@
       </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I99" s="10" t="n">
@@ -10989,16 +11137,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K99" s="10" t="n"/>
+      <c r="K99" s="10" t="inlineStr">
+        <is>
+          <t>body-language-lies</t>
+        </is>
+      </c>
       <c r="L99" s="11" t="n"/>
       <c r="M99" s="5">
         <f>IF(L99="","",TEXT(L99,"ddd"))</f>
         <v/>
       </c>
-      <c r="N99" s="10" t="n"/>
+      <c r="N99" s="10" t="inlineStr">
+        <is>
+          <t>eyes</t>
+        </is>
+      </c>
       <c r="O99" s="10" t="n"/>
       <c r="P99" s="10" t="n"/>
-      <c r="Q99" s="10" t="n"/>
+      <c r="Q99" s="10" t="inlineStr">
+        <is>
+          <t>Bond &amp; DePaulo 2006, PSPR 10(3):214-234; 206 studies, ~24,000 judges, 54% accuracy</t>
+        </is>
+      </c>
       <c r="R99" s="10" t="n"/>
       <c r="S99" s="12" t="n"/>
       <c r="T99" s="10" t="n"/>
@@ -11042,7 +11202,7 @@
       <c r="AN99" s="10" t="n"/>
       <c r="AO99" s="10" t="inlineStr">
         <is>
-          <t>spy-noir</t>
+          <t>ted2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
One More Never Enough: prebuilt Short (Shivam's Claude Design / Remotion build)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Long form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Looks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AO106"/>
+  <dimension ref="A2:AO107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11992,6 +11992,108 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Digital life and consumer behavior</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Why one more never feels like enough (dopamine and checking)</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>You opened your phone for a minute.</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>Dopamine helps the brain learn what to pursue; uncertain rewards keep you checking; small steps to make room for what matters.</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Claude Design editorial animation (One More Never Enough)</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I107" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="J107" s="10" t="n"/>
+      <c r="K107" s="10" t="inlineStr">
+        <is>
+          <t>one-more</t>
+        </is>
+      </c>
+      <c r="L107" s="11" t="n"/>
+      <c r="M107" s="5">
+        <f>IF(L107="","",TEXT(L107,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N107" s="10" t="n"/>
+      <c r="O107" s="10" t="n"/>
+      <c r="P107" s="10" t="n"/>
+      <c r="Q107" s="10" t="n"/>
+      <c r="R107" s="10" t="n"/>
+      <c r="S107" s="12" t="n"/>
+      <c r="T107" s="10" t="n"/>
+      <c r="U107" s="13">
+        <f>IF(OR(T107="",N(O107)=0),"",T107/O107)</f>
+        <v/>
+      </c>
+      <c r="V107" s="10" t="n"/>
+      <c r="W107" s="10" t="n"/>
+      <c r="X107" s="10" t="n"/>
+      <c r="Y107" s="12" t="n"/>
+      <c r="Z107" s="10" t="n"/>
+      <c r="AA107" s="12" t="n"/>
+      <c r="AB107" s="10" t="n"/>
+      <c r="AC107" s="14">
+        <f>IF(COUNT(S107,Y107,AA107)=0,"",SUM(S107,Y107,AA107))</f>
+        <v/>
+      </c>
+      <c r="AD107" s="13">
+        <f>IF(N(AC107)=0,"",SUM(V107,W107,X107,Z107,AB107)/AC107)</f>
+        <v/>
+      </c>
+      <c r="AE107" s="12" t="n"/>
+      <c r="AF107" s="12" t="n"/>
+      <c r="AG107" s="12" t="n"/>
+      <c r="AH107" s="14">
+        <f>IF(COUNT(AE107,AF107,AG107)=0,"",SUM(AE107,AF107,AG107))</f>
+        <v/>
+      </c>
+      <c r="AI107" s="12" t="n"/>
+      <c r="AJ107" s="12" t="n"/>
+      <c r="AK107" s="12" t="n"/>
+      <c r="AL107" s="14">
+        <f>IF(COUNT(AI107,AJ107,AK107)=0,"",SUM(AI107,AJ107,AK107))</f>
+        <v/>
+      </c>
+      <c r="AM107" s="5">
+        <f>IF(N(AC107)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC107&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC107&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN107" s="10" t="n"/>
+      <c r="AO107" s="10" t="inlineStr">
+        <is>
+          <t>editorial</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="AM6:AM105">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -12002,13 +12104,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H6:H106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Idea,Researching,Scripted,Scheduled,Published,Vetoed,Failed,Filming,Editing"</formula1>
     </dataValidation>
-    <dataValidation sqref="J6:J106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J6:J107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Strong,Weak"</formula1>
     </dataValidation>
-    <dataValidation sqref="AO6:AO106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AO6:AO107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Looks!$A$5:$A$21</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
tracker: six ideas set to story format (rows 6, 9, 16, 18, 23, 66)
Each has an animation style, storyboard, palette & type, characters and sound
cues for the script writer to follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0197TpBHCejxxHq4ERPHmDRZ
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1781,12 +1781,36 @@
           <t>riso</t>
         </is>
       </c>
-      <c r="AP11" s="51" t="n"/>
-      <c r="AQ11" s="51" t="n"/>
-      <c r="AR11" s="51" t="n"/>
-      <c r="AS11" s="51" t="n"/>
-      <c r="AT11" s="51" t="n"/>
-      <c r="AU11" s="51" t="n"/>
+      <c r="AP11" s="51" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="AQ11" s="51" t="inlineStr">
+        <is>
+          <t>Soft glow editorial: dusk gradient, a literal halo ring that tints everything it touches; slow push-ins.</t>
+        </is>
+      </c>
+      <c r="AR11" s="51" t="inlineStr">
+        <is>
+          <t>1. Hook: can one good trait change how you see everything else? 2. The same lecturer shown twice: warm and friendly vs cold and strict. 3. The study (Nisbett &amp; Wilson, 1977). 4. The stat: students rated the same looks, accent and mannerisms as appealing only when he was warm - and didn't know why. 5. Why: one impression colours the rest. 6. Takeaway: judge traits one at a time.</t>
+        </is>
+      </c>
+      <c r="AS11" s="51" t="inlineStr">
+        <is>
+          <t>Dusk violet #2D1B69, peach #FFB38A, gold halo #FFD66B, cream text; Playfair Display headlines, Barlow captions</t>
+        </is>
+      </c>
+      <c r="AT11" s="51" t="inlineStr">
+        <is>
+          <t>A lecturer (the One More protagonist with glasses), seen twice: warm and cold</t>
+        </is>
+      </c>
+      <c r="AU11" s="51" t="inlineStr">
+        <is>
+          <t>A chime when the halo appears, a flip between the warm and cold versions, a rising tone on the stat</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -2105,12 +2129,36 @@
           <t>keynote</t>
         </is>
       </c>
-      <c r="AP14" s="51" t="n"/>
-      <c r="AQ14" s="51" t="n"/>
-      <c r="AR14" s="51" t="n"/>
-      <c r="AS14" s="51" t="n"/>
-      <c r="AT14" s="51" t="n"/>
-      <c r="AU14" s="51" t="n"/>
+      <c r="AP14" s="51" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="AQ14" s="51" t="inlineStr">
+        <is>
+          <t>Minimal Swiss: white grid, black type, one red accent, a giant checkbox, crisp sliding panels and bar charts.</t>
+        </is>
+      </c>
+      <c r="AR14" s="51" t="inlineStr">
+        <is>
+          <t>1. Hook: a form with a box already ticked - did you choose it? 2. Two countries' donor forms side by side: opt in vs opt out. 3. The study (Johnson &amp; Goldstein, 2003). 4. The stat: consent bars - low where you must opt in, near 100% where you must opt out. 5. Why: doing nothing is easiest and feels recommended. 6. Takeaway: check what's pre-selected, and set good defaults for yourself.</t>
+        </is>
+      </c>
+      <c r="AS14" s="51" t="inlineStr">
+        <is>
+          <t>White, black #111111, red #E30613; Inter Tight headlines, Inter captions</t>
+        </is>
+      </c>
+      <c r="AT14" s="51" t="inlineStr">
+        <is>
+          <t>None - objects only (forms, checkboxes, a pen)</t>
+        </is>
+      </c>
+      <c r="AU14" s="51" t="inlineStr">
+        <is>
+          <t>Toggle click on the checkbox, pen tick, card slides, a settle when the bars stop</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -2949,12 +2997,36 @@
           <t>dossier</t>
         </is>
       </c>
-      <c r="AP21" s="51" t="n"/>
-      <c r="AQ21" s="51" t="n"/>
-      <c r="AR21" s="51" t="n"/>
-      <c r="AS21" s="51" t="n"/>
-      <c r="AT21" s="51" t="n"/>
-      <c r="AU21" s="51" t="n"/>
+      <c r="AP21" s="51" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="AQ21" s="51" t="inlineStr">
+        <is>
+          <t>Noir detective sketch: charcoal lines on cream paper, one red spot colour, slow pans across a crime board; the remembered scene redraws itself as the question changes.</t>
+        </is>
+      </c>
+      <c r="AR21" s="51" t="inlineStr">
+        <is>
+          <t>1. Hook: two cars bump at a junction; a witness watches. 2. A detective asks 'how fast were they going when they SMASHED?' - the word cracks the frame. 3. The study (Loftus &amp; Palmer, 1974): a film clip, two question cards, hit vs smashed. 4. The stat: two speedometers (lower for hit, higher for smashed); a week later, broken glass appears in the memory that was never in the film. 5. Why: each retelling redraws the memory - pencil strokes move. 6. Takeaway: ask open questions and write it down early.</t>
+        </is>
+      </c>
+      <c r="AS21" s="51" t="inlineStr">
+        <is>
+          <t>Cream paper #F3EBDD, charcoal ink #1E1B18, crime red #C8322B; Bebas Neue headlines, Courier Prime captions</t>
+        </is>
+      </c>
+      <c r="AT21" s="51" t="inlineStr">
+        <is>
+          <t>The witness (the One More protagonist redrawn in charcoal) and a faceless detective silhouette</t>
+        </is>
+      </c>
+      <c r="AU21" s="51" t="inlineStr">
+        <is>
+          <t>Soft car bump, pen scratches on the board, a glass tinkle when the broken glass appears, a page turn at the end</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="5" t="n">
@@ -3165,12 +3237,36 @@
           <t>data-story</t>
         </is>
       </c>
-      <c r="AP23" s="51" t="n"/>
-      <c r="AQ23" s="51" t="n"/>
-      <c r="AR23" s="51" t="n"/>
-      <c r="AS23" s="51" t="n"/>
-      <c r="AT23" s="51" t="n"/>
-      <c r="AU23" s="51" t="n"/>
+      <c r="AP23" s="51" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="AQ23" s="51" t="inlineStr">
+        <is>
+          <t>Game-show flat: a list of words on flip cards, then a U-shaped curve drawn live like a scoreboard; bouncy pops.</t>
+        </is>
+      </c>
+      <c r="AR23" s="51" t="inlineStr">
+        <is>
+          <t>1. Hook: try to remember this list - 12 words flip by. 2. Which ones stuck? The first and last glow. 3. The study (Murdock, 1962): people recalled word lists; points appear on a chart. 4. The stat: a U-curve - first (primacy) and last (recency) remembered best, the middle dips. 5. Why: early words get rehearsed, the last ones are still in mind. 6. Takeaway: put the important point first or last.</t>
+        </is>
+      </c>
+      <c r="AS23" s="51" t="inlineStr">
+        <is>
+          <t>Violet stage #4B2AA5, gold #FFD23F, white cards, pink #FF4FA3; Fredoka headlines, Nunito captions</t>
+        </is>
+      </c>
+      <c r="AT23" s="51" t="inlineStr">
+        <is>
+          <t>A quiz host (the One More protagonist in a bow tie)</t>
+        </is>
+      </c>
+      <c r="AU23" s="51" t="inlineStr">
+        <is>
+          <t>A card flip and tick per word, a rising tone as the curve draws, chime-bright on the takeaway</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="5" t="n">
@@ -3769,12 +3865,36 @@
           <t>spy-noir</t>
         </is>
       </c>
-      <c r="AP28" s="51" t="n"/>
-      <c r="AQ28" s="51" t="n"/>
-      <c r="AR28" s="51" t="n"/>
-      <c r="AS28" s="51" t="n"/>
-      <c r="AT28" s="51" t="n"/>
-      <c r="AU28" s="51" t="n"/>
+      <c r="AP28" s="51" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="AQ28" s="51" t="inlineStr">
+        <is>
+          <t>Bright flat cartoon street, playful and fast; spot-the-difference flicker panels; a big door slides through the frame and hides a swap.</t>
+        </is>
+      </c>
+      <c r="AR28" s="51" t="inlineStr">
+        <is>
+          <t>1. Hook: two pictures flicker - what changed? 2. A tourist with a map asks a stranger for directions. 3. Two workers carry a door between them; behind it the stranger is swapped for a different person. 4. The stat (Simons &amp; Levin, 1998): about half of people kept giving directions without noticing. 5. Why: we keep the gist, not the details. 6. Takeaway: double-check the details that matter.</t>
+        </is>
+      </c>
+      <c r="AS28" s="51" t="inlineStr">
+        <is>
+          <t>Sky #8FD3FF, sunny yellow #FFD447, coral #FF6B5B, ink #1D1D2C; Fredoka headlines, Nunito captions</t>
+        </is>
+      </c>
+      <c r="AT28" s="51" t="inlineStr">
+        <is>
+          <t>Two different strangers (one in a cap, one in glasses), a tourist with a map, two door carriers</t>
+        </is>
+      </c>
+      <c r="AU28" s="51" t="inlineStr">
+        <is>
+          <t>Camera-shutter flicker, footsteps, a whoosh as the door passes, a bright chime on the reveal</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="5" t="n">
@@ -8701,12 +8821,36 @@
           <t>blueprint</t>
         </is>
       </c>
-      <c r="AP71" s="51" t="n"/>
-      <c r="AQ71" s="51" t="n"/>
-      <c r="AR71" s="51" t="n"/>
-      <c r="AS71" s="51" t="n"/>
-      <c r="AT71" s="51" t="n"/>
-      <c r="AU71" s="51" t="n"/>
+      <c r="AP71" s="51" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="AQ71" s="51" t="inlineStr">
+        <is>
+          <t>Warm risograph print: grainy blue and fluorescent pink overprint, slightly misregistered; a tug-of-war rope and bouncy little figures.</t>
+        </is>
+      </c>
+      <c r="AR71" s="51" t="inlineStr">
+        <is>
+          <t>1. Hook: group project - who actually did the work? 2. Tug of war: one person pulls hard alone; as more join, each pulls less. 3. The study (Latane, Williams &amp; Harkins, 1979): blindfolded people shouting and clapping alone or in groups. 4. The stat: noise per person drops as the group grows. 5. Why: effort hides in a crowd. 6. Takeaway: make each person's part visible.</t>
+        </is>
+      </c>
+      <c r="AS71" s="51" t="inlineStr">
+        <is>
+          <t>Riso blue #0078BF, fluorescent pink #FF48B0, paper #F4EEE2; Rubik headlines and captions</t>
+        </is>
+      </c>
+      <c r="AT71" s="51" t="inlineStr">
+        <is>
+          <t>A crowd of small figures; the One More protagonist as the one who notices</t>
+        </is>
+      </c>
+      <c r="AU71" s="51" t="inlineStr">
+        <is>
+          <t>A whoosh per person who joins, airy fades as effort drops, three wooden taps at the end</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="60" customHeight="1">
       <c r="A72" s="5" t="n">

</xml_diff>

<commit_message>
scripts: 3 new (story: halo-warm, social-loafing, serial-position)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WAhXGtcLABXXJpnbCufssy
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Long form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Looks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
@@ -1725,16 +1725,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K11" s="10" t="n"/>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>halo-warm</t>
+        </is>
+      </c>
       <c r="L11" s="11" t="n"/>
       <c r="M11" s="5">
         <f>IF(L11="","",TEXT(L11,"ddd"))</f>
         <v/>
       </c>
-      <c r="N11" s="10" t="n"/>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
       <c r="O11" s="10" t="n"/>
       <c r="P11" s="10" t="n"/>
-      <c r="Q11" s="10" t="n"/>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Nisbett, R. E. &amp; Wilson, T. D. (1977). The halo effect: Evidence for unconscious alteration of judgments. JPSP 35(4):250-256 (118 Michigan students; warm vs cold guise of the same Belgian-accented instructor; most warm-condition subjects rated appearance and mannerisms appealing, most cold-condition subjects irritating, accent overwhelmingly irritating when cold; subjects denied liking affected ratings)</t>
+        </is>
+      </c>
       <c r="R11" s="10" t="n"/>
       <c r="S11" s="12" t="n"/>
       <c r="T11" s="10" t="n"/>
@@ -1775,7 +1787,11 @@
         <f>IF(N(AC11)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC11&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC11&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN11" s="10" t="n"/>
+      <c r="AN11" s="10" t="inlineStr">
+        <is>
+          <t>Story Short (2026-10-17). Held from posting until 2026-11-01.</t>
+        </is>
+      </c>
       <c r="AO11" s="10" t="inlineStr">
         <is>
           <t>riso</t>
@@ -2999,7 +3015,11 @@
         <f>IF(N(AC21)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC21&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC21&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN21" s="10" t="n"/>
+      <c r="AN21" s="10" t="inlineStr">
+        <is>
+          <t>Skipped by script writer 2026-10-17: storyboard is the same Loftus &amp; Palmer (1974) study as memory-rebuilds (No. 15, already Scripted) - near-duplicate. Needs a different angle (e.g. Loftus, Miller &amp; Burns 1978 stop/yield sign) or a later slot.</t>
+        </is>
+      </c>
       <c r="AO21" s="10" t="inlineStr">
         <is>
           <t>dossier</t>
@@ -3178,7 +3198,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I23" s="10" t="n">
@@ -3189,16 +3209,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K23" s="10" t="n"/>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>serial-position</t>
+        </is>
+      </c>
       <c r="L23" s="11" t="n"/>
       <c r="M23" s="5">
         <f>IF(L23="","",TEXT(L23,"ddd"))</f>
         <v/>
       </c>
-      <c r="N23" s="10" t="n"/>
+      <c r="N23" s="10" t="inlineStr">
+        <is>
+          <t>challenge</t>
+        </is>
+      </c>
       <c r="O23" s="10" t="n"/>
       <c r="P23" s="10" t="n"/>
-      <c r="Q23" s="10" t="n"/>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>Murdock, B. B., Jr. (1962). The serial position effect of free recall. J Exp Psychol 64(5):482-488 (free recall of 10-40 word lists; U-shaped curve with primacy and recency); rehearsal/short-term memory account per Rundus (1971), Glanzer &amp; Cunitz (1966)</t>
+        </is>
+      </c>
       <c r="R23" s="10" t="n"/>
       <c r="S23" s="12" t="n"/>
       <c r="T23" s="10" t="n"/>
@@ -3239,7 +3271,11 @@
         <f>IF(N(AC23)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC23&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC23&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN23" s="10" t="n"/>
+      <c r="AN23" s="10" t="inlineStr">
+        <is>
+          <t>Story Short (2026-10-17). Headline font Baloo 2 instead of Fredoka (Fredoka has no 800 weight, which the build requests). Held from posting until 2026-11-01.</t>
+        </is>
+      </c>
       <c r="AO23" s="10" t="inlineStr">
         <is>
           <t>data-story</t>
@@ -8778,7 +8814,7 @@
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I71" s="10" t="n">
@@ -8789,16 +8825,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K71" s="10" t="n"/>
+      <c r="K71" s="10" t="inlineStr">
+        <is>
+          <t>social-loafing</t>
+        </is>
+      </c>
       <c r="L71" s="11" t="n"/>
       <c r="M71" s="5">
         <f>IF(L71="","",TEXT(L71,"ddd"))</f>
         <v/>
       </c>
-      <c r="N71" s="10" t="n"/>
+      <c r="N71" s="10" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
       <c r="O71" s="10" t="n"/>
       <c r="P71" s="10" t="n"/>
-      <c r="Q71" s="10" t="n"/>
+      <c r="Q71" s="10" t="inlineStr">
+        <is>
+          <t>Latané, B., Williams, K. &amp; Harkins, S. (1979). Many hands make light the work. JPSP 37(6):822-832 (Exp 1 clapping/shouting: per-person output 71% in pairs, 51% in 4s, 40% in 6s; Exp 2 blindfolded + headphones pseudogroups: 82% / 74% when only believing others shouted)</t>
+        </is>
+      </c>
       <c r="R71" s="10" t="n"/>
       <c r="S71" s="12" t="n"/>
       <c r="T71" s="10" t="n"/>
@@ -8839,7 +8887,11 @@
         <f>IF(N(AC71)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC71&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC71&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN71" s="10" t="n"/>
+      <c r="AN71" s="10" t="inlineStr">
+        <is>
+          <t>Story Short (2026-10-17). Held from posting until 2026-11-01.</t>
+        </is>
+      </c>
       <c r="AO71" s="10" t="inlineStr">
         <is>
           <t>blueprint</t>

</xml_diff>

<commit_message>
Weekly review 2026-10-18: no per-video stats in Metricool; Instagram missing on Buffer posts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013gopdTJVHwQwbRFvxdNzgH
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Long form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Looks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="AN6" s="10" t="inlineStr">
         <is>
-          <t>Pilot: 16:9 horizontal, YouTube only — not comparable with the vertical Shorts.</t>
+          <t>Pilot: 16:9 horizontal, YouTube only — not comparable with the vertical Shorts. 2026-10-18 review: d7 stats not available (Metricool per-video YouTube data empty).</t>
         </is>
       </c>
       <c r="AO6" s="10" t="inlineStr">
@@ -2403,7 +2403,11 @@
         <f>IF(N(AC16)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC16&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC16&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN16" s="10" t="n"/>
+      <c r="AN16" s="10" t="inlineStr">
+        <is>
+          <t>Metricool confirms published 2026-10-12 on YouTube, Instagram and TikTok (Status still Scheduled; left for the workflow/Shivam). Per-video stats not in Metricool yet.</t>
+        </is>
+      </c>
       <c r="AO16" s="10" t="inlineStr">
         <is>
           <t>pixel-lab</t>
@@ -3795,7 +3799,11 @@
         <f>IF(N(AC27)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC27&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC27&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN27" s="10" t="n"/>
+      <c r="AN27" s="10" t="inlineStr">
+        <is>
+          <t>Metricool: published 2026-10-13 on YouTube + TikTok; Instagram ERROR (Unknown). Status still Scheduled. Per-video stats not in Metricool yet.</t>
+        </is>
+      </c>
       <c r="AO27" s="10" t="inlineStr">
         <is>
           <t>pixel-lab</t>

</xml_diff>

<commit_message>
Fix Published status: read Buffer posts per channel
A locked Buffer channel (reconnected Instagram, since Oct 15) made the
all-channels posts query fail, so reconcile silently skipped and no row
left Scheduled. Posts are now listed one channel at a time; unreadable
channels never count as deleted, and failures show in the daily issue.
Also marks No. 11 and 22 (posted via Metricool) Published.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JTVwXxJ1DJYhcYjPa1XYkK
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Long form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Looks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="I16" s="10" t="n">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="I27" s="10" t="n">

</xml_diff>

<commit_message>
ci: instagram catch-up 2026-10-18
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Long form" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Looks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="R8" s="10" t="inlineStr">
         <is>
-          <t>buffer:youtube=6ad14adb2b2233d4661582ae;tiktok=6ad14adc5533140b41cadc37</t>
+          <t>buffer:youtube=6ad14adb2b2233d4661582ae;tiktok=6ad14adc5533140b41cadc37;instagram=6ad5279e769b457934da2d97</t>
         </is>
       </c>
       <c r="S8" s="12" t="n"/>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
-          <t>buffer:youtube=6ad514440a208cb32379c365;tiktok=6ad51445938409f1d0e23e43</t>
+          <t>buffer:youtube=6ad514440a208cb32379c365;tiktok=6ad51445938409f1d0e23e43;instagram=6ad5279dae173d6e0017d665</t>
         </is>
       </c>
       <c r="S9" s="12" t="n"/>
@@ -10977,7 +10977,7 @@
       </c>
       <c r="R89" s="10" t="inlineStr">
         <is>
-          <t>buffer:youtube=6ad51440769b457934d63ba1;tiktok=6ad51440938409f1d0e23dff</t>
+          <t>buffer:youtube=6ad51440769b457934d63ba1;tiktok=6ad51440938409f1d0e23dff;instagram=6ad5279cae173d6e0017d609</t>
         </is>
       </c>
       <c r="S89" s="12" t="n"/>
@@ -12041,7 +12041,7 @@
       </c>
       <c r="R98" s="10" t="inlineStr">
         <is>
-          <t>buffer:youtube=6ad51441769b457934d63c00;tiktok=6ad514430a208cb32379c33b</t>
+          <t>buffer:youtube=6ad51441769b457934d63c00;tiktok=6ad514430a208cb32379c33b;instagram=6ad5279c938409f1d0e61830</t>
         </is>
       </c>
       <c r="S98" s="12" t="n"/>

</xml_diff>

<commit_message>
scripts: 8 new (6 Ted type 2, 2 story)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VwCks5bjxDZd79FzW4tKmb
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="H14" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I14" s="69" t="n">
@@ -2589,16 +2589,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K14" s="69" t="n"/>
+      <c r="K14" s="69" t="inlineStr">
+        <is>
+          <t>default-effect</t>
+        </is>
+      </c>
       <c r="L14" s="70" t="n"/>
       <c r="M14" s="68">
         <f>IF(L14="","",TEXT(L14,"ddd"))</f>
         <v/>
       </c>
-      <c r="N14" s="69" t="n"/>
+      <c r="N14" s="69" t="inlineStr">
+        <is>
+          <t>Study reveal</t>
+        </is>
+      </c>
       <c r="O14" s="69" t="n"/>
       <c r="P14" s="69" t="n"/>
-      <c r="Q14" s="69" t="n"/>
+      <c r="Q14" s="69" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Goldstein 2003, Science 'Do Defaults Save Lives?': Austria 99.98% vs Germany 12% (Columbia Business School release)</t>
+        </is>
+      </c>
       <c r="R14" s="69" t="n"/>
       <c r="S14" s="71" t="n"/>
       <c r="T14" s="69" t="n"/>
@@ -4428,7 +4440,7 @@
       </c>
       <c r="H28" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I28" s="69" t="n">
@@ -4439,16 +4451,28 @@
           <t>Weak</t>
         </is>
       </c>
-      <c r="K28" s="69" t="n"/>
+      <c r="K28" s="69" t="inlineStr">
+        <is>
+          <t>change-blindness</t>
+        </is>
+      </c>
       <c r="L28" s="70" t="n"/>
       <c r="M28" s="68">
         <f>IF(L28="","",TEXT(L28,"ddd"))</f>
         <v/>
       </c>
-      <c r="N28" s="69" t="n"/>
+      <c r="N28" s="69" t="inlineStr">
+        <is>
+          <t>Study reveal</t>
+        </is>
+      </c>
       <c r="O28" s="69" t="n"/>
       <c r="P28" s="69" t="n"/>
-      <c r="Q28" s="69" t="n"/>
+      <c r="Q28" s="69" t="inlineStr">
+        <is>
+          <t>Simons &amp; Levin 1998, Psychon Bull Rev: 7 of 15 noticed the door swap (paper PDF)</t>
+        </is>
+      </c>
       <c r="R28" s="69" t="n"/>
       <c r="S28" s="71" t="n"/>
       <c r="T28" s="69" t="n"/>
@@ -5065,7 +5089,7 @@
       </c>
       <c r="H33" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I33" s="69" t="n">
@@ -5076,16 +5100,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K33" s="69" t="n"/>
+      <c r="K33" s="69" t="inlineStr">
+        <is>
+          <t>frequency-illusion</t>
+        </is>
+      </c>
       <c r="L33" s="70" t="n"/>
       <c r="M33" s="68">
         <f>IF(L33="","",TEXT(L33,"ddd"))</f>
         <v/>
       </c>
-      <c r="N33" s="69" t="n"/>
+      <c r="N33" s="69" t="inlineStr">
+        <is>
+          <t>You-callout</t>
+        </is>
+      </c>
       <c r="O33" s="69" t="n"/>
       <c r="P33" s="69" t="n"/>
-      <c r="Q33" s="69" t="n"/>
+      <c r="Q33" s="69" t="inlineStr">
+        <is>
+          <t>Zwicky 2005, Language Log 'Just between Dr. Language and I' (term coined; OED entry noted on Language Log)</t>
+        </is>
+      </c>
       <c r="R33" s="69" t="n"/>
       <c r="S33" s="71" t="n"/>
       <c r="T33" s="69" t="n"/>
@@ -5129,7 +5165,7 @@
       <c r="AN33" s="69" t="n"/>
       <c r="AO33" s="69" t="inlineStr">
         <is>
-          <t>dossier</t>
+          <t>ted2</t>
         </is>
       </c>
       <c r="AP33" s="74" t="n"/>
@@ -5178,7 +5214,7 @@
       </c>
       <c r="H34" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I34" s="69" t="n">
@@ -5189,16 +5225,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K34" s="69" t="n"/>
+      <c r="K34" s="69" t="inlineStr">
+        <is>
+          <t>waiting-time</t>
+        </is>
+      </c>
       <c r="L34" s="70" t="n"/>
       <c r="M34" s="68">
         <f>IF(L34="","",TEXT(L34,"ddd"))</f>
         <v/>
       </c>
-      <c r="N34" s="69" t="n"/>
+      <c r="N34" s="69" t="inlineStr">
+        <is>
+          <t>Study reveal</t>
+        </is>
+      </c>
       <c r="O34" s="69" t="n"/>
       <c r="P34" s="69" t="n"/>
-      <c r="Q34" s="69" t="n"/>
+      <c r="Q34" s="69" t="inlineStr">
+        <is>
+          <t>Alex Stone, NYT 2012 'Why Waiting Is Torture' (APS summary): 8-min wait, 6x longer walk, complaints near zero; Maister 1985</t>
+        </is>
+      </c>
       <c r="R34" s="69" t="n"/>
       <c r="S34" s="71" t="n"/>
       <c r="T34" s="69" t="n"/>
@@ -5242,7 +5290,7 @@
       <c r="AN34" s="69" t="n"/>
       <c r="AO34" s="69" t="inlineStr">
         <is>
-          <t>cartoon-50s</t>
+          <t>ted2</t>
         </is>
       </c>
       <c r="AP34" s="74" t="n"/>
@@ -10655,7 +10703,7 @@
       </c>
       <c r="H79" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I79" s="69" t="n">
@@ -10666,16 +10714,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K79" s="69" t="n"/>
+      <c r="K79" s="69" t="inlineStr">
+        <is>
+          <t>perfectionism-start</t>
+        </is>
+      </c>
       <c r="L79" s="70" t="n"/>
       <c r="M79" s="68">
         <f>IF(L79="","",TEXT(L79,"ddd"))</f>
         <v/>
       </c>
-      <c r="N79" s="69" t="n"/>
+      <c r="N79" s="69" t="inlineStr">
+        <is>
+          <t>Contrarian</t>
+        </is>
+      </c>
       <c r="O79" s="69" t="n"/>
       <c r="P79" s="69" t="n"/>
-      <c r="Q79" s="69" t="n"/>
+      <c r="Q79" s="69" t="inlineStr">
+        <is>
+          <t>Sirois, Molnar &amp; Hirsch 2017, Eur J Personality (WRRO 112533): concerns r=.23 with procrastination (k=43, N≈10,000), strivings r=-.22</t>
+        </is>
+      </c>
       <c r="R79" s="69" t="n"/>
       <c r="S79" s="71" t="n"/>
       <c r="T79" s="69" t="n"/>
@@ -10719,7 +10779,7 @@
       <c r="AN79" s="69" t="n"/>
       <c r="AO79" s="69" t="inlineStr">
         <is>
-          <t>whiteboard</t>
+          <t>ted2</t>
         </is>
       </c>
       <c r="AP79" s="74" t="n"/>
@@ -10768,7 +10828,7 @@
       </c>
       <c r="H80" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I80" s="69" t="n">
@@ -10779,16 +10839,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K80" s="69" t="n"/>
+      <c r="K80" s="69" t="inlineStr">
+        <is>
+          <t>contingent-worth</t>
+        </is>
+      </c>
       <c r="L80" s="70" t="n"/>
       <c r="M80" s="68">
         <f>IF(L80="","",TEXT(L80,"ddd"))</f>
         <v/>
       </c>
-      <c r="N80" s="69" t="n"/>
+      <c r="N80" s="69" t="inlineStr">
+        <is>
+          <t>Study reveal</t>
+        </is>
+      </c>
       <c r="O80" s="69" t="n"/>
       <c r="P80" s="69" t="n"/>
-      <c r="Q80" s="69" t="n"/>
+      <c r="Q80" s="69" t="inlineStr">
+        <is>
+          <t>Crocker, Sommers &amp; Luhtanen 2002, PSPB 28:1275-1286 (year corrected from 2003; 'twice as hard' dropped)</t>
+        </is>
+      </c>
       <c r="R80" s="69" t="n"/>
       <c r="S80" s="71" t="n"/>
       <c r="T80" s="69" t="n"/>
@@ -10832,7 +10904,7 @@
       <c r="AN80" s="69" t="n"/>
       <c r="AO80" s="69" t="inlineStr">
         <is>
-          <t>one-line</t>
+          <t>ted2</t>
         </is>
       </c>
       <c r="AP80" s="74" t="n"/>
@@ -10881,7 +10953,7 @@
       </c>
       <c r="H81" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I81" s="69" t="n">
@@ -10892,16 +10964,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K81" s="69" t="n"/>
+      <c r="K81" s="69" t="inlineStr">
+        <is>
+          <t>self-serving-bias</t>
+        </is>
+      </c>
       <c r="L81" s="70" t="n"/>
       <c r="M81" s="68">
         <f>IF(L81="","",TEXT(L81,"ddd"))</f>
         <v/>
       </c>
-      <c r="N81" s="69" t="n"/>
+      <c r="N81" s="69" t="inlineStr">
+        <is>
+          <t>You-callout</t>
+        </is>
+      </c>
       <c r="O81" s="69" t="n"/>
       <c r="P81" s="69" t="n"/>
-      <c r="Q81" s="69" t="n"/>
+      <c r="Q81" s="69" t="inlineStr">
+        <is>
+          <t>Lau &amp; Russell 1980, JPSP 'Attributions in the sports pages'</t>
+        </is>
+      </c>
       <c r="R81" s="69" t="n"/>
       <c r="S81" s="71" t="n"/>
       <c r="T81" s="69" t="n"/>
@@ -10945,7 +11029,7 @@
       <c r="AN81" s="69" t="n"/>
       <c r="AO81" s="69" t="inlineStr">
         <is>
-          <t>dossier</t>
+          <t>ted2</t>
         </is>
       </c>
       <c r="AP81" s="74" t="n"/>
@@ -13212,7 +13296,7 @@
       </c>
       <c r="H100" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I100" s="69" t="n">
@@ -13223,16 +13307,28 @@
           <t>Strong</t>
         </is>
       </c>
-      <c r="K100" s="69" t="n"/>
+      <c r="K100" s="69" t="inlineStr">
+        <is>
+          <t>barnum-quiz</t>
+        </is>
+      </c>
       <c r="L100" s="70" t="n"/>
       <c r="M100" s="68">
         <f>IF(L100="","",TEXT(L100,"ddd"))</f>
         <v/>
       </c>
-      <c r="N100" s="69" t="n"/>
+      <c r="N100" s="69" t="inlineStr">
+        <is>
+          <t>Study reveal</t>
+        </is>
+      </c>
       <c r="O100" s="69" t="n"/>
       <c r="P100" s="69" t="n"/>
-      <c r="Q100" s="69" t="n"/>
+      <c r="Q100" s="69" t="inlineStr">
+        <is>
+          <t>Forer 1949 (experiment 1948), mean accuracy 4.26/5 (Wikipedia: Bertram Forer)</t>
+        </is>
+      </c>
       <c r="R100" s="69" t="n"/>
       <c r="S100" s="71" t="n"/>
       <c r="T100" s="69" t="n"/>
@@ -13276,7 +13372,7 @@
       <c r="AN100" s="69" t="n"/>
       <c r="AO100" s="69" t="inlineStr">
         <is>
-          <t>game-show</t>
+          <t>ted2</t>
         </is>
       </c>
       <c r="AP100" s="74" t="n"/>

</xml_diff>

<commit_message>
Pattern test: old queue shelved, 30 pattern ideas (10 patterns, 3 a day in rotation), first 6 scripts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -373,7 +373,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -739,6 +739,30 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -1117,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:AV107"/>
+  <dimension ref="A2:AV137"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="61" min="1" max="1"/>
@@ -2199,7 +2223,7 @@
       </c>
       <c r="H11" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I11" s="69" t="n">
@@ -2274,7 +2298,7 @@
       </c>
       <c r="AN11" s="69" t="inlineStr">
         <is>
-          <t>Story Short (2026-10-17). Held from posting until 2026-11-01.</t>
+          <t>Story Short (2026-10-17). Held from posting until 2026-11-01. | 2026-10-22: replaced by the pattern test (Shivam)</t>
         </is>
       </c>
       <c r="AO11" s="69" t="inlineStr">
@@ -2352,7 +2376,7 @@
       </c>
       <c r="H12" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I12" s="69" t="n">
@@ -2413,7 +2437,11 @@
         <f>IF(N(AC12)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC12&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC12&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN12" s="69" t="n"/>
+      <c r="AN12" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO12" s="69" t="inlineStr">
         <is>
           <t>spy-noir</t>
@@ -2465,7 +2493,7 @@
       </c>
       <c r="H13" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I13" s="69" t="n">
@@ -2526,7 +2554,11 @@
         <f>IF(N(AC13)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC13&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC13&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN13" s="69" t="n"/>
+      <c r="AN13" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO13" s="69" t="inlineStr">
         <is>
           <t>swiss</t>
@@ -2578,7 +2610,7 @@
       </c>
       <c r="H14" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I14" s="69" t="n">
@@ -2651,7 +2683,11 @@
         <f>IF(N(AC14)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC14&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC14&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN14" s="69" t="n"/>
+      <c r="AN14" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO14" s="69" t="inlineStr">
         <is>
           <t>keynote</t>
@@ -2727,7 +2763,7 @@
       </c>
       <c r="H15" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I15" s="69" t="n">
@@ -2788,7 +2824,11 @@
         <f>IF(N(AC15)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC15&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC15&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN15" s="69" t="n"/>
+      <c r="AN15" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO15" s="69" t="inlineStr">
         <is>
           <t>dossier</t>
@@ -3521,7 +3561,7 @@
       </c>
       <c r="H21" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I21" s="69" t="n">
@@ -3584,7 +3624,7 @@
       </c>
       <c r="AN21" s="69" t="inlineStr">
         <is>
-          <t>Skipped by script writer 2026-10-17: storyboard is the same Loftus &amp; Palmer (1974) study as memory-rebuilds (No. 15, already Scripted) - near-duplicate. Needs a different angle (e.g. Loftus, Miller &amp; Burns 1978 stop/yield sign) or a later slot.</t>
+          <t>Skipped by script writer 2026-10-17: storyboard is the same Loftus &amp; Palmer (1974) study as memory-rebuilds (No. 15, already Scripted) - near-duplicate. Needs a different angle (e.g. Loftus, Miller &amp; Burns 1978 stop/yield sign) or a later slot. | 2026-10-22: replaced by the pattern test (Shivam)</t>
         </is>
       </c>
       <c r="AO21" s="69" t="inlineStr">
@@ -3662,7 +3702,7 @@
       </c>
       <c r="H22" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I22" s="69" t="n">
@@ -3723,7 +3763,11 @@
         <f>IF(N(AC22)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC22&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC22&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN22" s="69" t="n"/>
+      <c r="AN22" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO22" s="69" t="inlineStr">
         <is>
           <t>crayon</t>
@@ -3775,7 +3819,7 @@
       </c>
       <c r="H23" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I23" s="69" t="n">
@@ -3850,7 +3894,7 @@
       </c>
       <c r="AN23" s="69" t="inlineStr">
         <is>
-          <t>Story Short (2026-10-17). Headline font Baloo 2 instead of Fredoka (Fredoka has no 800 weight, which the build requests). Held from posting until 2026-11-01.</t>
+          <t>Story Short (2026-10-17). Headline font Baloo 2 instead of Fredoka (Fredoka has no 800 weight, which the build requests). Held from posting until 2026-11-01. | 2026-10-22: replaced by the pattern test (Shivam)</t>
         </is>
       </c>
       <c r="AO23" s="69" t="inlineStr">
@@ -3928,7 +3972,7 @@
       </c>
       <c r="H24" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I24" s="69" t="n">
@@ -3989,7 +4033,11 @@
         <f>IF(N(AC24)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC24&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC24&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN24" s="69" t="n"/>
+      <c r="AN24" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO24" s="69" t="inlineStr">
         <is>
           <t>riso</t>
@@ -4041,7 +4089,7 @@
       </c>
       <c r="H25" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I25" s="69" t="n">
@@ -4102,7 +4150,11 @@
         <f>IF(N(AC25)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC25&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC25&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN25" s="69" t="n"/>
+      <c r="AN25" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO25" s="69" t="inlineStr">
         <is>
           <t>blueprint</t>
@@ -4154,7 +4206,7 @@
       </c>
       <c r="H26" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I26" s="69" t="n">
@@ -4229,7 +4281,7 @@
       </c>
       <c r="AN26" s="69" t="inlineStr">
         <is>
-          <t>Story format demo (2026-10-16). Held from posting until 2026-11-01.</t>
+          <t>Story format demo (2026-10-16). Held from posting until 2026-11-01. | 2026-10-22: replaced by the pattern test (Shivam)</t>
         </is>
       </c>
       <c r="AO26" s="69" t="inlineStr">
@@ -4448,7 +4500,7 @@
       </c>
       <c r="H28" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I28" s="69" t="n">
@@ -4521,7 +4573,11 @@
         <f>IF(N(AC28)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC28&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC28&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN28" s="69" t="n"/>
+      <c r="AN28" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO28" s="69" t="inlineStr">
         <is>
           <t>spy-noir</t>
@@ -4871,7 +4927,7 @@
       </c>
       <c r="H31" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I31" s="69" t="n">
@@ -4932,7 +4988,11 @@
         <f>IF(N(AC31)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC31&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC31&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN31" s="69" t="n"/>
+      <c r="AN31" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO31" s="69" t="inlineStr">
         <is>
           <t>one-line</t>
@@ -4984,7 +5044,7 @@
       </c>
       <c r="H32" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I32" s="69" t="n">
@@ -5045,7 +5105,11 @@
         <f>IF(N(AC32)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC32&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC32&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN32" s="69" t="n"/>
+      <c r="AN32" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO32" s="69" t="inlineStr">
         <is>
           <t>swiss</t>
@@ -5363,7 +5427,7 @@
       </c>
       <c r="H35" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I35" s="69" t="n">
@@ -5424,7 +5488,11 @@
         <f>IF(N(AC35)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC35&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC35&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN35" s="69" t="n"/>
+      <c r="AN35" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO35" s="69" t="inlineStr">
         <is>
           <t>terminal</t>
@@ -5476,7 +5544,7 @@
       </c>
       <c r="H36" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I36" s="69" t="n">
@@ -5537,7 +5605,11 @@
         <f>IF(N(AC36)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC36&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC36&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN36" s="69" t="n"/>
+      <c r="AN36" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO36" s="69" t="inlineStr">
         <is>
           <t>blueprint</t>
@@ -5726,7 +5798,7 @@
       </c>
       <c r="H38" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I38" s="69" t="n">
@@ -5787,7 +5859,11 @@
         <f>IF(N(AC38)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC38&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC38&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN38" s="69" t="n"/>
+      <c r="AN38" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO38" s="69" t="inlineStr">
         <is>
           <t>pixel-quest</t>
@@ -5839,7 +5915,7 @@
       </c>
       <c r="H39" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I39" s="69" t="n">
@@ -5900,7 +5976,11 @@
         <f>IF(N(AC39)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC39&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC39&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN39" s="69" t="n"/>
+      <c r="AN39" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO39" s="69" t="inlineStr">
         <is>
           <t>blueprint</t>
@@ -6351,7 +6431,7 @@
       </c>
       <c r="H43" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I43" s="69" t="n">
@@ -6412,7 +6492,11 @@
         <f>IF(N(AC43)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC43&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC43&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN43" s="69" t="n"/>
+      <c r="AN43" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO43" s="69" t="inlineStr">
         <is>
           <t>swiss</t>
@@ -6464,7 +6548,7 @@
       </c>
       <c r="H44" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I44" s="69" t="n">
@@ -6525,7 +6609,11 @@
         <f>IF(N(AC44)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC44&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC44&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN44" s="69" t="n"/>
+      <c r="AN44" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO44" s="69" t="inlineStr">
         <is>
           <t>cartoon-50s</t>
@@ -6577,7 +6665,7 @@
       </c>
       <c r="H45" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I45" s="69" t="n">
@@ -6638,7 +6726,11 @@
         <f>IF(N(AC45)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC45&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC45&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN45" s="69" t="n"/>
+      <c r="AN45" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO45" s="69" t="inlineStr">
         <is>
           <t>data-story</t>
@@ -6690,7 +6782,7 @@
       </c>
       <c r="H46" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I46" s="69" t="n">
@@ -6751,7 +6843,11 @@
         <f>IF(N(AC46)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC46&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC46&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN46" s="69" t="n"/>
+      <c r="AN46" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO46" s="69" t="inlineStr">
         <is>
           <t>crayon</t>
@@ -7073,7 +7169,7 @@
       </c>
       <c r="H49" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I49" s="69" t="n">
@@ -7134,7 +7230,11 @@
         <f>IF(N(AC49)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC49&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC49&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN49" s="69" t="n"/>
+      <c r="AN49" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO49" s="69" t="inlineStr">
         <is>
           <t>crayon</t>
@@ -7186,7 +7286,7 @@
       </c>
       <c r="H50" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I50" s="69" t="n">
@@ -7247,7 +7347,11 @@
         <f>IF(N(AC50)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC50&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC50&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN50" s="69" t="n"/>
+      <c r="AN50" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO50" s="69" t="inlineStr">
         <is>
           <t>one-line</t>
@@ -7299,7 +7403,7 @@
       </c>
       <c r="H51" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I51" s="69" t="n">
@@ -7360,7 +7464,11 @@
         <f>IF(N(AC51)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC51&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC51&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN51" s="69" t="n"/>
+      <c r="AN51" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO51" s="69" t="inlineStr">
         <is>
           <t>whiteboard</t>
@@ -7545,7 +7653,7 @@
       </c>
       <c r="H53" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I53" s="69" t="n">
@@ -7606,7 +7714,11 @@
         <f>IF(N(AC53)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC53&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC53&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN53" s="69" t="n"/>
+      <c r="AN53" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO53" s="69" t="inlineStr">
         <is>
           <t>crayon</t>
@@ -7658,7 +7770,7 @@
       </c>
       <c r="H54" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I54" s="69" t="n">
@@ -7719,7 +7831,11 @@
         <f>IF(N(AC54)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC54&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC54&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN54" s="69" t="n"/>
+      <c r="AN54" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO54" s="69" t="inlineStr">
         <is>
           <t>cartoon-50s</t>
@@ -7771,7 +7887,7 @@
       </c>
       <c r="H55" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I55" s="69" t="n">
@@ -7832,7 +7948,11 @@
         <f>IF(N(AC55)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC55&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC55&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN55" s="69" t="n"/>
+      <c r="AN55" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO55" s="69" t="inlineStr">
         <is>
           <t>keynote</t>
@@ -7884,7 +8004,7 @@
       </c>
       <c r="H56" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I56" s="69" t="n">
@@ -7945,7 +8065,11 @@
         <f>IF(N(AC56)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC56&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC56&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN56" s="69" t="n"/>
+      <c r="AN56" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO56" s="69" t="inlineStr">
         <is>
           <t>cartoon-50s</t>
@@ -7997,7 +8121,7 @@
       </c>
       <c r="H57" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I57" s="69" t="n">
@@ -8058,7 +8182,11 @@
         <f>IF(N(AC57)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC57&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC57&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN57" s="69" t="n"/>
+      <c r="AN57" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO57" s="69" t="inlineStr">
         <is>
           <t>one-line</t>
@@ -8110,7 +8238,7 @@
       </c>
       <c r="H58" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I58" s="69" t="n">
@@ -8171,7 +8299,11 @@
         <f>IF(N(AC58)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC58&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC58&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN58" s="69" t="n"/>
+      <c r="AN58" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO58" s="69" t="inlineStr">
         <is>
           <t>spy-noir</t>
@@ -8223,7 +8355,7 @@
       </c>
       <c r="H59" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I59" s="69" t="n">
@@ -8284,7 +8416,11 @@
         <f>IF(N(AC59)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC59&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC59&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN59" s="69" t="n"/>
+      <c r="AN59" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO59" s="69" t="inlineStr">
         <is>
           <t>cartoon-50s</t>
@@ -8336,7 +8472,7 @@
       </c>
       <c r="H60" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I60" s="69" t="n">
@@ -8397,7 +8533,11 @@
         <f>IF(N(AC60)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC60&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC60&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN60" s="69" t="n"/>
+      <c r="AN60" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO60" s="69" t="inlineStr">
         <is>
           <t>swiss</t>
@@ -8449,7 +8589,7 @@
       </c>
       <c r="H61" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I61" s="69" t="n">
@@ -8510,7 +8650,11 @@
         <f>IF(N(AC61)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC61&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC61&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN61" s="69" t="n"/>
+      <c r="AN61" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO61" s="69" t="inlineStr">
         <is>
           <t>crayon</t>
@@ -8562,7 +8706,7 @@
       </c>
       <c r="H62" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I62" s="69" t="n">
@@ -8623,7 +8767,11 @@
         <f>IF(N(AC62)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC62&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC62&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN62" s="69" t="n"/>
+      <c r="AN62" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO62" s="69" t="inlineStr">
         <is>
           <t>dossier</t>
@@ -8945,7 +9093,7 @@
       </c>
       <c r="H65" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I65" s="69" t="n">
@@ -9006,7 +9154,11 @@
         <f>IF(N(AC65)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC65&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC65&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN65" s="69" t="n"/>
+      <c r="AN65" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO65" s="69" t="inlineStr">
         <is>
           <t>terminal</t>
@@ -9727,7 +9879,7 @@
       </c>
       <c r="H71" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I71" s="69" t="n">
@@ -9802,7 +9954,7 @@
       </c>
       <c r="AN71" s="69" t="inlineStr">
         <is>
-          <t>Story Short (2026-10-17). Held from posting until 2026-11-01.</t>
+          <t>Story Short (2026-10-17). Held from posting until 2026-11-01. | 2026-10-22: replaced by the pattern test (Shivam)</t>
         </is>
       </c>
       <c r="AO71" s="69" t="inlineStr">
@@ -9880,7 +10032,7 @@
       </c>
       <c r="H72" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I72" s="69" t="n">
@@ -9941,7 +10093,11 @@
         <f>IF(N(AC72)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC72&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC72&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN72" s="69" t="n"/>
+      <c r="AN72" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO72" s="69" t="inlineStr">
         <is>
           <t>game-show</t>
@@ -9993,7 +10149,7 @@
       </c>
       <c r="H73" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I73" s="69" t="n">
@@ -10054,7 +10210,11 @@
         <f>IF(N(AC73)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC73&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC73&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN73" s="69" t="n"/>
+      <c r="AN73" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO73" s="69" t="inlineStr">
         <is>
           <t>spy-noir</t>
@@ -10106,7 +10266,7 @@
       </c>
       <c r="H74" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I74" s="69" t="n">
@@ -10167,7 +10327,11 @@
         <f>IF(N(AC74)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC74&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC74&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN74" s="69" t="n"/>
+      <c r="AN74" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO74" s="69" t="inlineStr">
         <is>
           <t>pixel-quest</t>
@@ -10219,7 +10383,7 @@
       </c>
       <c r="H75" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I75" s="69" t="n">
@@ -10280,7 +10444,11 @@
         <f>IF(N(AC75)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC75&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC75&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN75" s="69" t="n"/>
+      <c r="AN75" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO75" s="69" t="inlineStr">
         <is>
           <t>data-story</t>
@@ -11001,7 +11169,7 @@
       </c>
       <c r="H81" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I81" s="69" t="n">
@@ -11074,7 +11242,11 @@
         <f>IF(N(AC81)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC81&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC81&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN81" s="69" t="n"/>
+      <c r="AN81" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO81" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -11126,7 +11298,7 @@
       </c>
       <c r="H82" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I82" s="69" t="n">
@@ -11187,7 +11359,11 @@
         <f>IF(N(AC82)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC82&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC82&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN82" s="69" t="n"/>
+      <c r="AN82" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO82" s="69" t="inlineStr">
         <is>
           <t>swiss</t>
@@ -11239,7 +11415,7 @@
       </c>
       <c r="H83" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I83" s="69" t="n">
@@ -11300,7 +11476,11 @@
         <f>IF(N(AC83)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC83&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC83&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN83" s="69" t="n"/>
+      <c r="AN83" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO83" s="69" t="inlineStr">
         <is>
           <t>one-line</t>
@@ -11352,7 +11532,7 @@
       </c>
       <c r="H84" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I84" s="69" t="n">
@@ -11413,7 +11593,11 @@
         <f>IF(N(AC84)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC84&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC84&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN84" s="69" t="n"/>
+      <c r="AN84" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO84" s="69" t="inlineStr">
         <is>
           <t>pixel-quest</t>
@@ -11465,7 +11649,7 @@
       </c>
       <c r="H85" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I85" s="69" t="n">
@@ -11526,7 +11710,11 @@
         <f>IF(N(AC85)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC85&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC85&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN85" s="69" t="n"/>
+      <c r="AN85" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO85" s="69" t="inlineStr">
         <is>
           <t>spy-noir</t>
@@ -11578,7 +11766,7 @@
       </c>
       <c r="H86" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I86" s="69" t="n">
@@ -11639,7 +11827,11 @@
         <f>IF(N(AC86)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC86&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC86&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN86" s="69" t="n"/>
+      <c r="AN86" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO86" s="69" t="inlineStr">
         <is>
           <t>terminal</t>
@@ -12227,7 +12419,7 @@
       </c>
       <c r="H91" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I91" s="69" t="n">
@@ -12300,7 +12492,11 @@
         <f>IF(N(AC91)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC91&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC91&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN91" s="69" t="n"/>
+      <c r="AN91" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO91" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -12352,7 +12548,7 @@
       </c>
       <c r="H92" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I92" s="69" t="n">
@@ -12413,7 +12609,11 @@
         <f>IF(N(AC92)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC92&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC92&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN92" s="69" t="n"/>
+      <c r="AN92" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO92" s="69" t="inlineStr">
         <is>
           <t>dossier</t>
@@ -12465,7 +12665,7 @@
       </c>
       <c r="H93" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I93" s="69" t="n">
@@ -12526,7 +12726,11 @@
         <f>IF(N(AC93)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC93&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC93&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN93" s="69" t="n"/>
+      <c r="AN93" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO93" s="69" t="inlineStr">
         <is>
           <t>keynote</t>
@@ -12578,7 +12782,7 @@
       </c>
       <c r="H94" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I94" s="69" t="n">
@@ -12639,7 +12843,11 @@
         <f>IF(N(AC94)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC94&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC94&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN94" s="69" t="n"/>
+      <c r="AN94" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO94" s="69" t="inlineStr">
         <is>
           <t>cartoon-50s</t>
@@ -12691,7 +12899,7 @@
       </c>
       <c r="H95" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I95" s="69" t="n">
@@ -12752,7 +12960,11 @@
         <f>IF(N(AC95)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC95&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC95&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN95" s="69" t="n"/>
+      <c r="AN95" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO95" s="69" t="inlineStr">
         <is>
           <t>crayon</t>
@@ -13344,7 +13556,7 @@
       </c>
       <c r="H100" s="68" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I100" s="69" t="n">
@@ -13417,7 +13629,11 @@
         <f>IF(N(AC100)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC100&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC100&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN100" s="69" t="n"/>
+      <c r="AN100" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO100" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -13469,7 +13685,7 @@
       </c>
       <c r="H101" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I101" s="69" t="n">
@@ -13530,7 +13746,11 @@
         <f>IF(N(AC101)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC101&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC101&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN101" s="69" t="n"/>
+      <c r="AN101" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO101" s="69" t="inlineStr">
         <is>
           <t>one-line</t>
@@ -13582,7 +13802,7 @@
       </c>
       <c r="H102" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I102" s="69" t="n">
@@ -13643,7 +13863,11 @@
         <f>IF(N(AC102)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC102&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC102&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN102" s="69" t="n"/>
+      <c r="AN102" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO102" s="69" t="inlineStr">
         <is>
           <t>data-story</t>
@@ -13695,7 +13919,7 @@
       </c>
       <c r="H103" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I103" s="69" t="n">
@@ -13756,7 +13980,11 @@
         <f>IF(N(AC103)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC103&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC103&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN103" s="69" t="n"/>
+      <c r="AN103" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO103" s="69" t="inlineStr">
         <is>
           <t>data-story</t>
@@ -13808,7 +14036,7 @@
       </c>
       <c r="H104" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I104" s="69" t="n">
@@ -13869,7 +14097,11 @@
         <f>IF(N(AC104)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC104&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC104&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN104" s="69" t="n"/>
+      <c r="AN104" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO104" s="69" t="inlineStr">
         <is>
           <t>dossier</t>
@@ -13921,7 +14153,7 @@
       </c>
       <c r="H105" s="68" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I105" s="69" t="n">
@@ -13982,7 +14214,11 @@
         <f>IF(N(AC105)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC105&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC105&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN105" s="69" t="n"/>
+      <c r="AN105" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-22: replaced by the pattern test (Shivam)</t>
+        </is>
+      </c>
       <c r="AO105" s="69" t="inlineStr">
         <is>
           <t>whiteboard</t>
@@ -14251,6 +14487,3444 @@
       <c r="AV107" s="64" t="inlineStr">
         <is>
           <t>You-callout</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="123" t="n">
+        <v>103</v>
+      </c>
+      <c r="B108" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Experiment story</t>
+        </is>
+      </c>
+      <c r="C108" s="123" t="inlineStr">
+        <is>
+          <t>The experiment that fooled psychiatrists (Rosenhan)</t>
+        </is>
+      </c>
+      <c r="D108" s="123" t="inlineStr">
+        <is>
+          <t>Eight people faked ONE symptom, and every hospital admitted them.</t>
+        </is>
+      </c>
+      <c r="E108" s="123" t="inlineStr">
+        <is>
+          <t>Rosenhan 1973; 12 hospitals, 19 days avg, 35/118 patients suspected; turn: Cahalan 2019 doubts</t>
+        </is>
+      </c>
+      <c r="F108" s="123" t="n"/>
+      <c r="G108" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H108" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I108" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="J108" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K108" s="124" t="inlineStr">
+        <is>
+          <t>rosenhan-fake-patients</t>
+        </is>
+      </c>
+      <c r="L108" s="125" t="n"/>
+      <c r="M108" s="123">
+        <f>IF(L108="","",TEXT(L108,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N108" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="O108" s="124" t="n"/>
+      <c r="P108" s="124" t="n"/>
+      <c r="Q108" s="124" t="inlineStr">
+        <is>
+          <t>Rosenhan (1973, Science): 8 pseudopatients reported hearing a voice say "thud", were admitted to 12 hospitals and held 7 to 52 days (19 on average); 35 of 118 patients suspected them, staff didn't. Journalist Susannah Cahalan (The Great Pretender, 20</t>
+        </is>
+      </c>
+      <c r="R108" s="124" t="n"/>
+      <c r="S108" s="126" t="n"/>
+      <c r="T108" s="124" t="n"/>
+      <c r="U108" s="127">
+        <f>IF(OR(T108="",N(O108)=0),"",T108/O108)</f>
+        <v/>
+      </c>
+      <c r="V108" s="124" t="n"/>
+      <c r="W108" s="124" t="n"/>
+      <c r="X108" s="124" t="n"/>
+      <c r="Y108" s="126" t="n"/>
+      <c r="Z108" s="124" t="n"/>
+      <c r="AA108" s="126" t="n"/>
+      <c r="AB108" s="124" t="n"/>
+      <c r="AC108" s="128">
+        <f>IF(COUNT(S108,Y108,AA108)=0,"",SUM(S108,Y108,AA108))</f>
+        <v/>
+      </c>
+      <c r="AD108" s="127">
+        <f>IF(N(AC108)=0,"",SUM(V108,W108,X108,Z108,AB108)/AC108)</f>
+        <v/>
+      </c>
+      <c r="AE108" s="126" t="n"/>
+      <c r="AF108" s="126" t="n"/>
+      <c r="AG108" s="126" t="n"/>
+      <c r="AH108" s="128">
+        <f>IF(COUNT(AE108,AF108,AG108)=0,"",SUM(AE108,AF108,AG108))</f>
+        <v/>
+      </c>
+      <c r="AI108" s="126" t="n"/>
+      <c r="AJ108" s="126" t="n"/>
+      <c r="AK108" s="126" t="n"/>
+      <c r="AL108" s="128">
+        <f>IF(COUNT(AI108,AJ108,AK108)=0,"",SUM(AI108,AJ108,AK108))</f>
+        <v/>
+      </c>
+      <c r="AM108" s="123">
+        <f>IF(N(AC108)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC108&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC108&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN108" s="124" t="n"/>
+      <c r="AO108" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP108" s="129" t="n"/>
+      <c r="AQ108" s="129" t="n"/>
+      <c r="AR108" s="129" t="n"/>
+      <c r="AS108" s="129" t="n"/>
+      <c r="AT108" s="129" t="n"/>
+      <c r="AU108" s="129" t="n"/>
+      <c r="AV108" s="130" t="inlineStr">
+        <is>
+          <t>Experiment story</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="123" t="n">
+        <v>104</v>
+      </c>
+      <c r="B109" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Protect yourself</t>
+        </is>
+      </c>
+      <c r="C109" s="123" t="inlineStr">
+        <is>
+          <t>The tiny-yes trick (foot in the door)</t>
+        </is>
+      </c>
+      <c r="D109" s="123" t="inlineStr">
+        <is>
+          <t>If someone asks you for something TINY first, watch out.</t>
+        </is>
+      </c>
+      <c r="E109" s="123" t="inlineStr">
+        <is>
+          <t>Freedman &amp; Fraser 1966: 17% vs 76% big sign</t>
+        </is>
+      </c>
+      <c r="F109" s="123" t="n"/>
+      <c r="G109" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H109" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I109" s="124" t="n">
+        <v>2</v>
+      </c>
+      <c r="J109" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K109" s="124" t="inlineStr">
+        <is>
+          <t>foot-in-the-door</t>
+        </is>
+      </c>
+      <c r="L109" s="125" t="n"/>
+      <c r="M109" s="123">
+        <f>IF(L109="","",TEXT(L109,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N109" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="O109" s="124" t="n"/>
+      <c r="P109" s="124" t="n"/>
+      <c r="Q109" s="124" t="inlineStr">
+        <is>
+          <t>Freedman &amp; Fraser (1966): only 17% of homeowners agreed to a big "Drive Carefully" yard sign, but 76% agreed after first saying yes to a small "Be a Safe Driver" window sign. The foot-in-the-door technique.</t>
+        </is>
+      </c>
+      <c r="R109" s="124" t="n"/>
+      <c r="S109" s="126" t="n"/>
+      <c r="T109" s="124" t="n"/>
+      <c r="U109" s="127">
+        <f>IF(OR(T109="",N(O109)=0),"",T109/O109)</f>
+        <v/>
+      </c>
+      <c r="V109" s="124" t="n"/>
+      <c r="W109" s="124" t="n"/>
+      <c r="X109" s="124" t="n"/>
+      <c r="Y109" s="126" t="n"/>
+      <c r="Z109" s="124" t="n"/>
+      <c r="AA109" s="126" t="n"/>
+      <c r="AB109" s="124" t="n"/>
+      <c r="AC109" s="128">
+        <f>IF(COUNT(S109,Y109,AA109)=0,"",SUM(S109,Y109,AA109))</f>
+        <v/>
+      </c>
+      <c r="AD109" s="127">
+        <f>IF(N(AC109)=0,"",SUM(V109,W109,X109,Z109,AB109)/AC109)</f>
+        <v/>
+      </c>
+      <c r="AE109" s="126" t="n"/>
+      <c r="AF109" s="126" t="n"/>
+      <c r="AG109" s="126" t="n"/>
+      <c r="AH109" s="128">
+        <f>IF(COUNT(AE109,AF109,AG109)=0,"",SUM(AE109,AF109,AG109))</f>
+        <v/>
+      </c>
+      <c r="AI109" s="126" t="n"/>
+      <c r="AJ109" s="126" t="n"/>
+      <c r="AK109" s="126" t="n"/>
+      <c r="AL109" s="128">
+        <f>IF(COUNT(AI109,AJ109,AK109)=0,"",SUM(AI109,AJ109,AK109))</f>
+        <v/>
+      </c>
+      <c r="AM109" s="123">
+        <f>IF(N(AC109)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC109&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC109&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN109" s="124" t="n"/>
+      <c r="AO109" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP109" s="129" t="n"/>
+      <c r="AQ109" s="129" t="n"/>
+      <c r="AR109" s="129" t="n"/>
+      <c r="AS109" s="129" t="n"/>
+      <c r="AT109" s="129" t="n"/>
+      <c r="AU109" s="129" t="n"/>
+      <c r="AV109" s="130" t="inlineStr">
+        <is>
+          <t>Protect yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="123" t="n">
+        <v>105</v>
+      </c>
+      <c r="B110" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Psychology of people who</t>
+        </is>
+      </c>
+      <c r="C110" s="123" t="inlineStr">
+        <is>
+          <t>Psychology of people who are always late (planning fallacy)</t>
+        </is>
+      </c>
+      <c r="D110" s="123" t="inlineStr">
+        <is>
+          <t>Psychology of people who are ALWAYS late: it's usually not laziness.</t>
+        </is>
+      </c>
+      <c r="E110" s="123" t="inlineStr">
+        <is>
+          <t>Buehler, Griffin &amp; Ross 1994: 33.9 / 48.6 / 55.5 days, ~30% on time</t>
+        </is>
+      </c>
+      <c r="F110" s="123" t="n"/>
+      <c r="G110" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H110" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I110" s="124" t="n">
+        <v>3</v>
+      </c>
+      <c r="J110" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K110" s="124" t="inlineStr">
+        <is>
+          <t>always-late</t>
+        </is>
+      </c>
+      <c r="L110" s="125" t="n"/>
+      <c r="M110" s="123">
+        <f>IF(L110="","",TEXT(L110,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N110" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="O110" s="124" t="n"/>
+      <c r="P110" s="124" t="n"/>
+      <c r="Q110" s="124" t="inlineStr">
+        <is>
+          <t>Buehler, Griffin &amp; Ross (1994): students predicted their thesis would take 33.9 days (worst case 48.6); it took 55.5, and only about 30% finished by their own estimate. The planning fallacy. Fix: base plans on how long it took last time.</t>
+        </is>
+      </c>
+      <c r="R110" s="124" t="n"/>
+      <c r="S110" s="126" t="n"/>
+      <c r="T110" s="124" t="n"/>
+      <c r="U110" s="127">
+        <f>IF(OR(T110="",N(O110)=0),"",T110/O110)</f>
+        <v/>
+      </c>
+      <c r="V110" s="124" t="n"/>
+      <c r="W110" s="124" t="n"/>
+      <c r="X110" s="124" t="n"/>
+      <c r="Y110" s="126" t="n"/>
+      <c r="Z110" s="124" t="n"/>
+      <c r="AA110" s="126" t="n"/>
+      <c r="AB110" s="124" t="n"/>
+      <c r="AC110" s="128">
+        <f>IF(COUNT(S110,Y110,AA110)=0,"",SUM(S110,Y110,AA110))</f>
+        <v/>
+      </c>
+      <c r="AD110" s="127">
+        <f>IF(N(AC110)=0,"",SUM(V110,W110,X110,Z110,AB110)/AC110)</f>
+        <v/>
+      </c>
+      <c r="AE110" s="126" t="n"/>
+      <c r="AF110" s="126" t="n"/>
+      <c r="AG110" s="126" t="n"/>
+      <c r="AH110" s="128">
+        <f>IF(COUNT(AE110,AF110,AG110)=0,"",SUM(AE110,AF110,AG110))</f>
+        <v/>
+      </c>
+      <c r="AI110" s="126" t="n"/>
+      <c r="AJ110" s="126" t="n"/>
+      <c r="AK110" s="126" t="n"/>
+      <c r="AL110" s="128">
+        <f>IF(COUNT(AI110,AJ110,AK110)=0,"",SUM(AI110,AJ110,AK110))</f>
+        <v/>
+      </c>
+      <c r="AM110" s="123">
+        <f>IF(N(AC110)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC110&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC110&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN110" s="124" t="n"/>
+      <c r="AO110" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP110" s="129" t="n"/>
+      <c r="AQ110" s="129" t="n"/>
+      <c r="AR110" s="129" t="n"/>
+      <c r="AS110" s="129" t="n"/>
+      <c r="AT110" s="129" t="n"/>
+      <c r="AU110" s="129" t="n"/>
+      <c r="AV110" s="130" t="inlineStr">
+        <is>
+          <t>Psychology of people who</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="123" t="n">
+        <v>106</v>
+      </c>
+      <c r="B111" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Numbered facts</t>
+        </is>
+      </c>
+      <c r="C111" s="123" t="inlineStr">
+        <is>
+          <t>3 reasons your mind goes blank</t>
+        </is>
+      </c>
+      <c r="D111" s="123" t="inlineStr">
+        <is>
+          <t>Three reasons your mind goes BLANK.</t>
+        </is>
+      </c>
+      <c r="E111" s="123" t="inlineStr">
+        <is>
+          <t>Radvansky 2011 doorway; Brenner 1973 next-in-line; Sparrow 2011 Google effect</t>
+        </is>
+      </c>
+      <c r="F111" s="123" t="n"/>
+      <c r="G111" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H111" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I111" s="124" t="n">
+        <v>4</v>
+      </c>
+      <c r="J111" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K111" s="124" t="inlineStr">
+        <is>
+          <t>mind-goes-blank</t>
+        </is>
+      </c>
+      <c r="L111" s="125" t="n"/>
+      <c r="M111" s="123">
+        <f>IF(L111="","",TEXT(L111,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N111" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="O111" s="124" t="n"/>
+      <c r="P111" s="124" t="n"/>
+      <c r="Q111" s="124" t="inlineStr">
+        <is>
+          <t>1) Radvansky et al. (2011): walking through a doorway causes more forgetting than the same distance within a room (an event boundary). 2) Brenner (1973), the next-in-line effect: people recall least of what was said just before their own turn. 3) Spa</t>
+        </is>
+      </c>
+      <c r="R111" s="124" t="n"/>
+      <c r="S111" s="126" t="n"/>
+      <c r="T111" s="124" t="n"/>
+      <c r="U111" s="127">
+        <f>IF(OR(T111="",N(O111)=0),"",T111/O111)</f>
+        <v/>
+      </c>
+      <c r="V111" s="124" t="n"/>
+      <c r="W111" s="124" t="n"/>
+      <c r="X111" s="124" t="n"/>
+      <c r="Y111" s="126" t="n"/>
+      <c r="Z111" s="124" t="n"/>
+      <c r="AA111" s="126" t="n"/>
+      <c r="AB111" s="124" t="n"/>
+      <c r="AC111" s="128">
+        <f>IF(COUNT(S111,Y111,AA111)=0,"",SUM(S111,Y111,AA111))</f>
+        <v/>
+      </c>
+      <c r="AD111" s="127">
+        <f>IF(N(AC111)=0,"",SUM(V111,W111,X111,Z111,AB111)/AC111)</f>
+        <v/>
+      </c>
+      <c r="AE111" s="126" t="n"/>
+      <c r="AF111" s="126" t="n"/>
+      <c r="AG111" s="126" t="n"/>
+      <c r="AH111" s="128">
+        <f>IF(COUNT(AE111,AF111,AG111)=0,"",SUM(AE111,AF111,AG111))</f>
+        <v/>
+      </c>
+      <c r="AI111" s="126" t="n"/>
+      <c r="AJ111" s="126" t="n"/>
+      <c r="AK111" s="126" t="n"/>
+      <c r="AL111" s="128">
+        <f>IF(COUNT(AI111,AJ111,AK111)=0,"",SUM(AI111,AJ111,AK111))</f>
+        <v/>
+      </c>
+      <c r="AM111" s="123">
+        <f>IF(N(AC111)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC111&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC111&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN111" s="124" t="n"/>
+      <c r="AO111" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP111" s="129" t="n"/>
+      <c r="AQ111" s="129" t="n"/>
+      <c r="AR111" s="129" t="n"/>
+      <c r="AS111" s="129" t="n"/>
+      <c r="AT111" s="129" t="n"/>
+      <c r="AU111" s="129" t="n"/>
+      <c r="AV111" s="130" t="inlineStr">
+        <is>
+          <t>Numbered facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="123" t="n">
+        <v>107</v>
+      </c>
+      <c r="B112" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Therapist tip</t>
+        </is>
+      </c>
+      <c r="C112" s="123" t="inlineStr">
+        <is>
+          <t>The 5-minute breath that beat mindfulness (cyclic sighing)</t>
+        </is>
+      </c>
+      <c r="D112" s="123" t="inlineStr">
+        <is>
+          <t>This five-minute breath lifted mood MORE than mindfulness.</t>
+        </is>
+      </c>
+      <c r="E112" s="123" t="inlineStr">
+        <is>
+          <t>Balban et al. 2023 Cell Reports Medicine</t>
+        </is>
+      </c>
+      <c r="F112" s="123" t="n"/>
+      <c r="G112" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H112" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I112" s="124" t="n">
+        <v>5</v>
+      </c>
+      <c r="J112" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K112" s="124" t="inlineStr">
+        <is>
+          <t>five-minute-sigh</t>
+        </is>
+      </c>
+      <c r="L112" s="125" t="n"/>
+      <c r="M112" s="123">
+        <f>IF(L112="","",TEXT(L112,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N112" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="O112" s="124" t="n"/>
+      <c r="P112" s="124" t="n"/>
+      <c r="Q112" s="124" t="inlineStr">
+        <is>
+          <t>Balban et al. (2023, Cell Reports Medicine, Stanford): 5 minutes a day of cyclic sighing (inhale, second short inhale, long exhale) for a month raised daily positive mood more than mindfulness meditation; both reduced anxiety. Not medical advice.</t>
+        </is>
+      </c>
+      <c r="R112" s="124" t="n"/>
+      <c r="S112" s="126" t="n"/>
+      <c r="T112" s="124" t="n"/>
+      <c r="U112" s="127">
+        <f>IF(OR(T112="",N(O112)=0),"",T112/O112)</f>
+        <v/>
+      </c>
+      <c r="V112" s="124" t="n"/>
+      <c r="W112" s="124" t="n"/>
+      <c r="X112" s="124" t="n"/>
+      <c r="Y112" s="126" t="n"/>
+      <c r="Z112" s="124" t="n"/>
+      <c r="AA112" s="126" t="n"/>
+      <c r="AB112" s="124" t="n"/>
+      <c r="AC112" s="128">
+        <f>IF(COUNT(S112,Y112,AA112)=0,"",SUM(S112,Y112,AA112))</f>
+        <v/>
+      </c>
+      <c r="AD112" s="127">
+        <f>IF(N(AC112)=0,"",SUM(V112,W112,X112,Z112,AB112)/AC112)</f>
+        <v/>
+      </c>
+      <c r="AE112" s="126" t="n"/>
+      <c r="AF112" s="126" t="n"/>
+      <c r="AG112" s="126" t="n"/>
+      <c r="AH112" s="128">
+        <f>IF(COUNT(AE112,AF112,AG112)=0,"",SUM(AE112,AF112,AG112))</f>
+        <v/>
+      </c>
+      <c r="AI112" s="126" t="n"/>
+      <c r="AJ112" s="126" t="n"/>
+      <c r="AK112" s="126" t="n"/>
+      <c r="AL112" s="128">
+        <f>IF(COUNT(AI112,AJ112,AK112)=0,"",SUM(AI112,AJ112,AK112))</f>
+        <v/>
+      </c>
+      <c r="AM112" s="123">
+        <f>IF(N(AC112)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC112&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC112&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN112" s="124" t="n"/>
+      <c r="AO112" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP112" s="129" t="n"/>
+      <c r="AQ112" s="129" t="n"/>
+      <c r="AR112" s="129" t="n"/>
+      <c r="AS112" s="129" t="n"/>
+      <c r="AT112" s="129" t="n"/>
+      <c r="AU112" s="129" t="n"/>
+      <c r="AV112" s="130" t="inlineStr">
+        <is>
+          <t>Therapist tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="123" t="n">
+        <v>108</v>
+      </c>
+      <c r="B113" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Relationships &amp; likability</t>
+        </is>
+      </c>
+      <c r="C113" s="123" t="inlineStr">
+        <is>
+          <t>Why small mistakes make you likable (pratfall effect)</t>
+        </is>
+      </c>
+      <c r="D113" s="123" t="inlineStr">
+        <is>
+          <t>The most likable person might be the one who SPILLS their coffee.</t>
+        </is>
+      </c>
+      <c r="E113" s="123" t="inlineStr">
+        <is>
+          <t>Aronson, Willerman &amp; Floyd 1966: 92% contestant</t>
+        </is>
+      </c>
+      <c r="F113" s="123" t="n"/>
+      <c r="G113" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H113" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I113" s="124" t="n">
+        <v>6</v>
+      </c>
+      <c r="J113" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K113" s="124" t="inlineStr">
+        <is>
+          <t>coffee-spill-effect</t>
+        </is>
+      </c>
+      <c r="L113" s="125" t="n"/>
+      <c r="M113" s="123">
+        <f>IF(L113="","",TEXT(L113,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N113" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="O113" s="124" t="n"/>
+      <c r="P113" s="124" t="n"/>
+      <c r="Q113" s="124" t="inlineStr">
+        <is>
+          <t>Aronson, Willerman &amp; Floyd (1966): students heard a taped quiz contestant who answered 92% of questions right; when he spilled coffee on himself he was rated more likable. An average contestant who spilled was rated less likable. The pratfall effect.</t>
+        </is>
+      </c>
+      <c r="R113" s="124" t="n"/>
+      <c r="S113" s="126" t="n"/>
+      <c r="T113" s="124" t="n"/>
+      <c r="U113" s="127">
+        <f>IF(OR(T113="",N(O113)=0),"",T113/O113)</f>
+        <v/>
+      </c>
+      <c r="V113" s="124" t="n"/>
+      <c r="W113" s="124" t="n"/>
+      <c r="X113" s="124" t="n"/>
+      <c r="Y113" s="126" t="n"/>
+      <c r="Z113" s="124" t="n"/>
+      <c r="AA113" s="126" t="n"/>
+      <c r="AB113" s="124" t="n"/>
+      <c r="AC113" s="128">
+        <f>IF(COUNT(S113,Y113,AA113)=0,"",SUM(S113,Y113,AA113))</f>
+        <v/>
+      </c>
+      <c r="AD113" s="127">
+        <f>IF(N(AC113)=0,"",SUM(V113,W113,X113,Z113,AB113)/AC113)</f>
+        <v/>
+      </c>
+      <c r="AE113" s="126" t="n"/>
+      <c r="AF113" s="126" t="n"/>
+      <c r="AG113" s="126" t="n"/>
+      <c r="AH113" s="128">
+        <f>IF(COUNT(AE113,AF113,AG113)=0,"",SUM(AE113,AF113,AG113))</f>
+        <v/>
+      </c>
+      <c r="AI113" s="126" t="n"/>
+      <c r="AJ113" s="126" t="n"/>
+      <c r="AK113" s="126" t="n"/>
+      <c r="AL113" s="128">
+        <f>IF(COUNT(AI113,AJ113,AK113)=0,"",SUM(AI113,AJ113,AK113))</f>
+        <v/>
+      </c>
+      <c r="AM113" s="123">
+        <f>IF(N(AC113)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC113&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC113&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN113" s="124" t="n"/>
+      <c r="AO113" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP113" s="129" t="n"/>
+      <c r="AQ113" s="129" t="n"/>
+      <c r="AR113" s="129" t="n"/>
+      <c r="AS113" s="129" t="n"/>
+      <c r="AT113" s="129" t="n"/>
+      <c r="AU113" s="129" t="n"/>
+      <c r="AV113" s="130" t="inlineStr">
+        <is>
+          <t>Relationships &amp; likability</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="123" t="n">
+        <v>109</v>
+      </c>
+      <c r="B114" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Strange named effect</t>
+        </is>
+      </c>
+      <c r="C114" s="123" t="inlineStr">
+        <is>
+          <t>The Tetris effect: your brain replays what you repeat</t>
+        </is>
+      </c>
+      <c r="D114" s="123" t="inlineStr">
+        <is>
+          <t>Play a game for hours and your brain plays it while you SLEEP.</t>
+        </is>
+      </c>
+      <c r="E114" s="123" t="inlineStr">
+        <is>
+          <t>Stickgold et al. 2000 Science: Tetris imagery at sleep onset, even in amnesic patients</t>
+        </is>
+      </c>
+      <c r="F114" s="123" t="n"/>
+      <c r="G114" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H114" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I114" s="124" t="n">
+        <v>7</v>
+      </c>
+      <c r="J114" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K114" s="124" t="inlineStr">
+        <is>
+          <t>tetris-effect</t>
+        </is>
+      </c>
+      <c r="L114" s="125" t="n"/>
+      <c r="M114" s="123">
+        <f>IF(L114="","",TEXT(L114,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N114" s="124" t="n"/>
+      <c r="O114" s="124" t="n"/>
+      <c r="P114" s="124" t="n"/>
+      <c r="Q114" s="124" t="n"/>
+      <c r="R114" s="124" t="n"/>
+      <c r="S114" s="126" t="n"/>
+      <c r="T114" s="124" t="n"/>
+      <c r="U114" s="127">
+        <f>IF(OR(T114="",N(O114)=0),"",T114/O114)</f>
+        <v/>
+      </c>
+      <c r="V114" s="124" t="n"/>
+      <c r="W114" s="124" t="n"/>
+      <c r="X114" s="124" t="n"/>
+      <c r="Y114" s="126" t="n"/>
+      <c r="Z114" s="124" t="n"/>
+      <c r="AA114" s="126" t="n"/>
+      <c r="AB114" s="124" t="n"/>
+      <c r="AC114" s="128">
+        <f>IF(COUNT(S114,Y114,AA114)=0,"",SUM(S114,Y114,AA114))</f>
+        <v/>
+      </c>
+      <c r="AD114" s="127">
+        <f>IF(N(AC114)=0,"",SUM(V114,W114,X114,Z114,AB114)/AC114)</f>
+        <v/>
+      </c>
+      <c r="AE114" s="126" t="n"/>
+      <c r="AF114" s="126" t="n"/>
+      <c r="AG114" s="126" t="n"/>
+      <c r="AH114" s="128">
+        <f>IF(COUNT(AE114,AF114,AG114)=0,"",SUM(AE114,AF114,AG114))</f>
+        <v/>
+      </c>
+      <c r="AI114" s="126" t="n"/>
+      <c r="AJ114" s="126" t="n"/>
+      <c r="AK114" s="126" t="n"/>
+      <c r="AL114" s="128">
+        <f>IF(COUNT(AI114,AJ114,AK114)=0,"",SUM(AI114,AJ114,AK114))</f>
+        <v/>
+      </c>
+      <c r="AM114" s="123">
+        <f>IF(N(AC114)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC114&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC114&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN114" s="124" t="n"/>
+      <c r="AO114" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP114" s="129" t="n"/>
+      <c r="AQ114" s="129" t="n"/>
+      <c r="AR114" s="129" t="n"/>
+      <c r="AS114" s="129" t="n"/>
+      <c r="AT114" s="129" t="n"/>
+      <c r="AU114" s="129" t="n"/>
+      <c r="AV114" s="130" t="inlineStr">
+        <is>
+          <t>Strange named effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="123" t="n">
+        <v>110</v>
+      </c>
+      <c r="B115" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Quiz / test yourself</t>
+        </is>
+      </c>
+      <c r="C115" s="123" t="inlineStr">
+        <is>
+          <t>Can you solve the bat-and-ball question? (CRT)</t>
+        </is>
+      </c>
+      <c r="D115" s="123" t="inlineStr">
+        <is>
+          <t>A bat and a ball cost $1.10. Most Ivy League students got this WRONG.</t>
+        </is>
+      </c>
+      <c r="E115" s="123" t="inlineStr">
+        <is>
+          <t>Frederick 2005 Cognitive Reflection Test</t>
+        </is>
+      </c>
+      <c r="F115" s="123" t="n"/>
+      <c r="G115" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H115" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I115" s="124" t="n">
+        <v>8</v>
+      </c>
+      <c r="J115" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K115" s="124" t="inlineStr">
+        <is>
+          <t>bat-and-ball</t>
+        </is>
+      </c>
+      <c r="L115" s="125" t="n"/>
+      <c r="M115" s="123">
+        <f>IF(L115="","",TEXT(L115,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N115" s="124" t="n"/>
+      <c r="O115" s="124" t="n"/>
+      <c r="P115" s="124" t="n"/>
+      <c r="Q115" s="124" t="n"/>
+      <c r="R115" s="124" t="n"/>
+      <c r="S115" s="126" t="n"/>
+      <c r="T115" s="124" t="n"/>
+      <c r="U115" s="127">
+        <f>IF(OR(T115="",N(O115)=0),"",T115/O115)</f>
+        <v/>
+      </c>
+      <c r="V115" s="124" t="n"/>
+      <c r="W115" s="124" t="n"/>
+      <c r="X115" s="124" t="n"/>
+      <c r="Y115" s="126" t="n"/>
+      <c r="Z115" s="124" t="n"/>
+      <c r="AA115" s="126" t="n"/>
+      <c r="AB115" s="124" t="n"/>
+      <c r="AC115" s="128">
+        <f>IF(COUNT(S115,Y115,AA115)=0,"",SUM(S115,Y115,AA115))</f>
+        <v/>
+      </c>
+      <c r="AD115" s="127">
+        <f>IF(N(AC115)=0,"",SUM(V115,W115,X115,Z115,AB115)/AC115)</f>
+        <v/>
+      </c>
+      <c r="AE115" s="126" t="n"/>
+      <c r="AF115" s="126" t="n"/>
+      <c r="AG115" s="126" t="n"/>
+      <c r="AH115" s="128">
+        <f>IF(COUNT(AE115,AF115,AG115)=0,"",SUM(AE115,AF115,AG115))</f>
+        <v/>
+      </c>
+      <c r="AI115" s="126" t="n"/>
+      <c r="AJ115" s="126" t="n"/>
+      <c r="AK115" s="126" t="n"/>
+      <c r="AL115" s="128">
+        <f>IF(COUNT(AI115,AJ115,AK115)=0,"",SUM(AI115,AJ115,AK115))</f>
+        <v/>
+      </c>
+      <c r="AM115" s="123">
+        <f>IF(N(AC115)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC115&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC115&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN115" s="124" t="n"/>
+      <c r="AO115" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP115" s="129" t="n"/>
+      <c r="AQ115" s="129" t="n"/>
+      <c r="AR115" s="129" t="n"/>
+      <c r="AS115" s="129" t="n"/>
+      <c r="AT115" s="129" t="n"/>
+      <c r="AU115" s="129" t="n"/>
+      <c r="AV115" s="130" t="inlineStr">
+        <is>
+          <t>Quiz / test yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="123" t="n">
+        <v>111</v>
+      </c>
+      <c r="B116" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Presence &amp; influence rules</t>
+        </is>
+      </c>
+      <c r="C116" s="123" t="inlineStr">
+        <is>
+          <t>Repeat their words, get bigger tips (mirroring)</t>
+        </is>
+      </c>
+      <c r="D116" s="123" t="inlineStr">
+        <is>
+          <t>Waiters who did ONE thing got much bigger tips.</t>
+        </is>
+      </c>
+      <c r="E116" s="123" t="inlineStr">
+        <is>
+          <t>van Baaren et al. 2003: repeating orders verbatim raised tips</t>
+        </is>
+      </c>
+      <c r="F116" s="123" t="n"/>
+      <c r="G116" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H116" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I116" s="124" t="n">
+        <v>9</v>
+      </c>
+      <c r="J116" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K116" s="124" t="inlineStr">
+        <is>
+          <t>mirroring-tips</t>
+        </is>
+      </c>
+      <c r="L116" s="125" t="n"/>
+      <c r="M116" s="123">
+        <f>IF(L116="","",TEXT(L116,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N116" s="124" t="n"/>
+      <c r="O116" s="124" t="n"/>
+      <c r="P116" s="124" t="n"/>
+      <c r="Q116" s="124" t="n"/>
+      <c r="R116" s="124" t="n"/>
+      <c r="S116" s="126" t="n"/>
+      <c r="T116" s="124" t="n"/>
+      <c r="U116" s="127">
+        <f>IF(OR(T116="",N(O116)=0),"",T116/O116)</f>
+        <v/>
+      </c>
+      <c r="V116" s="124" t="n"/>
+      <c r="W116" s="124" t="n"/>
+      <c r="X116" s="124" t="n"/>
+      <c r="Y116" s="126" t="n"/>
+      <c r="Z116" s="124" t="n"/>
+      <c r="AA116" s="126" t="n"/>
+      <c r="AB116" s="124" t="n"/>
+      <c r="AC116" s="128">
+        <f>IF(COUNT(S116,Y116,AA116)=0,"",SUM(S116,Y116,AA116))</f>
+        <v/>
+      </c>
+      <c r="AD116" s="127">
+        <f>IF(N(AC116)=0,"",SUM(V116,W116,X116,Z116,AB116)/AC116)</f>
+        <v/>
+      </c>
+      <c r="AE116" s="126" t="n"/>
+      <c r="AF116" s="126" t="n"/>
+      <c r="AG116" s="126" t="n"/>
+      <c r="AH116" s="128">
+        <f>IF(COUNT(AE116,AF116,AG116)=0,"",SUM(AE116,AF116,AG116))</f>
+        <v/>
+      </c>
+      <c r="AI116" s="126" t="n"/>
+      <c r="AJ116" s="126" t="n"/>
+      <c r="AK116" s="126" t="n"/>
+      <c r="AL116" s="128">
+        <f>IF(COUNT(AI116,AJ116,AK116)=0,"",SUM(AI116,AJ116,AK116))</f>
+        <v/>
+      </c>
+      <c r="AM116" s="123">
+        <f>IF(N(AC116)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC116&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC116&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN116" s="124" t="n"/>
+      <c r="AO116" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP116" s="129" t="n"/>
+      <c r="AQ116" s="129" t="n"/>
+      <c r="AR116" s="129" t="n"/>
+      <c r="AS116" s="129" t="n"/>
+      <c r="AT116" s="129" t="n"/>
+      <c r="AU116" s="129" t="n"/>
+      <c r="AV116" s="130" t="inlineStr">
+        <is>
+          <t>Presence &amp; influence rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="123" t="n">
+        <v>112</v>
+      </c>
+      <c r="B117" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Psychology says (15 s loop)</t>
+        </is>
+      </c>
+      <c r="C117" s="123" t="inlineStr">
+        <is>
+          <t>Psychology says: asking a favor makes them like you</t>
+        </is>
+      </c>
+      <c r="D117" s="123" t="inlineStr">
+        <is>
+          <t>Psychology says: want someone to like you? Ask THEM for a favor.</t>
+        </is>
+      </c>
+      <c r="E117" s="123" t="inlineStr">
+        <is>
+          <t>Jecker &amp; Landy 1969; Franklin's book anecdote</t>
+        </is>
+      </c>
+      <c r="F117" s="123" t="n"/>
+      <c r="G117" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H117" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I117" s="124" t="n">
+        <v>10</v>
+      </c>
+      <c r="J117" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K117" s="124" t="inlineStr">
+        <is>
+          <t>ben-franklin-effect</t>
+        </is>
+      </c>
+      <c r="L117" s="125" t="n"/>
+      <c r="M117" s="123">
+        <f>IF(L117="","",TEXT(L117,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N117" s="124" t="n"/>
+      <c r="O117" s="124" t="n"/>
+      <c r="P117" s="124" t="n"/>
+      <c r="Q117" s="124" t="n"/>
+      <c r="R117" s="124" t="n"/>
+      <c r="S117" s="126" t="n"/>
+      <c r="T117" s="124" t="n"/>
+      <c r="U117" s="127">
+        <f>IF(OR(T117="",N(O117)=0),"",T117/O117)</f>
+        <v/>
+      </c>
+      <c r="V117" s="124" t="n"/>
+      <c r="W117" s="124" t="n"/>
+      <c r="X117" s="124" t="n"/>
+      <c r="Y117" s="126" t="n"/>
+      <c r="Z117" s="124" t="n"/>
+      <c r="AA117" s="126" t="n"/>
+      <c r="AB117" s="124" t="n"/>
+      <c r="AC117" s="128">
+        <f>IF(COUNT(S117,Y117,AA117)=0,"",SUM(S117,Y117,AA117))</f>
+        <v/>
+      </c>
+      <c r="AD117" s="127">
+        <f>IF(N(AC117)=0,"",SUM(V117,W117,X117,Z117,AB117)/AC117)</f>
+        <v/>
+      </c>
+      <c r="AE117" s="126" t="n"/>
+      <c r="AF117" s="126" t="n"/>
+      <c r="AG117" s="126" t="n"/>
+      <c r="AH117" s="128">
+        <f>IF(COUNT(AE117,AF117,AG117)=0,"",SUM(AE117,AF117,AG117))</f>
+        <v/>
+      </c>
+      <c r="AI117" s="126" t="n"/>
+      <c r="AJ117" s="126" t="n"/>
+      <c r="AK117" s="126" t="n"/>
+      <c r="AL117" s="128">
+        <f>IF(COUNT(AI117,AJ117,AK117)=0,"",SUM(AI117,AJ117,AK117))</f>
+        <v/>
+      </c>
+      <c r="AM117" s="123">
+        <f>IF(N(AC117)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC117&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC117&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN117" s="124" t="n"/>
+      <c r="AO117" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP117" s="129" t="n"/>
+      <c r="AQ117" s="129" t="n"/>
+      <c r="AR117" s="129" t="n"/>
+      <c r="AS117" s="129" t="n"/>
+      <c r="AT117" s="129" t="n"/>
+      <c r="AU117" s="129" t="n"/>
+      <c r="AV117" s="130" t="inlineStr">
+        <is>
+          <t>Psychology says (15 s loop)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="123" t="n">
+        <v>113</v>
+      </c>
+      <c r="B118" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Experiment story</t>
+        </is>
+      </c>
+      <c r="C118" s="123" t="inlineStr">
+        <is>
+          <t>The Good Samaritan experiment: hurry kills kindness</t>
+        </is>
+      </c>
+      <c r="D118" s="123" t="inlineStr">
+        <is>
+          <t>Seminary students on their way to talk about HELPING walked past a man in need.</t>
+        </is>
+      </c>
+      <c r="E118" s="123" t="inlineStr">
+        <is>
+          <t>Darley &amp; Batson 1973: 63% vs 10% helped by hurry level</t>
+        </is>
+      </c>
+      <c r="F118" s="123" t="n"/>
+      <c r="G118" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H118" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I118" s="124" t="n">
+        <v>11</v>
+      </c>
+      <c r="J118" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K118" s="124" t="inlineStr">
+        <is>
+          <t>good-samaritan-hurry</t>
+        </is>
+      </c>
+      <c r="L118" s="125" t="n"/>
+      <c r="M118" s="123">
+        <f>IF(L118="","",TEXT(L118,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N118" s="124" t="n"/>
+      <c r="O118" s="124" t="n"/>
+      <c r="P118" s="124" t="n"/>
+      <c r="Q118" s="124" t="n"/>
+      <c r="R118" s="124" t="n"/>
+      <c r="S118" s="126" t="n"/>
+      <c r="T118" s="124" t="n"/>
+      <c r="U118" s="127">
+        <f>IF(OR(T118="",N(O118)=0),"",T118/O118)</f>
+        <v/>
+      </c>
+      <c r="V118" s="124" t="n"/>
+      <c r="W118" s="124" t="n"/>
+      <c r="X118" s="124" t="n"/>
+      <c r="Y118" s="126" t="n"/>
+      <c r="Z118" s="124" t="n"/>
+      <c r="AA118" s="126" t="n"/>
+      <c r="AB118" s="124" t="n"/>
+      <c r="AC118" s="128">
+        <f>IF(COUNT(S118,Y118,AA118)=0,"",SUM(S118,Y118,AA118))</f>
+        <v/>
+      </c>
+      <c r="AD118" s="127">
+        <f>IF(N(AC118)=0,"",SUM(V118,W118,X118,Z118,AB118)/AC118)</f>
+        <v/>
+      </c>
+      <c r="AE118" s="126" t="n"/>
+      <c r="AF118" s="126" t="n"/>
+      <c r="AG118" s="126" t="n"/>
+      <c r="AH118" s="128">
+        <f>IF(COUNT(AE118,AF118,AG118)=0,"",SUM(AE118,AF118,AG118))</f>
+        <v/>
+      </c>
+      <c r="AI118" s="126" t="n"/>
+      <c r="AJ118" s="126" t="n"/>
+      <c r="AK118" s="126" t="n"/>
+      <c r="AL118" s="128">
+        <f>IF(COUNT(AI118,AJ118,AK118)=0,"",SUM(AI118,AJ118,AK118))</f>
+        <v/>
+      </c>
+      <c r="AM118" s="123">
+        <f>IF(N(AC118)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC118&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC118&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN118" s="124" t="n"/>
+      <c r="AO118" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP118" s="129" t="n"/>
+      <c r="AQ118" s="129" t="n"/>
+      <c r="AR118" s="129" t="n"/>
+      <c r="AS118" s="129" t="n"/>
+      <c r="AT118" s="129" t="n"/>
+      <c r="AU118" s="129" t="n"/>
+      <c r="AV118" s="130" t="inlineStr">
+        <is>
+          <t>Experiment story</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="123" t="n">
+        <v>114</v>
+      </c>
+      <c r="B119" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Protect yourself</t>
+        </is>
+      </c>
+      <c r="C119" s="123" t="inlineStr">
+        <is>
+          <t>The big-no trick (door in the face)</t>
+        </is>
+      </c>
+      <c r="D119" s="123" t="inlineStr">
+        <is>
+          <t>If someone asks for something HUGE first, the real ask is next.</t>
+        </is>
+      </c>
+      <c r="E119" s="123" t="inlineStr">
+        <is>
+          <t>Cialdini et al. 1975: zoo chaperone 50% vs 17%</t>
+        </is>
+      </c>
+      <c r="F119" s="123" t="n"/>
+      <c r="G119" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H119" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I119" s="124" t="n">
+        <v>12</v>
+      </c>
+      <c r="J119" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K119" s="124" t="inlineStr">
+        <is>
+          <t>door-in-the-face</t>
+        </is>
+      </c>
+      <c r="L119" s="125" t="n"/>
+      <c r="M119" s="123">
+        <f>IF(L119="","",TEXT(L119,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N119" s="124" t="n"/>
+      <c r="O119" s="124" t="n"/>
+      <c r="P119" s="124" t="n"/>
+      <c r="Q119" s="124" t="n"/>
+      <c r="R119" s="124" t="n"/>
+      <c r="S119" s="126" t="n"/>
+      <c r="T119" s="124" t="n"/>
+      <c r="U119" s="127">
+        <f>IF(OR(T119="",N(O119)=0),"",T119/O119)</f>
+        <v/>
+      </c>
+      <c r="V119" s="124" t="n"/>
+      <c r="W119" s="124" t="n"/>
+      <c r="X119" s="124" t="n"/>
+      <c r="Y119" s="126" t="n"/>
+      <c r="Z119" s="124" t="n"/>
+      <c r="AA119" s="126" t="n"/>
+      <c r="AB119" s="124" t="n"/>
+      <c r="AC119" s="128">
+        <f>IF(COUNT(S119,Y119,AA119)=0,"",SUM(S119,Y119,AA119))</f>
+        <v/>
+      </c>
+      <c r="AD119" s="127">
+        <f>IF(N(AC119)=0,"",SUM(V119,W119,X119,Z119,AB119)/AC119)</f>
+        <v/>
+      </c>
+      <c r="AE119" s="126" t="n"/>
+      <c r="AF119" s="126" t="n"/>
+      <c r="AG119" s="126" t="n"/>
+      <c r="AH119" s="128">
+        <f>IF(COUNT(AE119,AF119,AG119)=0,"",SUM(AE119,AF119,AG119))</f>
+        <v/>
+      </c>
+      <c r="AI119" s="126" t="n"/>
+      <c r="AJ119" s="126" t="n"/>
+      <c r="AK119" s="126" t="n"/>
+      <c r="AL119" s="128">
+        <f>IF(COUNT(AI119,AJ119,AK119)=0,"",SUM(AI119,AJ119,AK119))</f>
+        <v/>
+      </c>
+      <c r="AM119" s="123">
+        <f>IF(N(AC119)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC119&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC119&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN119" s="124" t="n"/>
+      <c r="AO119" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP119" s="129" t="n"/>
+      <c r="AQ119" s="129" t="n"/>
+      <c r="AR119" s="129" t="n"/>
+      <c r="AS119" s="129" t="n"/>
+      <c r="AT119" s="129" t="n"/>
+      <c r="AU119" s="129" t="n"/>
+      <c r="AV119" s="130" t="inlineStr">
+        <is>
+          <t>Protect yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="123" t="n">
+        <v>115</v>
+      </c>
+      <c r="B120" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Psychology of people who</t>
+        </is>
+      </c>
+      <c r="C120" s="123" t="inlineStr">
+        <is>
+          <t>Psychology of people who doodle in meetings</t>
+        </is>
+      </c>
+      <c r="D120" s="123" t="inlineStr">
+        <is>
+          <t>Psychology of people who DOODLE: they may remember more.</t>
+        </is>
+      </c>
+      <c r="E120" s="123" t="inlineStr">
+        <is>
+          <t>Andrade 2009: doodlers recalled 29% more</t>
+        </is>
+      </c>
+      <c r="F120" s="123" t="n"/>
+      <c r="G120" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H120" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I120" s="124" t="n">
+        <v>13</v>
+      </c>
+      <c r="J120" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K120" s="124" t="inlineStr">
+        <is>
+          <t>doodlers</t>
+        </is>
+      </c>
+      <c r="L120" s="125" t="n"/>
+      <c r="M120" s="123">
+        <f>IF(L120="","",TEXT(L120,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N120" s="124" t="n"/>
+      <c r="O120" s="124" t="n"/>
+      <c r="P120" s="124" t="n"/>
+      <c r="Q120" s="124" t="n"/>
+      <c r="R120" s="124" t="n"/>
+      <c r="S120" s="126" t="n"/>
+      <c r="T120" s="124" t="n"/>
+      <c r="U120" s="127">
+        <f>IF(OR(T120="",N(O120)=0),"",T120/O120)</f>
+        <v/>
+      </c>
+      <c r="V120" s="124" t="n"/>
+      <c r="W120" s="124" t="n"/>
+      <c r="X120" s="124" t="n"/>
+      <c r="Y120" s="126" t="n"/>
+      <c r="Z120" s="124" t="n"/>
+      <c r="AA120" s="126" t="n"/>
+      <c r="AB120" s="124" t="n"/>
+      <c r="AC120" s="128">
+        <f>IF(COUNT(S120,Y120,AA120)=0,"",SUM(S120,Y120,AA120))</f>
+        <v/>
+      </c>
+      <c r="AD120" s="127">
+        <f>IF(N(AC120)=0,"",SUM(V120,W120,X120,Z120,AB120)/AC120)</f>
+        <v/>
+      </c>
+      <c r="AE120" s="126" t="n"/>
+      <c r="AF120" s="126" t="n"/>
+      <c r="AG120" s="126" t="n"/>
+      <c r="AH120" s="128">
+        <f>IF(COUNT(AE120,AF120,AG120)=0,"",SUM(AE120,AF120,AG120))</f>
+        <v/>
+      </c>
+      <c r="AI120" s="126" t="n"/>
+      <c r="AJ120" s="126" t="n"/>
+      <c r="AK120" s="126" t="n"/>
+      <c r="AL120" s="128">
+        <f>IF(COUNT(AI120,AJ120,AK120)=0,"",SUM(AI120,AJ120,AK120))</f>
+        <v/>
+      </c>
+      <c r="AM120" s="123">
+        <f>IF(N(AC120)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC120&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC120&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN120" s="124" t="n"/>
+      <c r="AO120" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP120" s="129" t="n"/>
+      <c r="AQ120" s="129" t="n"/>
+      <c r="AR120" s="129" t="n"/>
+      <c r="AS120" s="129" t="n"/>
+      <c r="AT120" s="129" t="n"/>
+      <c r="AU120" s="129" t="n"/>
+      <c r="AV120" s="130" t="inlineStr">
+        <is>
+          <t>Psychology of people who</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="123" t="n">
+        <v>116</v>
+      </c>
+      <c r="B121" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Numbered facts</t>
+        </is>
+      </c>
+      <c r="C121" s="123" t="inlineStr">
+        <is>
+          <t>3 facts about first impressions</t>
+        </is>
+      </c>
+      <c r="D121" s="123" t="inlineStr">
+        <is>
+          <t>People judge your face in a TENTH of a second.</t>
+        </is>
+      </c>
+      <c r="E121" s="123" t="inlineStr">
+        <is>
+          <t>Willis &amp; Todorov 2006 (100 ms); Nisbett &amp; Wilson 1977 halo; Dion et al. 1972</t>
+        </is>
+      </c>
+      <c r="F121" s="123" t="n"/>
+      <c r="G121" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H121" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I121" s="124" t="n">
+        <v>14</v>
+      </c>
+      <c r="J121" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K121" s="124" t="inlineStr">
+        <is>
+          <t>first-impressions</t>
+        </is>
+      </c>
+      <c r="L121" s="125" t="n"/>
+      <c r="M121" s="123">
+        <f>IF(L121="","",TEXT(L121,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N121" s="124" t="n"/>
+      <c r="O121" s="124" t="n"/>
+      <c r="P121" s="124" t="n"/>
+      <c r="Q121" s="124" t="n"/>
+      <c r="R121" s="124" t="n"/>
+      <c r="S121" s="126" t="n"/>
+      <c r="T121" s="124" t="n"/>
+      <c r="U121" s="127">
+        <f>IF(OR(T121="",N(O121)=0),"",T121/O121)</f>
+        <v/>
+      </c>
+      <c r="V121" s="124" t="n"/>
+      <c r="W121" s="124" t="n"/>
+      <c r="X121" s="124" t="n"/>
+      <c r="Y121" s="126" t="n"/>
+      <c r="Z121" s="124" t="n"/>
+      <c r="AA121" s="126" t="n"/>
+      <c r="AB121" s="124" t="n"/>
+      <c r="AC121" s="128">
+        <f>IF(COUNT(S121,Y121,AA121)=0,"",SUM(S121,Y121,AA121))</f>
+        <v/>
+      </c>
+      <c r="AD121" s="127">
+        <f>IF(N(AC121)=0,"",SUM(V121,W121,X121,Z121,AB121)/AC121)</f>
+        <v/>
+      </c>
+      <c r="AE121" s="126" t="n"/>
+      <c r="AF121" s="126" t="n"/>
+      <c r="AG121" s="126" t="n"/>
+      <c r="AH121" s="128">
+        <f>IF(COUNT(AE121,AF121,AG121)=0,"",SUM(AE121,AF121,AG121))</f>
+        <v/>
+      </c>
+      <c r="AI121" s="126" t="n"/>
+      <c r="AJ121" s="126" t="n"/>
+      <c r="AK121" s="126" t="n"/>
+      <c r="AL121" s="128">
+        <f>IF(COUNT(AI121,AJ121,AK121)=0,"",SUM(AI121,AJ121,AK121))</f>
+        <v/>
+      </c>
+      <c r="AM121" s="123">
+        <f>IF(N(AC121)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC121&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC121&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN121" s="124" t="n"/>
+      <c r="AO121" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP121" s="129" t="n"/>
+      <c r="AQ121" s="129" t="n"/>
+      <c r="AR121" s="129" t="n"/>
+      <c r="AS121" s="129" t="n"/>
+      <c r="AT121" s="129" t="n"/>
+      <c r="AU121" s="129" t="n"/>
+      <c r="AV121" s="130" t="inlineStr">
+        <is>
+          <t>Numbered facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="123" t="n">
+        <v>117</v>
+      </c>
+      <c r="B122" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Therapist tip</t>
+        </is>
+      </c>
+      <c r="C122" s="123" t="inlineStr">
+        <is>
+          <t>Ask yourself this question when you're stuck (Solomon's paradox)</t>
+        </is>
+      </c>
+      <c r="D122" s="123" t="inlineStr">
+        <is>
+          <t>Ask yourself THIS when you're stuck: what would I tell a friend?</t>
+        </is>
+      </c>
+      <c r="E122" s="123" t="inlineStr">
+        <is>
+          <t>Grossmann &amp; Kross 2014: wiser reasoning about others' problems; self-distancing</t>
+        </is>
+      </c>
+      <c r="F122" s="123" t="n"/>
+      <c r="G122" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H122" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I122" s="124" t="n">
+        <v>15</v>
+      </c>
+      <c r="J122" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K122" s="124" t="inlineStr">
+        <is>
+          <t>friend-question</t>
+        </is>
+      </c>
+      <c r="L122" s="125" t="n"/>
+      <c r="M122" s="123">
+        <f>IF(L122="","",TEXT(L122,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N122" s="124" t="n"/>
+      <c r="O122" s="124" t="n"/>
+      <c r="P122" s="124" t="n"/>
+      <c r="Q122" s="124" t="n"/>
+      <c r="R122" s="124" t="n"/>
+      <c r="S122" s="126" t="n"/>
+      <c r="T122" s="124" t="n"/>
+      <c r="U122" s="127">
+        <f>IF(OR(T122="",N(O122)=0),"",T122/O122)</f>
+        <v/>
+      </c>
+      <c r="V122" s="124" t="n"/>
+      <c r="W122" s="124" t="n"/>
+      <c r="X122" s="124" t="n"/>
+      <c r="Y122" s="126" t="n"/>
+      <c r="Z122" s="124" t="n"/>
+      <c r="AA122" s="126" t="n"/>
+      <c r="AB122" s="124" t="n"/>
+      <c r="AC122" s="128">
+        <f>IF(COUNT(S122,Y122,AA122)=0,"",SUM(S122,Y122,AA122))</f>
+        <v/>
+      </c>
+      <c r="AD122" s="127">
+        <f>IF(N(AC122)=0,"",SUM(V122,W122,X122,Z122,AB122)/AC122)</f>
+        <v/>
+      </c>
+      <c r="AE122" s="126" t="n"/>
+      <c r="AF122" s="126" t="n"/>
+      <c r="AG122" s="126" t="n"/>
+      <c r="AH122" s="128">
+        <f>IF(COUNT(AE122,AF122,AG122)=0,"",SUM(AE122,AF122,AG122))</f>
+        <v/>
+      </c>
+      <c r="AI122" s="126" t="n"/>
+      <c r="AJ122" s="126" t="n"/>
+      <c r="AK122" s="126" t="n"/>
+      <c r="AL122" s="128">
+        <f>IF(COUNT(AI122,AJ122,AK122)=0,"",SUM(AI122,AJ122,AK122))</f>
+        <v/>
+      </c>
+      <c r="AM122" s="123">
+        <f>IF(N(AC122)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC122&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC122&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN122" s="124" t="n"/>
+      <c r="AO122" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP122" s="129" t="n"/>
+      <c r="AQ122" s="129" t="n"/>
+      <c r="AR122" s="129" t="n"/>
+      <c r="AS122" s="129" t="n"/>
+      <c r="AT122" s="129" t="n"/>
+      <c r="AU122" s="129" t="n"/>
+      <c r="AV122" s="130" t="inlineStr">
+        <is>
+          <t>Therapist tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="123" t="n">
+        <v>118</v>
+      </c>
+      <c r="B123" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Relationships &amp; likability</t>
+        </is>
+      </c>
+      <c r="C123" s="123" t="inlineStr">
+        <is>
+          <t>The shaky-bridge study: why fear feels like attraction</t>
+        </is>
+      </c>
+      <c r="D123" s="123" t="inlineStr">
+        <is>
+          <t>Men on a SHAKY bridge were far more likely to call a woman they just met.</t>
+        </is>
+      </c>
+      <c r="E123" s="123" t="inlineStr">
+        <is>
+          <t>Dutton &amp; Aron 1974 misattribution of arousal</t>
+        </is>
+      </c>
+      <c r="F123" s="123" t="n"/>
+      <c r="G123" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H123" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I123" s="124" t="n">
+        <v>16</v>
+      </c>
+      <c r="J123" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K123" s="124" t="inlineStr">
+        <is>
+          <t>shaky-bridge</t>
+        </is>
+      </c>
+      <c r="L123" s="125" t="n"/>
+      <c r="M123" s="123">
+        <f>IF(L123="","",TEXT(L123,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N123" s="124" t="n"/>
+      <c r="O123" s="124" t="n"/>
+      <c r="P123" s="124" t="n"/>
+      <c r="Q123" s="124" t="n"/>
+      <c r="R123" s="124" t="n"/>
+      <c r="S123" s="126" t="n"/>
+      <c r="T123" s="124" t="n"/>
+      <c r="U123" s="127">
+        <f>IF(OR(T123="",N(O123)=0),"",T123/O123)</f>
+        <v/>
+      </c>
+      <c r="V123" s="124" t="n"/>
+      <c r="W123" s="124" t="n"/>
+      <c r="X123" s="124" t="n"/>
+      <c r="Y123" s="126" t="n"/>
+      <c r="Z123" s="124" t="n"/>
+      <c r="AA123" s="126" t="n"/>
+      <c r="AB123" s="124" t="n"/>
+      <c r="AC123" s="128">
+        <f>IF(COUNT(S123,Y123,AA123)=0,"",SUM(S123,Y123,AA123))</f>
+        <v/>
+      </c>
+      <c r="AD123" s="127">
+        <f>IF(N(AC123)=0,"",SUM(V123,W123,X123,Z123,AB123)/AC123)</f>
+        <v/>
+      </c>
+      <c r="AE123" s="126" t="n"/>
+      <c r="AF123" s="126" t="n"/>
+      <c r="AG123" s="126" t="n"/>
+      <c r="AH123" s="128">
+        <f>IF(COUNT(AE123,AF123,AG123)=0,"",SUM(AE123,AF123,AG123))</f>
+        <v/>
+      </c>
+      <c r="AI123" s="126" t="n"/>
+      <c r="AJ123" s="126" t="n"/>
+      <c r="AK123" s="126" t="n"/>
+      <c r="AL123" s="128">
+        <f>IF(COUNT(AI123,AJ123,AK123)=0,"",SUM(AI123,AJ123,AK123))</f>
+        <v/>
+      </c>
+      <c r="AM123" s="123">
+        <f>IF(N(AC123)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC123&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC123&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN123" s="124" t="n"/>
+      <c r="AO123" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP123" s="129" t="n"/>
+      <c r="AQ123" s="129" t="n"/>
+      <c r="AR123" s="129" t="n"/>
+      <c r="AS123" s="129" t="n"/>
+      <c r="AT123" s="129" t="n"/>
+      <c r="AU123" s="129" t="n"/>
+      <c r="AV123" s="130" t="inlineStr">
+        <is>
+          <t>Relationships &amp; likability</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="123" t="n">
+        <v>119</v>
+      </c>
+      <c r="B124" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Strange named effect</t>
+        </is>
+      </c>
+      <c r="C124" s="123" t="inlineStr">
+        <is>
+          <t>Say a word 30 times and it stops meaning anything</t>
+        </is>
+      </c>
+      <c r="D124" s="123" t="inlineStr">
+        <is>
+          <t>Say any word thirty times and it stops MEANING anything.</t>
+        </is>
+      </c>
+      <c r="E124" s="123" t="inlineStr">
+        <is>
+          <t>Semantic satiation; Severance &amp; Washburn 1907; Lambert &amp; Jakobovits 1962</t>
+        </is>
+      </c>
+      <c r="F124" s="123" t="n"/>
+      <c r="G124" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H124" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I124" s="124" t="n">
+        <v>17</v>
+      </c>
+      <c r="J124" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K124" s="124" t="inlineStr">
+        <is>
+          <t>semantic-satiation</t>
+        </is>
+      </c>
+      <c r="L124" s="125" t="n"/>
+      <c r="M124" s="123">
+        <f>IF(L124="","",TEXT(L124,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N124" s="124" t="n"/>
+      <c r="O124" s="124" t="n"/>
+      <c r="P124" s="124" t="n"/>
+      <c r="Q124" s="124" t="n"/>
+      <c r="R124" s="124" t="n"/>
+      <c r="S124" s="126" t="n"/>
+      <c r="T124" s="124" t="n"/>
+      <c r="U124" s="127">
+        <f>IF(OR(T124="",N(O124)=0),"",T124/O124)</f>
+        <v/>
+      </c>
+      <c r="V124" s="124" t="n"/>
+      <c r="W124" s="124" t="n"/>
+      <c r="X124" s="124" t="n"/>
+      <c r="Y124" s="126" t="n"/>
+      <c r="Z124" s="124" t="n"/>
+      <c r="AA124" s="126" t="n"/>
+      <c r="AB124" s="124" t="n"/>
+      <c r="AC124" s="128">
+        <f>IF(COUNT(S124,Y124,AA124)=0,"",SUM(S124,Y124,AA124))</f>
+        <v/>
+      </c>
+      <c r="AD124" s="127">
+        <f>IF(N(AC124)=0,"",SUM(V124,W124,X124,Z124,AB124)/AC124)</f>
+        <v/>
+      </c>
+      <c r="AE124" s="126" t="n"/>
+      <c r="AF124" s="126" t="n"/>
+      <c r="AG124" s="126" t="n"/>
+      <c r="AH124" s="128">
+        <f>IF(COUNT(AE124,AF124,AG124)=0,"",SUM(AE124,AF124,AG124))</f>
+        <v/>
+      </c>
+      <c r="AI124" s="126" t="n"/>
+      <c r="AJ124" s="126" t="n"/>
+      <c r="AK124" s="126" t="n"/>
+      <c r="AL124" s="128">
+        <f>IF(COUNT(AI124,AJ124,AK124)=0,"",SUM(AI124,AJ124,AK124))</f>
+        <v/>
+      </c>
+      <c r="AM124" s="123">
+        <f>IF(N(AC124)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC124&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC124&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN124" s="124" t="n"/>
+      <c r="AO124" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP124" s="129" t="n"/>
+      <c r="AQ124" s="129" t="n"/>
+      <c r="AR124" s="129" t="n"/>
+      <c r="AS124" s="129" t="n"/>
+      <c r="AT124" s="129" t="n"/>
+      <c r="AU124" s="129" t="n"/>
+      <c r="AV124" s="130" t="inlineStr">
+        <is>
+          <t>Strange named effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="123" t="n">
+        <v>120</v>
+      </c>
+      <c r="B125" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Quiz / test yourself</t>
+        </is>
+      </c>
+      <c r="C125" s="123" t="inlineStr">
+        <is>
+          <t>Say the colour, not the word (Stroop test)</t>
+        </is>
+      </c>
+      <c r="D125" s="123" t="inlineStr">
+        <is>
+          <t>Say the COLOUR, not the word. Most people trip in seconds.</t>
+        </is>
+      </c>
+      <c r="E125" s="123" t="inlineStr">
+        <is>
+          <t>Stroop 1935; automatic reading</t>
+        </is>
+      </c>
+      <c r="F125" s="123" t="n"/>
+      <c r="G125" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H125" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I125" s="124" t="n">
+        <v>18</v>
+      </c>
+      <c r="J125" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K125" s="124" t="inlineStr">
+        <is>
+          <t>stroop-test</t>
+        </is>
+      </c>
+      <c r="L125" s="125" t="n"/>
+      <c r="M125" s="123">
+        <f>IF(L125="","",TEXT(L125,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N125" s="124" t="n"/>
+      <c r="O125" s="124" t="n"/>
+      <c r="P125" s="124" t="n"/>
+      <c r="Q125" s="124" t="n"/>
+      <c r="R125" s="124" t="n"/>
+      <c r="S125" s="126" t="n"/>
+      <c r="T125" s="124" t="n"/>
+      <c r="U125" s="127">
+        <f>IF(OR(T125="",N(O125)=0),"",T125/O125)</f>
+        <v/>
+      </c>
+      <c r="V125" s="124" t="n"/>
+      <c r="W125" s="124" t="n"/>
+      <c r="X125" s="124" t="n"/>
+      <c r="Y125" s="126" t="n"/>
+      <c r="Z125" s="124" t="n"/>
+      <c r="AA125" s="126" t="n"/>
+      <c r="AB125" s="124" t="n"/>
+      <c r="AC125" s="128">
+        <f>IF(COUNT(S125,Y125,AA125)=0,"",SUM(S125,Y125,AA125))</f>
+        <v/>
+      </c>
+      <c r="AD125" s="127">
+        <f>IF(N(AC125)=0,"",SUM(V125,W125,X125,Z125,AB125)/AC125)</f>
+        <v/>
+      </c>
+      <c r="AE125" s="126" t="n"/>
+      <c r="AF125" s="126" t="n"/>
+      <c r="AG125" s="126" t="n"/>
+      <c r="AH125" s="128">
+        <f>IF(COUNT(AE125,AF125,AG125)=0,"",SUM(AE125,AF125,AG125))</f>
+        <v/>
+      </c>
+      <c r="AI125" s="126" t="n"/>
+      <c r="AJ125" s="126" t="n"/>
+      <c r="AK125" s="126" t="n"/>
+      <c r="AL125" s="128">
+        <f>IF(COUNT(AI125,AJ125,AK125)=0,"",SUM(AI125,AJ125,AK125))</f>
+        <v/>
+      </c>
+      <c r="AM125" s="123">
+        <f>IF(N(AC125)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC125&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC125&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN125" s="124" t="n"/>
+      <c r="AO125" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP125" s="129" t="n"/>
+      <c r="AQ125" s="129" t="n"/>
+      <c r="AR125" s="129" t="n"/>
+      <c r="AS125" s="129" t="n"/>
+      <c r="AT125" s="129" t="n"/>
+      <c r="AU125" s="129" t="n"/>
+      <c r="AV125" s="130" t="inlineStr">
+        <is>
+          <t>Quiz / test yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="123" t="n">
+        <v>121</v>
+      </c>
+      <c r="B126" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Presence &amp; influence rules</t>
+        </is>
+      </c>
+      <c r="C126" s="123" t="inlineStr">
+        <is>
+          <t>The one word that gets people to say yes ('because')</t>
+        </is>
+      </c>
+      <c r="D126" s="123" t="inlineStr">
+        <is>
+          <t>ONE word got people to let a stranger cut the line.</t>
+        </is>
+      </c>
+      <c r="E126" s="123" t="inlineStr">
+        <is>
+          <t>Langer, Blank &amp; Chanowitz 1978: 94% / 93% / 60%</t>
+        </is>
+      </c>
+      <c r="F126" s="123" t="n"/>
+      <c r="G126" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H126" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I126" s="124" t="n">
+        <v>19</v>
+      </c>
+      <c r="J126" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K126" s="124" t="inlineStr">
+        <is>
+          <t>because-copier</t>
+        </is>
+      </c>
+      <c r="L126" s="125" t="n"/>
+      <c r="M126" s="123">
+        <f>IF(L126="","",TEXT(L126,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N126" s="124" t="n"/>
+      <c r="O126" s="124" t="n"/>
+      <c r="P126" s="124" t="n"/>
+      <c r="Q126" s="124" t="n"/>
+      <c r="R126" s="124" t="n"/>
+      <c r="S126" s="126" t="n"/>
+      <c r="T126" s="124" t="n"/>
+      <c r="U126" s="127">
+        <f>IF(OR(T126="",N(O126)=0),"",T126/O126)</f>
+        <v/>
+      </c>
+      <c r="V126" s="124" t="n"/>
+      <c r="W126" s="124" t="n"/>
+      <c r="X126" s="124" t="n"/>
+      <c r="Y126" s="126" t="n"/>
+      <c r="Z126" s="124" t="n"/>
+      <c r="AA126" s="126" t="n"/>
+      <c r="AB126" s="124" t="n"/>
+      <c r="AC126" s="128">
+        <f>IF(COUNT(S126,Y126,AA126)=0,"",SUM(S126,Y126,AA126))</f>
+        <v/>
+      </c>
+      <c r="AD126" s="127">
+        <f>IF(N(AC126)=0,"",SUM(V126,W126,X126,Z126,AB126)/AC126)</f>
+        <v/>
+      </c>
+      <c r="AE126" s="126" t="n"/>
+      <c r="AF126" s="126" t="n"/>
+      <c r="AG126" s="126" t="n"/>
+      <c r="AH126" s="128">
+        <f>IF(COUNT(AE126,AF126,AG126)=0,"",SUM(AE126,AF126,AG126))</f>
+        <v/>
+      </c>
+      <c r="AI126" s="126" t="n"/>
+      <c r="AJ126" s="126" t="n"/>
+      <c r="AK126" s="126" t="n"/>
+      <c r="AL126" s="128">
+        <f>IF(COUNT(AI126,AJ126,AK126)=0,"",SUM(AI126,AJ126,AK126))</f>
+        <v/>
+      </c>
+      <c r="AM126" s="123">
+        <f>IF(N(AC126)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC126&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC126&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN126" s="124" t="n"/>
+      <c r="AO126" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP126" s="129" t="n"/>
+      <c r="AQ126" s="129" t="n"/>
+      <c r="AR126" s="129" t="n"/>
+      <c r="AS126" s="129" t="n"/>
+      <c r="AT126" s="129" t="n"/>
+      <c r="AU126" s="129" t="n"/>
+      <c r="AV126" s="130" t="inlineStr">
+        <is>
+          <t>Presence &amp; influence rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B127" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Psychology says (15 s loop)</t>
+        </is>
+      </c>
+      <c r="C127" s="123" t="inlineStr">
+        <is>
+          <t>Psychology says: you remember the ending, not the whole thing</t>
+        </is>
+      </c>
+      <c r="D127" s="123" t="inlineStr">
+        <is>
+          <t>Psychology says: you'll remember how something ENDS, not how long it lasted.</t>
+        </is>
+      </c>
+      <c r="E127" s="123" t="inlineStr">
+        <is>
+          <t>Kahneman et al. 1993 cold-hand study</t>
+        </is>
+      </c>
+      <c r="F127" s="123" t="n"/>
+      <c r="G127" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H127" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I127" s="124" t="n">
+        <v>20</v>
+      </c>
+      <c r="J127" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K127" s="124" t="inlineStr">
+        <is>
+          <t>peak-end-rule</t>
+        </is>
+      </c>
+      <c r="L127" s="125" t="n"/>
+      <c r="M127" s="123">
+        <f>IF(L127="","",TEXT(L127,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N127" s="124" t="n"/>
+      <c r="O127" s="124" t="n"/>
+      <c r="P127" s="124" t="n"/>
+      <c r="Q127" s="124" t="n"/>
+      <c r="R127" s="124" t="n"/>
+      <c r="S127" s="126" t="n"/>
+      <c r="T127" s="124" t="n"/>
+      <c r="U127" s="127">
+        <f>IF(OR(T127="",N(O127)=0),"",T127/O127)</f>
+        <v/>
+      </c>
+      <c r="V127" s="124" t="n"/>
+      <c r="W127" s="124" t="n"/>
+      <c r="X127" s="124" t="n"/>
+      <c r="Y127" s="126" t="n"/>
+      <c r="Z127" s="124" t="n"/>
+      <c r="AA127" s="126" t="n"/>
+      <c r="AB127" s="124" t="n"/>
+      <c r="AC127" s="128">
+        <f>IF(COUNT(S127,Y127,AA127)=0,"",SUM(S127,Y127,AA127))</f>
+        <v/>
+      </c>
+      <c r="AD127" s="127">
+        <f>IF(N(AC127)=0,"",SUM(V127,W127,X127,Z127,AB127)/AC127)</f>
+        <v/>
+      </c>
+      <c r="AE127" s="126" t="n"/>
+      <c r="AF127" s="126" t="n"/>
+      <c r="AG127" s="126" t="n"/>
+      <c r="AH127" s="128">
+        <f>IF(COUNT(AE127,AF127,AG127)=0,"",SUM(AE127,AF127,AG127))</f>
+        <v/>
+      </c>
+      <c r="AI127" s="126" t="n"/>
+      <c r="AJ127" s="126" t="n"/>
+      <c r="AK127" s="126" t="n"/>
+      <c r="AL127" s="128">
+        <f>IF(COUNT(AI127,AJ127,AK127)=0,"",SUM(AI127,AJ127,AK127))</f>
+        <v/>
+      </c>
+      <c r="AM127" s="123">
+        <f>IF(N(AC127)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC127&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC127&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN127" s="124" t="n"/>
+      <c r="AO127" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP127" s="129" t="n"/>
+      <c r="AQ127" s="129" t="n"/>
+      <c r="AR127" s="129" t="n"/>
+      <c r="AS127" s="129" t="n"/>
+      <c r="AT127" s="129" t="n"/>
+      <c r="AU127" s="129" t="n"/>
+      <c r="AV127" s="130" t="inlineStr">
+        <is>
+          <t>Psychology says (15 s loop)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="123" t="n">
+        <v>123</v>
+      </c>
+      <c r="B128" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Experiment story</t>
+        </is>
+      </c>
+      <c r="C128" s="123" t="inlineStr">
+        <is>
+          <t>The experiment where people kept pressing the button (Milgram)</t>
+        </is>
+      </c>
+      <c r="D128" s="123" t="inlineStr">
+        <is>
+          <t>Two out of three ordinary people kept going to the highest SHOCK.</t>
+        </is>
+      </c>
+      <c r="E128" s="123" t="inlineStr">
+        <is>
+          <t>Milgram 1963: 65% to 450V; turn: variations &amp; critiques</t>
+        </is>
+      </c>
+      <c r="F128" s="123" t="n"/>
+      <c r="G128" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H128" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I128" s="124" t="n">
+        <v>21</v>
+      </c>
+      <c r="J128" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K128" s="124" t="inlineStr">
+        <is>
+          <t>milgram-obedience</t>
+        </is>
+      </c>
+      <c r="L128" s="125" t="n"/>
+      <c r="M128" s="123">
+        <f>IF(L128="","",TEXT(L128,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N128" s="124" t="n"/>
+      <c r="O128" s="124" t="n"/>
+      <c r="P128" s="124" t="n"/>
+      <c r="Q128" s="124" t="n"/>
+      <c r="R128" s="124" t="n"/>
+      <c r="S128" s="126" t="n"/>
+      <c r="T128" s="124" t="n"/>
+      <c r="U128" s="127">
+        <f>IF(OR(T128="",N(O128)=0),"",T128/O128)</f>
+        <v/>
+      </c>
+      <c r="V128" s="124" t="n"/>
+      <c r="W128" s="124" t="n"/>
+      <c r="X128" s="124" t="n"/>
+      <c r="Y128" s="126" t="n"/>
+      <c r="Z128" s="124" t="n"/>
+      <c r="AA128" s="126" t="n"/>
+      <c r="AB128" s="124" t="n"/>
+      <c r="AC128" s="128">
+        <f>IF(COUNT(S128,Y128,AA128)=0,"",SUM(S128,Y128,AA128))</f>
+        <v/>
+      </c>
+      <c r="AD128" s="127">
+        <f>IF(N(AC128)=0,"",SUM(V128,W128,X128,Z128,AB128)/AC128)</f>
+        <v/>
+      </c>
+      <c r="AE128" s="126" t="n"/>
+      <c r="AF128" s="126" t="n"/>
+      <c r="AG128" s="126" t="n"/>
+      <c r="AH128" s="128">
+        <f>IF(COUNT(AE128,AF128,AG128)=0,"",SUM(AE128,AF128,AG128))</f>
+        <v/>
+      </c>
+      <c r="AI128" s="126" t="n"/>
+      <c r="AJ128" s="126" t="n"/>
+      <c r="AK128" s="126" t="n"/>
+      <c r="AL128" s="128">
+        <f>IF(COUNT(AI128,AJ128,AK128)=0,"",SUM(AI128,AJ128,AK128))</f>
+        <v/>
+      </c>
+      <c r="AM128" s="123">
+        <f>IF(N(AC128)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC128&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC128&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN128" s="124" t="n"/>
+      <c r="AO128" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP128" s="129" t="n"/>
+      <c r="AQ128" s="129" t="n"/>
+      <c r="AR128" s="129" t="n"/>
+      <c r="AS128" s="129" t="n"/>
+      <c r="AT128" s="129" t="n"/>
+      <c r="AU128" s="129" t="n"/>
+      <c r="AV128" s="130" t="inlineStr">
+        <is>
+          <t>Experiment story</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="123" t="n">
+        <v>124</v>
+      </c>
+      <c r="B129" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Protect yourself</t>
+        </is>
+      </c>
+      <c r="C129" s="123" t="inlineStr">
+        <is>
+          <t>Why 'only 2 left' works on you (scarcity)</t>
+        </is>
+      </c>
+      <c r="D129" s="123" t="inlineStr">
+        <is>
+          <t>Same cookies, but people rated them BETTER from a nearly empty jar.</t>
+        </is>
+      </c>
+      <c r="E129" s="123" t="inlineStr">
+        <is>
+          <t>Worchel, Lee &amp; Adewole 1975</t>
+        </is>
+      </c>
+      <c r="F129" s="123" t="n"/>
+      <c r="G129" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H129" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I129" s="124" t="n">
+        <v>22</v>
+      </c>
+      <c r="J129" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K129" s="124" t="inlineStr">
+        <is>
+          <t>scarcity-cookies</t>
+        </is>
+      </c>
+      <c r="L129" s="125" t="n"/>
+      <c r="M129" s="123">
+        <f>IF(L129="","",TEXT(L129,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N129" s="124" t="n"/>
+      <c r="O129" s="124" t="n"/>
+      <c r="P129" s="124" t="n"/>
+      <c r="Q129" s="124" t="n"/>
+      <c r="R129" s="124" t="n"/>
+      <c r="S129" s="126" t="n"/>
+      <c r="T129" s="124" t="n"/>
+      <c r="U129" s="127">
+        <f>IF(OR(T129="",N(O129)=0),"",T129/O129)</f>
+        <v/>
+      </c>
+      <c r="V129" s="124" t="n"/>
+      <c r="W129" s="124" t="n"/>
+      <c r="X129" s="124" t="n"/>
+      <c r="Y129" s="126" t="n"/>
+      <c r="Z129" s="124" t="n"/>
+      <c r="AA129" s="126" t="n"/>
+      <c r="AB129" s="124" t="n"/>
+      <c r="AC129" s="128">
+        <f>IF(COUNT(S129,Y129,AA129)=0,"",SUM(S129,Y129,AA129))</f>
+        <v/>
+      </c>
+      <c r="AD129" s="127">
+        <f>IF(N(AC129)=0,"",SUM(V129,W129,X129,Z129,AB129)/AC129)</f>
+        <v/>
+      </c>
+      <c r="AE129" s="126" t="n"/>
+      <c r="AF129" s="126" t="n"/>
+      <c r="AG129" s="126" t="n"/>
+      <c r="AH129" s="128">
+        <f>IF(COUNT(AE129,AF129,AG129)=0,"",SUM(AE129,AF129,AG129))</f>
+        <v/>
+      </c>
+      <c r="AI129" s="126" t="n"/>
+      <c r="AJ129" s="126" t="n"/>
+      <c r="AK129" s="126" t="n"/>
+      <c r="AL129" s="128">
+        <f>IF(COUNT(AI129,AJ129,AK129)=0,"",SUM(AI129,AJ129,AK129))</f>
+        <v/>
+      </c>
+      <c r="AM129" s="123">
+        <f>IF(N(AC129)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC129&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC129&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN129" s="124" t="n"/>
+      <c r="AO129" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP129" s="129" t="n"/>
+      <c r="AQ129" s="129" t="n"/>
+      <c r="AR129" s="129" t="n"/>
+      <c r="AS129" s="129" t="n"/>
+      <c r="AT129" s="129" t="n"/>
+      <c r="AU129" s="129" t="n"/>
+      <c r="AV129" s="130" t="inlineStr">
+        <is>
+          <t>Protect yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="123" t="n">
+        <v>125</v>
+      </c>
+      <c r="B130" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Psychology of people who</t>
+        </is>
+      </c>
+      <c r="C130" s="123" t="inlineStr">
+        <is>
+          <t>Psychology of people who talk to themselves in third person</t>
+        </is>
+      </c>
+      <c r="D130" s="123" t="inlineStr">
+        <is>
+          <t>Psychology of people who talk to themselves by NAME.</t>
+        </is>
+      </c>
+      <c r="E130" s="123" t="inlineStr">
+        <is>
+          <t>Kross et al. 2014 self-distancing reduces anxiety</t>
+        </is>
+      </c>
+      <c r="F130" s="123" t="n"/>
+      <c r="G130" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H130" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I130" s="124" t="n">
+        <v>23</v>
+      </c>
+      <c r="J130" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K130" s="124" t="inlineStr">
+        <is>
+          <t>talk-to-yourself</t>
+        </is>
+      </c>
+      <c r="L130" s="125" t="n"/>
+      <c r="M130" s="123">
+        <f>IF(L130="","",TEXT(L130,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N130" s="124" t="n"/>
+      <c r="O130" s="124" t="n"/>
+      <c r="P130" s="124" t="n"/>
+      <c r="Q130" s="124" t="n"/>
+      <c r="R130" s="124" t="n"/>
+      <c r="S130" s="126" t="n"/>
+      <c r="T130" s="124" t="n"/>
+      <c r="U130" s="127">
+        <f>IF(OR(T130="",N(O130)=0),"",T130/O130)</f>
+        <v/>
+      </c>
+      <c r="V130" s="124" t="n"/>
+      <c r="W130" s="124" t="n"/>
+      <c r="X130" s="124" t="n"/>
+      <c r="Y130" s="126" t="n"/>
+      <c r="Z130" s="124" t="n"/>
+      <c r="AA130" s="126" t="n"/>
+      <c r="AB130" s="124" t="n"/>
+      <c r="AC130" s="128">
+        <f>IF(COUNT(S130,Y130,AA130)=0,"",SUM(S130,Y130,AA130))</f>
+        <v/>
+      </c>
+      <c r="AD130" s="127">
+        <f>IF(N(AC130)=0,"",SUM(V130,W130,X130,Z130,AB130)/AC130)</f>
+        <v/>
+      </c>
+      <c r="AE130" s="126" t="n"/>
+      <c r="AF130" s="126" t="n"/>
+      <c r="AG130" s="126" t="n"/>
+      <c r="AH130" s="128">
+        <f>IF(COUNT(AE130,AF130,AG130)=0,"",SUM(AE130,AF130,AG130))</f>
+        <v/>
+      </c>
+      <c r="AI130" s="126" t="n"/>
+      <c r="AJ130" s="126" t="n"/>
+      <c r="AK130" s="126" t="n"/>
+      <c r="AL130" s="128">
+        <f>IF(COUNT(AI130,AJ130,AK130)=0,"",SUM(AI130,AJ130,AK130))</f>
+        <v/>
+      </c>
+      <c r="AM130" s="123">
+        <f>IF(N(AC130)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC130&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC130&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN130" s="124" t="n"/>
+      <c r="AO130" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP130" s="129" t="n"/>
+      <c r="AQ130" s="129" t="n"/>
+      <c r="AR130" s="129" t="n"/>
+      <c r="AS130" s="129" t="n"/>
+      <c r="AT130" s="129" t="n"/>
+      <c r="AU130" s="129" t="n"/>
+      <c r="AV130" s="130" t="inlineStr">
+        <is>
+          <t>Psychology of people who</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="123" t="n">
+        <v>126</v>
+      </c>
+      <c r="B131" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Numbered facts</t>
+        </is>
+      </c>
+      <c r="C131" s="123" t="inlineStr">
+        <is>
+          <t>3 facts about how you decide</t>
+        </is>
+      </c>
+      <c r="D131" s="123" t="inlineStr">
+        <is>
+          <t>Three facts about your decisions. Number one could change who gets an ORGAN.</t>
+        </is>
+      </c>
+      <c r="E131" s="123" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Goldstein 2003 defaults; Iyengar &amp; Lepper 2000 jam (mixed replications); Shafir decoy</t>
+        </is>
+      </c>
+      <c r="F131" s="123" t="n"/>
+      <c r="G131" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H131" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I131" s="124" t="n">
+        <v>24</v>
+      </c>
+      <c r="J131" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K131" s="124" t="inlineStr">
+        <is>
+          <t>decision-facts</t>
+        </is>
+      </c>
+      <c r="L131" s="125" t="n"/>
+      <c r="M131" s="123">
+        <f>IF(L131="","",TEXT(L131,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N131" s="124" t="n"/>
+      <c r="O131" s="124" t="n"/>
+      <c r="P131" s="124" t="n"/>
+      <c r="Q131" s="124" t="n"/>
+      <c r="R131" s="124" t="n"/>
+      <c r="S131" s="126" t="n"/>
+      <c r="T131" s="124" t="n"/>
+      <c r="U131" s="127">
+        <f>IF(OR(T131="",N(O131)=0),"",T131/O131)</f>
+        <v/>
+      </c>
+      <c r="V131" s="124" t="n"/>
+      <c r="W131" s="124" t="n"/>
+      <c r="X131" s="124" t="n"/>
+      <c r="Y131" s="126" t="n"/>
+      <c r="Z131" s="124" t="n"/>
+      <c r="AA131" s="126" t="n"/>
+      <c r="AB131" s="124" t="n"/>
+      <c r="AC131" s="128">
+        <f>IF(COUNT(S131,Y131,AA131)=0,"",SUM(S131,Y131,AA131))</f>
+        <v/>
+      </c>
+      <c r="AD131" s="127">
+        <f>IF(N(AC131)=0,"",SUM(V131,W131,X131,Z131,AB131)/AC131)</f>
+        <v/>
+      </c>
+      <c r="AE131" s="126" t="n"/>
+      <c r="AF131" s="126" t="n"/>
+      <c r="AG131" s="126" t="n"/>
+      <c r="AH131" s="128">
+        <f>IF(COUNT(AE131,AF131,AG131)=0,"",SUM(AE131,AF131,AG131))</f>
+        <v/>
+      </c>
+      <c r="AI131" s="126" t="n"/>
+      <c r="AJ131" s="126" t="n"/>
+      <c r="AK131" s="126" t="n"/>
+      <c r="AL131" s="128">
+        <f>IF(COUNT(AI131,AJ131,AK131)=0,"",SUM(AI131,AJ131,AK131))</f>
+        <v/>
+      </c>
+      <c r="AM131" s="123">
+        <f>IF(N(AC131)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC131&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC131&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN131" s="124" t="n"/>
+      <c r="AO131" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP131" s="129" t="n"/>
+      <c r="AQ131" s="129" t="n"/>
+      <c r="AR131" s="129" t="n"/>
+      <c r="AS131" s="129" t="n"/>
+      <c r="AT131" s="129" t="n"/>
+      <c r="AU131" s="129" t="n"/>
+      <c r="AV131" s="130" t="inlineStr">
+        <is>
+          <t>Numbered facts</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="123" t="n">
+        <v>127</v>
+      </c>
+      <c r="B132" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Therapist tip</t>
+        </is>
+      </c>
+      <c r="C132" s="123" t="inlineStr">
+        <is>
+          <t>The gratitude visit: one letter, a month of happiness</t>
+        </is>
+      </c>
+      <c r="D132" s="123" t="inlineStr">
+        <is>
+          <t>One letter made people happier for a MONTH.</t>
+        </is>
+      </c>
+      <c r="E132" s="123" t="inlineStr">
+        <is>
+          <t>Seligman et al. 2005 gratitude visit</t>
+        </is>
+      </c>
+      <c r="F132" s="123" t="n"/>
+      <c r="G132" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H132" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I132" s="124" t="n">
+        <v>25</v>
+      </c>
+      <c r="J132" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K132" s="124" t="inlineStr">
+        <is>
+          <t>gratitude-visit</t>
+        </is>
+      </c>
+      <c r="L132" s="125" t="n"/>
+      <c r="M132" s="123">
+        <f>IF(L132="","",TEXT(L132,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N132" s="124" t="n"/>
+      <c r="O132" s="124" t="n"/>
+      <c r="P132" s="124" t="n"/>
+      <c r="Q132" s="124" t="n"/>
+      <c r="R132" s="124" t="n"/>
+      <c r="S132" s="126" t="n"/>
+      <c r="T132" s="124" t="n"/>
+      <c r="U132" s="127">
+        <f>IF(OR(T132="",N(O132)=0),"",T132/O132)</f>
+        <v/>
+      </c>
+      <c r="V132" s="124" t="n"/>
+      <c r="W132" s="124" t="n"/>
+      <c r="X132" s="124" t="n"/>
+      <c r="Y132" s="126" t="n"/>
+      <c r="Z132" s="124" t="n"/>
+      <c r="AA132" s="126" t="n"/>
+      <c r="AB132" s="124" t="n"/>
+      <c r="AC132" s="128">
+        <f>IF(COUNT(S132,Y132,AA132)=0,"",SUM(S132,Y132,AA132))</f>
+        <v/>
+      </c>
+      <c r="AD132" s="127">
+        <f>IF(N(AC132)=0,"",SUM(V132,W132,X132,Z132,AB132)/AC132)</f>
+        <v/>
+      </c>
+      <c r="AE132" s="126" t="n"/>
+      <c r="AF132" s="126" t="n"/>
+      <c r="AG132" s="126" t="n"/>
+      <c r="AH132" s="128">
+        <f>IF(COUNT(AE132,AF132,AG132)=0,"",SUM(AE132,AF132,AG132))</f>
+        <v/>
+      </c>
+      <c r="AI132" s="126" t="n"/>
+      <c r="AJ132" s="126" t="n"/>
+      <c r="AK132" s="126" t="n"/>
+      <c r="AL132" s="128">
+        <f>IF(COUNT(AI132,AJ132,AK132)=0,"",SUM(AI132,AJ132,AK132))</f>
+        <v/>
+      </c>
+      <c r="AM132" s="123">
+        <f>IF(N(AC132)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC132&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC132&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN132" s="124" t="n"/>
+      <c r="AO132" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP132" s="129" t="n"/>
+      <c r="AQ132" s="129" t="n"/>
+      <c r="AR132" s="129" t="n"/>
+      <c r="AS132" s="129" t="n"/>
+      <c r="AT132" s="129" t="n"/>
+      <c r="AU132" s="129" t="n"/>
+      <c r="AV132" s="130" t="inlineStr">
+        <is>
+          <t>Therapist tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="123" t="n">
+        <v>128</v>
+      </c>
+      <c r="B133" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Relationships &amp; likability</t>
+        </is>
+      </c>
+      <c r="C133" s="123" t="inlineStr">
+        <is>
+          <t>The 36 questions that made strangers close</t>
+        </is>
+      </c>
+      <c r="D133" s="123" t="inlineStr">
+        <is>
+          <t>Thirty-six questions made strangers feel CLOSE in under an hour.</t>
+        </is>
+      </c>
+      <c r="E133" s="123" t="inlineStr">
+        <is>
+          <t>Aron et al. 1997</t>
+        </is>
+      </c>
+      <c r="F133" s="123" t="n"/>
+      <c r="G133" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H133" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I133" s="124" t="n">
+        <v>26</v>
+      </c>
+      <c r="J133" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K133" s="124" t="inlineStr">
+        <is>
+          <t>thirty-six-questions</t>
+        </is>
+      </c>
+      <c r="L133" s="125" t="n"/>
+      <c r="M133" s="123">
+        <f>IF(L133="","",TEXT(L133,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N133" s="124" t="n"/>
+      <c r="O133" s="124" t="n"/>
+      <c r="P133" s="124" t="n"/>
+      <c r="Q133" s="124" t="n"/>
+      <c r="R133" s="124" t="n"/>
+      <c r="S133" s="126" t="n"/>
+      <c r="T133" s="124" t="n"/>
+      <c r="U133" s="127">
+        <f>IF(OR(T133="",N(O133)=0),"",T133/O133)</f>
+        <v/>
+      </c>
+      <c r="V133" s="124" t="n"/>
+      <c r="W133" s="124" t="n"/>
+      <c r="X133" s="124" t="n"/>
+      <c r="Y133" s="126" t="n"/>
+      <c r="Z133" s="124" t="n"/>
+      <c r="AA133" s="126" t="n"/>
+      <c r="AB133" s="124" t="n"/>
+      <c r="AC133" s="128">
+        <f>IF(COUNT(S133,Y133,AA133)=0,"",SUM(S133,Y133,AA133))</f>
+        <v/>
+      </c>
+      <c r="AD133" s="127">
+        <f>IF(N(AC133)=0,"",SUM(V133,W133,X133,Z133,AB133)/AC133)</f>
+        <v/>
+      </c>
+      <c r="AE133" s="126" t="n"/>
+      <c r="AF133" s="126" t="n"/>
+      <c r="AG133" s="126" t="n"/>
+      <c r="AH133" s="128">
+        <f>IF(COUNT(AE133,AF133,AG133)=0,"",SUM(AE133,AF133,AG133))</f>
+        <v/>
+      </c>
+      <c r="AI133" s="126" t="n"/>
+      <c r="AJ133" s="126" t="n"/>
+      <c r="AK133" s="126" t="n"/>
+      <c r="AL133" s="128">
+        <f>IF(COUNT(AI133,AJ133,AK133)=0,"",SUM(AI133,AJ133,AK133))</f>
+        <v/>
+      </c>
+      <c r="AM133" s="123">
+        <f>IF(N(AC133)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC133&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC133&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN133" s="124" t="n"/>
+      <c r="AO133" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP133" s="129" t="n"/>
+      <c r="AQ133" s="129" t="n"/>
+      <c r="AR133" s="129" t="n"/>
+      <c r="AS133" s="129" t="n"/>
+      <c r="AT133" s="129" t="n"/>
+      <c r="AU133" s="129" t="n"/>
+      <c r="AV133" s="130" t="inlineStr">
+        <is>
+          <t>Relationships &amp; likability</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="123" t="n">
+        <v>129</v>
+      </c>
+      <c r="B134" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Strange named effect</t>
+        </is>
+      </c>
+      <c r="C134" s="123" t="inlineStr">
+        <is>
+          <t>Lima syndrome: when captors bond with hostages</t>
+        </is>
+      </c>
+      <c r="D134" s="123" t="inlineStr">
+        <is>
+          <t>You've heard of Stockholm syndrome. This is the REVERSE.</t>
+        </is>
+      </c>
+      <c r="E134" s="123" t="inlineStr">
+        <is>
+          <t>1996 Lima Japanese embassy hostage crisis; captors released hostages</t>
+        </is>
+      </c>
+      <c r="F134" s="123" t="n"/>
+      <c r="G134" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H134" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I134" s="124" t="n">
+        <v>27</v>
+      </c>
+      <c r="J134" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K134" s="124" t="inlineStr">
+        <is>
+          <t>lima-syndrome</t>
+        </is>
+      </c>
+      <c r="L134" s="125" t="n"/>
+      <c r="M134" s="123">
+        <f>IF(L134="","",TEXT(L134,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N134" s="124" t="n"/>
+      <c r="O134" s="124" t="n"/>
+      <c r="P134" s="124" t="n"/>
+      <c r="Q134" s="124" t="n"/>
+      <c r="R134" s="124" t="n"/>
+      <c r="S134" s="126" t="n"/>
+      <c r="T134" s="124" t="n"/>
+      <c r="U134" s="127">
+        <f>IF(OR(T134="",N(O134)=0),"",T134/O134)</f>
+        <v/>
+      </c>
+      <c r="V134" s="124" t="n"/>
+      <c r="W134" s="124" t="n"/>
+      <c r="X134" s="124" t="n"/>
+      <c r="Y134" s="126" t="n"/>
+      <c r="Z134" s="124" t="n"/>
+      <c r="AA134" s="126" t="n"/>
+      <c r="AB134" s="124" t="n"/>
+      <c r="AC134" s="128">
+        <f>IF(COUNT(S134,Y134,AA134)=0,"",SUM(S134,Y134,AA134))</f>
+        <v/>
+      </c>
+      <c r="AD134" s="127">
+        <f>IF(N(AC134)=0,"",SUM(V134,W134,X134,Z134,AB134)/AC134)</f>
+        <v/>
+      </c>
+      <c r="AE134" s="126" t="n"/>
+      <c r="AF134" s="126" t="n"/>
+      <c r="AG134" s="126" t="n"/>
+      <c r="AH134" s="128">
+        <f>IF(COUNT(AE134,AF134,AG134)=0,"",SUM(AE134,AF134,AG134))</f>
+        <v/>
+      </c>
+      <c r="AI134" s="126" t="n"/>
+      <c r="AJ134" s="126" t="n"/>
+      <c r="AK134" s="126" t="n"/>
+      <c r="AL134" s="128">
+        <f>IF(COUNT(AI134,AJ134,AK134)=0,"",SUM(AI134,AJ134,AK134))</f>
+        <v/>
+      </c>
+      <c r="AM134" s="123">
+        <f>IF(N(AC134)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC134&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC134&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN134" s="124" t="n"/>
+      <c r="AO134" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP134" s="129" t="n"/>
+      <c r="AQ134" s="129" t="n"/>
+      <c r="AR134" s="129" t="n"/>
+      <c r="AS134" s="129" t="n"/>
+      <c r="AT134" s="129" t="n"/>
+      <c r="AU134" s="129" t="n"/>
+      <c r="AV134" s="130" t="inlineStr">
+        <is>
+          <t>Strange named effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="123" t="n">
+        <v>130</v>
+      </c>
+      <c r="B135" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Quiz / test yourself</t>
+        </is>
+      </c>
+      <c r="C135" s="123" t="inlineStr">
+        <is>
+          <t>Are you a maximizer or a satisficer? Take the test</t>
+        </is>
+      </c>
+      <c r="D135" s="123" t="inlineStr">
+        <is>
+          <t>Do you always look for the BEST option? That might be making you less happy.</t>
+        </is>
+      </c>
+      <c r="E135" s="123" t="inlineStr">
+        <is>
+          <t>Schwartz et al. 2002 maximizers less satisfied</t>
+        </is>
+      </c>
+      <c r="F135" s="123" t="n"/>
+      <c r="G135" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H135" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I135" s="124" t="n">
+        <v>28</v>
+      </c>
+      <c r="J135" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K135" s="124" t="inlineStr">
+        <is>
+          <t>maximizer-test</t>
+        </is>
+      </c>
+      <c r="L135" s="125" t="n"/>
+      <c r="M135" s="123">
+        <f>IF(L135="","",TEXT(L135,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N135" s="124" t="n"/>
+      <c r="O135" s="124" t="n"/>
+      <c r="P135" s="124" t="n"/>
+      <c r="Q135" s="124" t="n"/>
+      <c r="R135" s="124" t="n"/>
+      <c r="S135" s="126" t="n"/>
+      <c r="T135" s="124" t="n"/>
+      <c r="U135" s="127">
+        <f>IF(OR(T135="",N(O135)=0),"",T135/O135)</f>
+        <v/>
+      </c>
+      <c r="V135" s="124" t="n"/>
+      <c r="W135" s="124" t="n"/>
+      <c r="X135" s="124" t="n"/>
+      <c r="Y135" s="126" t="n"/>
+      <c r="Z135" s="124" t="n"/>
+      <c r="AA135" s="126" t="n"/>
+      <c r="AB135" s="124" t="n"/>
+      <c r="AC135" s="128">
+        <f>IF(COUNT(S135,Y135,AA135)=0,"",SUM(S135,Y135,AA135))</f>
+        <v/>
+      </c>
+      <c r="AD135" s="127">
+        <f>IF(N(AC135)=0,"",SUM(V135,W135,X135,Z135,AB135)/AC135)</f>
+        <v/>
+      </c>
+      <c r="AE135" s="126" t="n"/>
+      <c r="AF135" s="126" t="n"/>
+      <c r="AG135" s="126" t="n"/>
+      <c r="AH135" s="128">
+        <f>IF(COUNT(AE135,AF135,AG135)=0,"",SUM(AE135,AF135,AG135))</f>
+        <v/>
+      </c>
+      <c r="AI135" s="126" t="n"/>
+      <c r="AJ135" s="126" t="n"/>
+      <c r="AK135" s="126" t="n"/>
+      <c r="AL135" s="128">
+        <f>IF(COUNT(AI135,AJ135,AK135)=0,"",SUM(AI135,AJ135,AK135))</f>
+        <v/>
+      </c>
+      <c r="AM135" s="123">
+        <f>IF(N(AC135)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC135&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC135&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN135" s="124" t="n"/>
+      <c r="AO135" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP135" s="129" t="n"/>
+      <c r="AQ135" s="129" t="n"/>
+      <c r="AR135" s="129" t="n"/>
+      <c r="AS135" s="129" t="n"/>
+      <c r="AT135" s="129" t="n"/>
+      <c r="AU135" s="129" t="n"/>
+      <c r="AV135" s="130" t="inlineStr">
+        <is>
+          <t>Quiz / test yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="123" t="n">
+        <v>131</v>
+      </c>
+      <c r="B136" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Presence &amp; influence rules</t>
+        </is>
+      </c>
+      <c r="C136" s="123" t="inlineStr">
+        <is>
+          <t>Why lower voices sound like leaders</t>
+        </is>
+      </c>
+      <c r="D136" s="123" t="inlineStr">
+        <is>
+          <t>People pick leaders by VOICE more than you think.</t>
+        </is>
+      </c>
+      <c r="E136" s="123" t="inlineStr">
+        <is>
+          <t>Klofstad, Anderson &amp; Peters 2012</t>
+        </is>
+      </c>
+      <c r="F136" s="123" t="n"/>
+      <c r="G136" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H136" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I136" s="124" t="n">
+        <v>29</v>
+      </c>
+      <c r="J136" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K136" s="124" t="inlineStr">
+        <is>
+          <t>lower-voice</t>
+        </is>
+      </c>
+      <c r="L136" s="125" t="n"/>
+      <c r="M136" s="123">
+        <f>IF(L136="","",TEXT(L136,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N136" s="124" t="n"/>
+      <c r="O136" s="124" t="n"/>
+      <c r="P136" s="124" t="n"/>
+      <c r="Q136" s="124" t="n"/>
+      <c r="R136" s="124" t="n"/>
+      <c r="S136" s="126" t="n"/>
+      <c r="T136" s="124" t="n"/>
+      <c r="U136" s="127">
+        <f>IF(OR(T136="",N(O136)=0),"",T136/O136)</f>
+        <v/>
+      </c>
+      <c r="V136" s="124" t="n"/>
+      <c r="W136" s="124" t="n"/>
+      <c r="X136" s="124" t="n"/>
+      <c r="Y136" s="126" t="n"/>
+      <c r="Z136" s="124" t="n"/>
+      <c r="AA136" s="126" t="n"/>
+      <c r="AB136" s="124" t="n"/>
+      <c r="AC136" s="128">
+        <f>IF(COUNT(S136,Y136,AA136)=0,"",SUM(S136,Y136,AA136))</f>
+        <v/>
+      </c>
+      <c r="AD136" s="127">
+        <f>IF(N(AC136)=0,"",SUM(V136,W136,X136,Z136,AB136)/AC136)</f>
+        <v/>
+      </c>
+      <c r="AE136" s="126" t="n"/>
+      <c r="AF136" s="126" t="n"/>
+      <c r="AG136" s="126" t="n"/>
+      <c r="AH136" s="128">
+        <f>IF(COUNT(AE136,AF136,AG136)=0,"",SUM(AE136,AF136,AG136))</f>
+        <v/>
+      </c>
+      <c r="AI136" s="126" t="n"/>
+      <c r="AJ136" s="126" t="n"/>
+      <c r="AK136" s="126" t="n"/>
+      <c r="AL136" s="128">
+        <f>IF(COUNT(AI136,AJ136,AK136)=0,"",SUM(AI136,AJ136,AK136))</f>
+        <v/>
+      </c>
+      <c r="AM136" s="123">
+        <f>IF(N(AC136)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC136&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC136&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN136" s="124" t="n"/>
+      <c r="AO136" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP136" s="129" t="n"/>
+      <c r="AQ136" s="129" t="n"/>
+      <c r="AR136" s="129" t="n"/>
+      <c r="AS136" s="129" t="n"/>
+      <c r="AT136" s="129" t="n"/>
+      <c r="AU136" s="129" t="n"/>
+      <c r="AV136" s="130" t="inlineStr">
+        <is>
+          <t>Presence &amp; influence rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="123" t="n">
+        <v>132</v>
+      </c>
+      <c r="B137" s="123" t="inlineStr">
+        <is>
+          <t>Pattern: Psychology says (15 s loop)</t>
+        </is>
+      </c>
+      <c r="C137" s="123" t="inlineStr">
+        <is>
+          <t>Psychology says: you overvalue what you build (IKEA effect)</t>
+        </is>
+      </c>
+      <c r="D137" s="123" t="inlineStr">
+        <is>
+          <t>Psychology says: you'll pay MORE for something you built yourself.</t>
+        </is>
+      </c>
+      <c r="E137" s="123" t="inlineStr">
+        <is>
+          <t>Norton, Mochon &amp; Ariely 2012</t>
+        </is>
+      </c>
+      <c r="F137" s="123" t="n"/>
+      <c r="G137" s="123" t="n">
+        <v>30</v>
+      </c>
+      <c r="H137" s="123" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="I137" s="124" t="n">
+        <v>30</v>
+      </c>
+      <c r="J137" s="124" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="K137" s="124" t="inlineStr">
+        <is>
+          <t>ikea-effect</t>
+        </is>
+      </c>
+      <c r="L137" s="125" t="n"/>
+      <c r="M137" s="123">
+        <f>IF(L137="","",TEXT(L137,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N137" s="124" t="n"/>
+      <c r="O137" s="124" t="n"/>
+      <c r="P137" s="124" t="n"/>
+      <c r="Q137" s="124" t="n"/>
+      <c r="R137" s="124" t="n"/>
+      <c r="S137" s="126" t="n"/>
+      <c r="T137" s="124" t="n"/>
+      <c r="U137" s="127">
+        <f>IF(OR(T137="",N(O137)=0),"",T137/O137)</f>
+        <v/>
+      </c>
+      <c r="V137" s="124" t="n"/>
+      <c r="W137" s="124" t="n"/>
+      <c r="X137" s="124" t="n"/>
+      <c r="Y137" s="126" t="n"/>
+      <c r="Z137" s="124" t="n"/>
+      <c r="AA137" s="126" t="n"/>
+      <c r="AB137" s="124" t="n"/>
+      <c r="AC137" s="128">
+        <f>IF(COUNT(S137,Y137,AA137)=0,"",SUM(S137,Y137,AA137))</f>
+        <v/>
+      </c>
+      <c r="AD137" s="127">
+        <f>IF(N(AC137)=0,"",SUM(V137,W137,X137,Z137,AB137)/AC137)</f>
+        <v/>
+      </c>
+      <c r="AE137" s="126" t="n"/>
+      <c r="AF137" s="126" t="n"/>
+      <c r="AG137" s="126" t="n"/>
+      <c r="AH137" s="128">
+        <f>IF(COUNT(AE137,AF137,AG137)=0,"",SUM(AE137,AF137,AG137))</f>
+        <v/>
+      </c>
+      <c r="AI137" s="126" t="n"/>
+      <c r="AJ137" s="126" t="n"/>
+      <c r="AK137" s="126" t="n"/>
+      <c r="AL137" s="128">
+        <f>IF(COUNT(AI137,AJ137,AK137)=0,"",SUM(AI137,AJ137,AK137))</f>
+        <v/>
+      </c>
+      <c r="AM137" s="123">
+        <f>IF(N(AC137)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC137&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC137&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN137" s="124" t="n"/>
+      <c r="AO137" s="124" t="inlineStr">
+        <is>
+          <t>ted2</t>
+        </is>
+      </c>
+      <c r="AP137" s="129" t="n"/>
+      <c r="AQ137" s="129" t="n"/>
+      <c r="AR137" s="129" t="n"/>
+      <c r="AS137" s="129" t="n"/>
+      <c r="AT137" s="129" t="n"/>
+      <c r="AU137" s="129" t="n"/>
+      <c r="AV137" s="130" t="inlineStr">
+        <is>
+          <t>Psychology says (15 s loop)</t>
         </is>
       </c>
     </row>
@@ -14264,19 +17938,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="H6:H107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H6:H137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Idea,Researching,Scripted,Scheduled,Published,Vetoed,Failed,Filming,Editing"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="J6:J107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="J6:J137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Strong,Weak"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AO6:AO107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AO6:AO137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>Looks!$A$5:$A$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AP6:AP107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AP6:AP137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"ted2,story"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Pattern scripts day 3: tetris-effect, bat-and-ball, mirroring-tips
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -15246,7 +15246,7 @@
       </c>
       <c r="H114" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I114" s="124" t="n">
@@ -15267,10 +15267,18 @@
         <f>IF(L114="","",TEXT(L114,"ddd"))</f>
         <v/>
       </c>
-      <c r="N114" s="124" t="n"/>
+      <c r="N114" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
       <c r="O114" s="124" t="n"/>
       <c r="P114" s="124" t="n"/>
-      <c r="Q114" s="124" t="n"/>
+      <c r="Q114" s="124" t="inlineStr">
+        <is>
+          <t>Stickgold et al. (2000, Science): after playing Tetris for hours over three days, more than 60% of players (17 of 27) saw falling blocks at sleep onset, including 3 of 5 amnesic patients who couldn't remember playing. The Tetris effect.</t>
+        </is>
+      </c>
       <c r="R114" s="124" t="n"/>
       <c r="S114" s="126" t="n"/>
       <c r="T114" s="124" t="n"/>
@@ -15359,7 +15367,7 @@
       </c>
       <c r="H115" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I115" s="124" t="n">
@@ -15380,10 +15388,18 @@
         <f>IF(L115="","",TEXT(L115,"ddd"))</f>
         <v/>
       </c>
-      <c r="N115" s="124" t="n"/>
+      <c r="N115" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
       <c r="O115" s="124" t="n"/>
       <c r="P115" s="124" t="n"/>
-      <c r="Q115" s="124" t="n"/>
+      <c r="Q115" s="124" t="inlineStr">
+        <is>
+          <t>The bat-and-ball question from Shane Frederick's Cognitive Reflection Test (2005): a bat and a ball cost $1.10 together and the bat costs $1 more than the ball. The intuitive answer (10 cents) is wrong; the ball costs 5 cents. More than half of stude</t>
+        </is>
+      </c>
       <c r="R115" s="124" t="n"/>
       <c r="S115" s="126" t="n"/>
       <c r="T115" s="124" t="n"/>
@@ -15472,7 +15488,7 @@
       </c>
       <c r="H116" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I116" s="124" t="n">
@@ -15493,10 +15509,18 @@
         <f>IF(L116="","",TEXT(L116,"ddd"))</f>
         <v/>
       </c>
-      <c r="N116" s="124" t="n"/>
+      <c r="N116" s="124" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
       <c r="O116" s="124" t="n"/>
       <c r="P116" s="124" t="n"/>
-      <c r="Q116" s="124" t="n"/>
+      <c r="Q116" s="124" t="inlineStr">
+        <is>
+          <t>van Baaren, Holland, Steenaert &amp; van Knippenberg (2003): in a restaurant in the Netherlands, a waitress who repeated customers' orders back word for word received almost twice the tip she got when she only said things like "coming right up". Verbal m</t>
+        </is>
+      </c>
       <c r="R116" s="124" t="n"/>
       <c r="S116" s="126" t="n"/>
       <c r="T116" s="124" t="n"/>

</xml_diff>

<commit_message>
Stick story format: recurring cast (Arjun, Maya, Kabir, Zoe), hand-drawn engine, episode 1 (mind reading)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -1141,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:AV137"/>
+  <dimension ref="A2:AV138"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="61" min="1" max="1"/>
@@ -14907,7 +14907,7 @@
       </c>
       <c r="H111" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I111" s="124" t="n">
@@ -14988,7 +14988,11 @@
         <f>IF(N(AC111)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC111&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC111&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN111" s="124" t="n"/>
+      <c r="AN111" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-24: pulled from Buffer for the stick story format (Shivam)</t>
+        </is>
+      </c>
       <c r="AO111" s="124" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -15036,7 +15040,7 @@
       </c>
       <c r="H112" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I112" s="124" t="n">
@@ -15117,7 +15121,11 @@
         <f>IF(N(AC112)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC112&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC112&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN112" s="124" t="n"/>
+      <c r="AN112" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-24: pulled from Buffer for the stick story format (Shivam)</t>
+        </is>
+      </c>
       <c r="AO112" s="124" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -15165,7 +15173,7 @@
       </c>
       <c r="H113" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I113" s="124" t="n">
@@ -15246,7 +15254,11 @@
         <f>IF(N(AC113)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC113&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC113&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN113" s="124" t="n"/>
+      <c r="AN113" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-24: pulled from Buffer for the stick story format (Shivam)</t>
+        </is>
+      </c>
       <c r="AO113" s="124" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -17999,6 +18011,119 @@
           <t>Psychology says (15 s loop)</t>
         </is>
       </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="123" t="n">
+        <v>133</v>
+      </c>
+      <c r="B138" s="123" t="inlineStr">
+        <is>
+          <t>Character story: Arjun</t>
+        </is>
+      </c>
+      <c r="C138" s="123" t="inlineStr">
+        <is>
+          <t>Arjun ep.1: thinks Kabir is mad at him (mind reading)</t>
+        </is>
+      </c>
+      <c r="D138" s="123" t="inlineStr">
+        <is>
+          <t>Arjun waved at Kabir. Kabir walked right past him.</t>
+        </is>
+      </c>
+      <c r="E138" s="123" t="inlineStr">
+        <is>
+          <t>Mind reading cognitive distortion (Beck; Burns 1980)</t>
+        </is>
+      </c>
+      <c r="F138" s="123" t="n"/>
+      <c r="G138" s="123" t="n">
+        <v>32</v>
+      </c>
+      <c r="H138" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I138" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" s="124" t="n"/>
+      <c r="K138" s="124" t="inlineStr">
+        <is>
+          <t>arjun-mind-reading</t>
+        </is>
+      </c>
+      <c r="L138" s="125" t="n"/>
+      <c r="M138" s="123">
+        <f>IF(L138="","",TEXT(L138,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N138" s="124" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="O138" s="124" t="n"/>
+      <c r="P138" s="124" t="n"/>
+      <c r="Q138" s="124" t="inlineStr">
+        <is>
+          <t>Beck cognitive distortions; Burns, Feeling Good (1980)</t>
+        </is>
+      </c>
+      <c r="R138" s="124" t="n"/>
+      <c r="S138" s="126" t="n"/>
+      <c r="T138" s="124" t="n"/>
+      <c r="U138" s="127">
+        <f>IF(OR(T138="",N(O138)=0),"",T138/O138)</f>
+        <v/>
+      </c>
+      <c r="V138" s="124" t="n"/>
+      <c r="W138" s="124" t="n"/>
+      <c r="X138" s="124" t="n"/>
+      <c r="Y138" s="126" t="n"/>
+      <c r="Z138" s="124" t="n"/>
+      <c r="AA138" s="126" t="n"/>
+      <c r="AB138" s="124" t="n"/>
+      <c r="AC138" s="128">
+        <f>IF(COUNT(S138,Y138,AA138)=0,"",SUM(S138,Y138,AA138))</f>
+        <v/>
+      </c>
+      <c r="AD138" s="127">
+        <f>IF(N(AC138)=0,"",SUM(V138,W138,X138,Z138,AB138)/AC138)</f>
+        <v/>
+      </c>
+      <c r="AE138" s="126" t="n"/>
+      <c r="AF138" s="126" t="n"/>
+      <c r="AG138" s="126" t="n"/>
+      <c r="AH138" s="128">
+        <f>IF(COUNT(AE138,AF138,AG138)=0,"",SUM(AE138,AF138,AG138))</f>
+        <v/>
+      </c>
+      <c r="AI138" s="126" t="n"/>
+      <c r="AJ138" s="126" t="n"/>
+      <c r="AK138" s="126" t="n"/>
+      <c r="AL138" s="128">
+        <f>IF(COUNT(AI138,AJ138,AK138)=0,"",SUM(AI138,AJ138,AK138))</f>
+        <v/>
+      </c>
+      <c r="AM138" s="123">
+        <f>IF(N(AC138)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC138&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC138&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN138" s="124" t="n"/>
+      <c r="AO138" s="124" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP138" s="129" t="n"/>
+      <c r="AQ138" s="129" t="n"/>
+      <c r="AR138" s="129" t="n"/>
+      <c r="AS138" s="129" t="n"/>
+      <c r="AT138" s="129" t="n"/>
+      <c r="AU138" s="129" t="n"/>
+      <c r="AV138" s="130" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="AM6:AM105">
@@ -18010,19 +18135,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="H6:H137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H6:H138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Idea,Researching,Scripted,Scheduled,Published,Vetoed,Failed,Filming,Editing"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="J6:J137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="J6:J138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Strong,Weak"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AO6:AO137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AO6:AO138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>Looks!$A$5:$A$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AP6:AP137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AP6:AP138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"ted2,story"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Stick stories: Zoe ep.1 (foot in the door), Kabir ep.1 (planning fallacy)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1141,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:AV138"/>
+  <dimension ref="A2:AV140"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="61" min="1" max="1"/>
@@ -18125,6 +18125,232 @@
       <c r="AU138" s="129" t="n"/>
       <c r="AV138" s="130" t="n"/>
     </row>
+    <row r="139">
+      <c r="A139" s="123" t="n">
+        <v>134</v>
+      </c>
+      <c r="B139" s="123" t="inlineStr">
+        <is>
+          <t>Character story: Zoe</t>
+        </is>
+      </c>
+      <c r="C139" s="123" t="inlineStr">
+        <is>
+          <t>Zoe ep.1: tiny favor then weekend shift (foot in the door)</t>
+        </is>
+      </c>
+      <c r="D139" s="123" t="inlineStr">
+        <is>
+          <t>Maya asked Zoe for one tiny favor.</t>
+        </is>
+      </c>
+      <c r="E139" s="123" t="inlineStr">
+        <is>
+          <t>Freedman &amp; Fraser 1966 17% vs 76%</t>
+        </is>
+      </c>
+      <c r="F139" s="123" t="n"/>
+      <c r="G139" s="123" t="n">
+        <v>36</v>
+      </c>
+      <c r="H139" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I139" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" s="124" t="n"/>
+      <c r="K139" s="124" t="inlineStr">
+        <is>
+          <t>zoe-tiny-favor</t>
+        </is>
+      </c>
+      <c r="L139" s="125" t="n"/>
+      <c r="M139" s="123">
+        <f>IF(L139="","",TEXT(L139,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N139" s="124" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="O139" s="124" t="n"/>
+      <c r="P139" s="124" t="n"/>
+      <c r="Q139" s="124" t="inlineStr">
+        <is>
+          <t>Freedman &amp; Fraser (1966) JPSP: 17% vs 76%</t>
+        </is>
+      </c>
+      <c r="R139" s="124" t="n"/>
+      <c r="S139" s="126" t="n"/>
+      <c r="T139" s="124" t="n"/>
+      <c r="U139" s="127">
+        <f>IF(OR(T139="",N(O139)=0),"",T139/O139)</f>
+        <v/>
+      </c>
+      <c r="V139" s="124" t="n"/>
+      <c r="W139" s="124" t="n"/>
+      <c r="X139" s="124" t="n"/>
+      <c r="Y139" s="126" t="n"/>
+      <c r="Z139" s="124" t="n"/>
+      <c r="AA139" s="126" t="n"/>
+      <c r="AB139" s="124" t="n"/>
+      <c r="AC139" s="128">
+        <f>IF(COUNT(S139,Y139,AA139)=0,"",SUM(S139,Y139,AA139))</f>
+        <v/>
+      </c>
+      <c r="AD139" s="127">
+        <f>IF(N(AC139)=0,"",SUM(V139,W139,X139,Z139,AB139)/AC139)</f>
+        <v/>
+      </c>
+      <c r="AE139" s="126" t="n"/>
+      <c r="AF139" s="126" t="n"/>
+      <c r="AG139" s="126" t="n"/>
+      <c r="AH139" s="128">
+        <f>IF(COUNT(AE139,AF139,AG139)=0,"",SUM(AE139,AF139,AG139))</f>
+        <v/>
+      </c>
+      <c r="AI139" s="126" t="n"/>
+      <c r="AJ139" s="126" t="n"/>
+      <c r="AK139" s="126" t="n"/>
+      <c r="AL139" s="128">
+        <f>IF(COUNT(AI139,AJ139,AK139)=0,"",SUM(AI139,AJ139,AK139))</f>
+        <v/>
+      </c>
+      <c r="AM139" s="123">
+        <f>IF(N(AC139)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC139&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC139&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN139" s="124" t="n"/>
+      <c r="AO139" s="124" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP139" s="129" t="n"/>
+      <c r="AQ139" s="129" t="n"/>
+      <c r="AR139" s="129" t="n"/>
+      <c r="AS139" s="129" t="n"/>
+      <c r="AT139" s="129" t="n"/>
+      <c r="AU139" s="129" t="n"/>
+      <c r="AV139" s="130" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="123" t="n">
+        <v>135</v>
+      </c>
+      <c r="B140" s="123" t="inlineStr">
+        <is>
+          <t>Character story: Kabir</t>
+        </is>
+      </c>
+      <c r="C140" s="123" t="inlineStr">
+        <is>
+          <t>Kabir ep.1: two days, tops (planning fallacy)</t>
+        </is>
+      </c>
+      <c r="D140" s="123" t="inlineStr">
+        <is>
+          <t>Kabir had a whole week for his essay.</t>
+        </is>
+      </c>
+      <c r="E140" s="123" t="inlineStr">
+        <is>
+          <t>Buehler, Griffin &amp; Ross 1994: 33.9 / 55.5 days, ~30%</t>
+        </is>
+      </c>
+      <c r="F140" s="123" t="n"/>
+      <c r="G140" s="123" t="n">
+        <v>34</v>
+      </c>
+      <c r="H140" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I140" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" s="124" t="n"/>
+      <c r="K140" s="124" t="inlineStr">
+        <is>
+          <t>kabir-two-days</t>
+        </is>
+      </c>
+      <c r="L140" s="125" t="n"/>
+      <c r="M140" s="123">
+        <f>IF(L140="","",TEXT(L140,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N140" s="124" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="O140" s="124" t="n"/>
+      <c r="P140" s="124" t="n"/>
+      <c r="Q140" s="124" t="inlineStr">
+        <is>
+          <t>Buehler, Griffin &amp; Ross (1994) JPSP: 33.9 predicted, 55.5 actual, ~30% on time</t>
+        </is>
+      </c>
+      <c r="R140" s="124" t="n"/>
+      <c r="S140" s="126" t="n"/>
+      <c r="T140" s="124" t="n"/>
+      <c r="U140" s="127">
+        <f>IF(OR(T140="",N(O140)=0),"",T140/O140)</f>
+        <v/>
+      </c>
+      <c r="V140" s="124" t="n"/>
+      <c r="W140" s="124" t="n"/>
+      <c r="X140" s="124" t="n"/>
+      <c r="Y140" s="126" t="n"/>
+      <c r="Z140" s="124" t="n"/>
+      <c r="AA140" s="126" t="n"/>
+      <c r="AB140" s="124" t="n"/>
+      <c r="AC140" s="128">
+        <f>IF(COUNT(S140,Y140,AA140)=0,"",SUM(S140,Y140,AA140))</f>
+        <v/>
+      </c>
+      <c r="AD140" s="127">
+        <f>IF(N(AC140)=0,"",SUM(V140,W140,X140,Z140,AB140)/AC140)</f>
+        <v/>
+      </c>
+      <c r="AE140" s="126" t="n"/>
+      <c r="AF140" s="126" t="n"/>
+      <c r="AG140" s="126" t="n"/>
+      <c r="AH140" s="128">
+        <f>IF(COUNT(AE140,AF140,AG140)=0,"",SUM(AE140,AF140,AG140))</f>
+        <v/>
+      </c>
+      <c r="AI140" s="126" t="n"/>
+      <c r="AJ140" s="126" t="n"/>
+      <c r="AK140" s="126" t="n"/>
+      <c r="AL140" s="128">
+        <f>IF(COUNT(AI140,AJ140,AK140)=0,"",SUM(AI140,AJ140,AK140))</f>
+        <v/>
+      </c>
+      <c r="AM140" s="123">
+        <f>IF(N(AC140)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC140&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC140&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN140" s="124" t="n"/>
+      <c r="AO140" s="124" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP140" s="129" t="n"/>
+      <c r="AQ140" s="129" t="n"/>
+      <c r="AR140" s="129" t="n"/>
+      <c r="AS140" s="129" t="n"/>
+      <c r="AT140" s="129" t="n"/>
+      <c r="AU140" s="129" t="n"/>
+      <c r="AV140" s="130" t="n"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="AM6:AM105">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="4" text="" percent="0" bottom="0">
@@ -18135,19 +18361,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="H6:H138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H6:H140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Idea,Researching,Scripted,Scheduled,Published,Vetoed,Failed,Filming,Editing"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="J6:J138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="J6:J140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Strong,Weak"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AO6:AO138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AO6:AO140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>Looks!$A$5:$A$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AP6:AP138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AP6:AP140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"ted2,story"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
runbook: stick character stories replace explainers; shelve unbuilt explainer scripts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nL4Az71PnVXhG3KH2Utv3
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -15306,7 +15306,7 @@
       </c>
       <c r="H114" s="123" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Idea</t>
         </is>
       </c>
       <c r="I114" s="124" t="n">
@@ -15379,7 +15379,11 @@
         <f>IF(N(AC114)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC114&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC114&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN114" s="124" t="n"/>
+      <c r="AN114" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-25: explainer script shelved; rewrite as a stick character story (Shivam)</t>
+        </is>
+      </c>
       <c r="AO114" s="124" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -15427,7 +15431,7 @@
       </c>
       <c r="H115" s="123" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Idea</t>
         </is>
       </c>
       <c r="I115" s="124" t="n">
@@ -15500,7 +15504,11 @@
         <f>IF(N(AC115)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC115&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC115&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN115" s="124" t="n"/>
+      <c r="AN115" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-25: explainer script shelved; rewrite as a stick character story (Shivam)</t>
+        </is>
+      </c>
       <c r="AO115" s="124" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -15548,7 +15556,7 @@
       </c>
       <c r="H116" s="123" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Idea</t>
         </is>
       </c>
       <c r="I116" s="124" t="n">
@@ -15621,7 +15629,11 @@
         <f>IF(N(AC116)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC116&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC116&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN116" s="124" t="n"/>
+      <c r="AN116" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-25: explainer script shelved; rewrite as a stick character story (Shivam)</t>
+        </is>
+      </c>
       <c r="AO116" s="124" t="inlineStr">
         <is>
           <t>ted2</t>

</xml_diff>

<commit_message>
Scripts: 6 stick character stories (Kabir ep2-3, Maya ep1-2, Zoe ep2, Arjun ep2); tracker rows 109-114 Scripted; cast history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ly87qoiJRpDzuYuM4ZHG5r
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -15306,7 +15306,7 @@
       </c>
       <c r="H114" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I114" s="124" t="n">
@@ -15319,7 +15319,7 @@
       </c>
       <c r="K114" s="124" t="inlineStr">
         <is>
-          <t>tetris-effect</t>
+          <t>kabir-tetris-dreams</t>
         </is>
       </c>
       <c r="L114" s="125" t="n"/>
@@ -15329,14 +15329,14 @@
       </c>
       <c r="N114" s="124" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>story</t>
         </is>
       </c>
       <c r="O114" s="124" t="n"/>
       <c r="P114" s="124" t="n"/>
       <c r="Q114" s="124" t="inlineStr">
         <is>
-          <t>Stickgold et al. (2000, Science): after playing Tetris for hours over three days, more than 60% of players (17 of 27) saw falling blocks at sleep onset, including 3 of 5 amnesic patients who couldn't remember playing. The Tetris effect.</t>
+          <t>Stickgold et al. (2000, Science): after hours of Tetris over three days, 17 of 27 players reported Tetris images at sleep onset, incl. 3 of 5 amnesic patients who couldn't remember playing (Harvard Gazette 2000). Retold as stick story (Kabir ep. 2).</t>
         </is>
       </c>
       <c r="R114" s="124" t="n"/>
@@ -15386,10 +15386,14 @@
       </c>
       <c r="AO114" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
-        </is>
-      </c>
-      <c r="AP114" s="129" t="n"/>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP114" s="129" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
       <c r="AQ114" s="129" t="n"/>
       <c r="AR114" s="129" t="n"/>
       <c r="AS114" s="129" t="n"/>
@@ -15431,7 +15435,7 @@
       </c>
       <c r="H115" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I115" s="124" t="n">
@@ -15444,7 +15448,7 @@
       </c>
       <c r="K115" s="124" t="inlineStr">
         <is>
-          <t>bat-and-ball</t>
+          <t>maya-bat-and-ball</t>
         </is>
       </c>
       <c r="L115" s="125" t="n"/>
@@ -15454,14 +15458,14 @@
       </c>
       <c r="N115" s="124" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>story</t>
         </is>
       </c>
       <c r="O115" s="124" t="n"/>
       <c r="P115" s="124" t="n"/>
       <c r="Q115" s="124" t="inlineStr">
         <is>
-          <t>The bat-and-ball question from Shane Frederick's Cognitive Reflection Test (2005): a bat and a ball cost $1.10 together and the bat costs $1 more than the ball. The intuitive answer (10 cents) is wrong; the ball costs 5 cents. More than half of stude</t>
+          <t>Frederick (2005, J. Econ. Perspectives), Cognitive Reflection Test: about half of students at Harvard, MIT and Princeton gave the intuitive 10-cent answer (correct: 5 cents). Retold as stick story (Maya ep. 1).</t>
         </is>
       </c>
       <c r="R115" s="124" t="n"/>
@@ -15511,10 +15515,14 @@
       </c>
       <c r="AO115" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
-        </is>
-      </c>
-      <c r="AP115" s="129" t="n"/>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP115" s="129" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
       <c r="AQ115" s="129" t="n"/>
       <c r="AR115" s="129" t="n"/>
       <c r="AS115" s="129" t="n"/>
@@ -15556,7 +15564,7 @@
       </c>
       <c r="H116" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I116" s="124" t="n">
@@ -15569,7 +15577,7 @@
       </c>
       <c r="K116" s="124" t="inlineStr">
         <is>
-          <t>mirroring-tips</t>
+          <t>zoe-repeat-order</t>
         </is>
       </c>
       <c r="L116" s="125" t="n"/>
@@ -15579,14 +15587,14 @@
       </c>
       <c r="N116" s="124" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>story</t>
         </is>
       </c>
       <c r="O116" s="124" t="n"/>
       <c r="P116" s="124" t="n"/>
       <c r="Q116" s="124" t="inlineStr">
         <is>
-          <t>van Baaren, Holland, Steenaert &amp; van Knippenberg (2003): in a restaurant in the Netherlands, a waitress who repeated customers' orders back word for word received almost twice the tip she got when she only said things like "coming right up". Verbal m</t>
+          <t>van Baaren, Holland, Steenaert &amp; van Knippenberg (2003): a Dutch waitress who repeated orders verbatim got almost twice the tips (~3 guilders) vs not mimicking. Retold as stick story (Zoe ep. 2).</t>
         </is>
       </c>
       <c r="R116" s="124" t="n"/>
@@ -15636,10 +15644,14 @@
       </c>
       <c r="AO116" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
-        </is>
-      </c>
-      <c r="AP116" s="129" t="n"/>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP116" s="129" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
       <c r="AQ116" s="129" t="n"/>
       <c r="AR116" s="129" t="n"/>
       <c r="AS116" s="129" t="n"/>
@@ -15681,7 +15693,7 @@
       </c>
       <c r="H117" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I117" s="124" t="n">
@@ -15694,7 +15706,7 @@
       </c>
       <c r="K117" s="124" t="inlineStr">
         <is>
-          <t>ben-franklin-effect</t>
+          <t>arjun-borrow-notes</t>
         </is>
       </c>
       <c r="L117" s="125" t="n"/>
@@ -15702,10 +15714,18 @@
         <f>IF(L117="","",TEXT(L117,"ddd"))</f>
         <v/>
       </c>
-      <c r="N117" s="124" t="n"/>
+      <c r="N117" s="124" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
       <c r="O117" s="124" t="n"/>
       <c r="P117" s="124" t="n"/>
-      <c r="Q117" s="124" t="n"/>
+      <c r="Q117" s="124" t="inlineStr">
+        <is>
+          <t>Jecker &amp; Landy (1969, Human Relations): participants asked by the experimenter to return their winnings as a personal favor liked him more than those not asked (Ben Franklin effect). Retold as stick story (Arjun ep. 2).</t>
+        </is>
+      </c>
       <c r="R117" s="124" t="n"/>
       <c r="S117" s="126" t="n"/>
       <c r="T117" s="124" t="n"/>
@@ -15749,10 +15769,14 @@
       <c r="AN117" s="124" t="n"/>
       <c r="AO117" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
-        </is>
-      </c>
-      <c r="AP117" s="129" t="n"/>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP117" s="129" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
       <c r="AQ117" s="129" t="n"/>
       <c r="AR117" s="129" t="n"/>
       <c r="AS117" s="129" t="n"/>
@@ -15794,7 +15818,7 @@
       </c>
       <c r="H118" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I118" s="124" t="n">
@@ -15807,7 +15831,7 @@
       </c>
       <c r="K118" s="124" t="inlineStr">
         <is>
-          <t>good-samaritan-hurry</t>
+          <t>kabir-late-samaritan</t>
         </is>
       </c>
       <c r="L118" s="125" t="n"/>
@@ -15815,10 +15839,18 @@
         <f>IF(L118="","",TEXT(L118,"ddd"))</f>
         <v/>
       </c>
-      <c r="N118" s="124" t="n"/>
+      <c r="N118" s="124" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
       <c r="O118" s="124" t="n"/>
       <c r="P118" s="124" t="n"/>
-      <c r="Q118" s="124" t="n"/>
+      <c r="Q118" s="124" t="inlineStr">
+        <is>
+          <t>Darley &amp; Batson (1973, JPSP): seminary students going to give a talk (some on the Good Samaritan) passed a slumped man; 63% helped with no hurry, 45% intermediate, 10% high hurry. Retold as stick story (Kabir ep. 3).</t>
+        </is>
+      </c>
       <c r="R118" s="124" t="n"/>
       <c r="S118" s="126" t="n"/>
       <c r="T118" s="124" t="n"/>
@@ -15862,10 +15894,14 @@
       <c r="AN118" s="124" t="n"/>
       <c r="AO118" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
-        </is>
-      </c>
-      <c r="AP118" s="129" t="n"/>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP118" s="129" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
       <c r="AQ118" s="129" t="n"/>
       <c r="AR118" s="129" t="n"/>
       <c r="AS118" s="129" t="n"/>
@@ -15907,7 +15943,7 @@
       </c>
       <c r="H119" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I119" s="124" t="n">
@@ -15920,7 +15956,7 @@
       </c>
       <c r="K119" s="124" t="inlineStr">
         <is>
-          <t>door-in-the-face</t>
+          <t>maya-big-ask</t>
         </is>
       </c>
       <c r="L119" s="125" t="n"/>
@@ -15928,10 +15964,18 @@
         <f>IF(L119="","",TEXT(L119,"ddd"))</f>
         <v/>
       </c>
-      <c r="N119" s="124" t="n"/>
+      <c r="N119" s="124" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
       <c r="O119" s="124" t="n"/>
       <c r="P119" s="124" t="n"/>
-      <c r="Q119" s="124" t="n"/>
+      <c r="Q119" s="124" t="inlineStr">
+        <is>
+          <t>Cialdini et al. (1975, JPSP): 17% agreed to chaperone juvenile delinquents on a zoo trip; 50% after first refusing 2 hrs/week for 2 years as counselors (25% when large request only described). Retold as stick story (Maya ep. 2).</t>
+        </is>
+      </c>
       <c r="R119" s="124" t="n"/>
       <c r="S119" s="126" t="n"/>
       <c r="T119" s="124" t="n"/>
@@ -15975,10 +16019,14 @@
       <c r="AN119" s="124" t="n"/>
       <c r="AO119" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
-        </is>
-      </c>
-      <c r="AP119" s="129" t="n"/>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="AP119" s="129" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
       <c r="AQ119" s="129" t="n"/>
       <c r="AR119" s="129" t="n"/>
       <c r="AS119" s="129" t="n"/>

</xml_diff>

<commit_message>
Tracker: leave Format empty on stick rows (as rows 133-135)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ly87qoiJRpDzuYuM4ZHG5r
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -15389,11 +15389,7 @@
           <t>stick</t>
         </is>
       </c>
-      <c r="AP114" s="129" t="inlineStr">
-        <is>
-          <t>stick</t>
-        </is>
-      </c>
+      <c r="AP114" s="129" t="n"/>
       <c r="AQ114" s="129" t="n"/>
       <c r="AR114" s="129" t="n"/>
       <c r="AS114" s="129" t="n"/>
@@ -15518,11 +15514,7 @@
           <t>stick</t>
         </is>
       </c>
-      <c r="AP115" s="129" t="inlineStr">
-        <is>
-          <t>stick</t>
-        </is>
-      </c>
+      <c r="AP115" s="129" t="n"/>
       <c r="AQ115" s="129" t="n"/>
       <c r="AR115" s="129" t="n"/>
       <c r="AS115" s="129" t="n"/>
@@ -15647,11 +15639,7 @@
           <t>stick</t>
         </is>
       </c>
-      <c r="AP116" s="129" t="inlineStr">
-        <is>
-          <t>stick</t>
-        </is>
-      </c>
+      <c r="AP116" s="129" t="n"/>
       <c r="AQ116" s="129" t="n"/>
       <c r="AR116" s="129" t="n"/>
       <c r="AS116" s="129" t="n"/>
@@ -15772,11 +15760,7 @@
           <t>stick</t>
         </is>
       </c>
-      <c r="AP117" s="129" t="inlineStr">
-        <is>
-          <t>stick</t>
-        </is>
-      </c>
+      <c r="AP117" s="129" t="n"/>
       <c r="AQ117" s="129" t="n"/>
       <c r="AR117" s="129" t="n"/>
       <c r="AS117" s="129" t="n"/>
@@ -15897,11 +15881,7 @@
           <t>stick</t>
         </is>
       </c>
-      <c r="AP118" s="129" t="inlineStr">
-        <is>
-          <t>stick</t>
-        </is>
-      </c>
+      <c r="AP118" s="129" t="n"/>
       <c r="AQ118" s="129" t="n"/>
       <c r="AR118" s="129" t="n"/>
       <c r="AS118" s="129" t="n"/>
@@ -16022,11 +16002,7 @@
           <t>stick</t>
         </is>
       </c>
-      <c r="AP119" s="129" t="inlineStr">
-        <is>
-          <t>stick</t>
-        </is>
-      </c>
+      <c r="AP119" s="129" t="n"/>
       <c r="AQ119" s="129" t="n"/>
       <c r="AR119" s="129" t="n"/>
       <c r="AS119" s="129" t="n"/>

</xml_diff>

<commit_message>
Weekly review 2026-10-25: Buffer stats, d7 fill, rows 103-105 Published
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TbCS67kjez9kVA5MBtqEZS
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1609,7 +1609,9 @@
         <f>IF(N(AC6)=0,"",SUM(V6,W6,X6,Z6,AB6)/AC6)</f>
         <v/>
       </c>
-      <c r="AE6" s="71" t="n"/>
+      <c r="AE6" s="71" t="n">
+        <v>14</v>
+      </c>
       <c r="AF6" s="71" t="n"/>
       <c r="AG6" s="71" t="n"/>
       <c r="AH6" s="73">
@@ -1629,7 +1631,7 @@
       </c>
       <c r="AN6" s="69" t="inlineStr">
         <is>
-          <t>Pilot: 16:9 horizontal, YouTube only — not comparable with the vertical Shorts. 2026-10-18 review: d7 stats not available (Metricool per-video YouTube data empty).</t>
+          <t>Pilot: 16:9 horizontal, YouTube only — not comparable with the vertical Shorts. 2026-10-18 review: d7 stats not available (Metricool per-video YouTube data empty). 2026-10-25 review: d14 from Buffer at age 14 d: YT 14.</t>
         </is>
       </c>
       <c r="AO6" s="69" t="inlineStr">
@@ -1866,19 +1868,33 @@
           <t>buffer:youtube=6ad14adb2b2233d4661582ae;tiktok=6ad14adc5533140b41cadc37;instagram=6ad5279e769b457934da2d97</t>
         </is>
       </c>
-      <c r="S8" s="71" t="n"/>
+      <c r="S8" s="71" t="n">
+        <v>538</v>
+      </c>
       <c r="T8" s="69" t="n"/>
       <c r="U8" s="72">
         <f>IF(OR(T8="",N(O8)=0),"",T8/O8)</f>
         <v/>
       </c>
-      <c r="V8" s="69" t="n"/>
-      <c r="W8" s="69" t="n"/>
+      <c r="V8" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="W8" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X8" s="69" t="n"/>
-      <c r="Y8" s="71" t="n"/>
-      <c r="Z8" s="69" t="n"/>
-      <c r="AA8" s="71" t="n"/>
-      <c r="AB8" s="69" t="n"/>
+      <c r="Y8" s="71" t="n">
+        <v>1342</v>
+      </c>
+      <c r="Z8" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA8" s="71" t="n">
+        <v>83</v>
+      </c>
+      <c r="AB8" s="69" t="n">
+        <v>7</v>
+      </c>
       <c r="AC8" s="73">
         <f>IF(COUNT(S8,Y8,AA8)=0,"",SUM(S8,Y8,AA8))</f>
         <v/>
@@ -1905,7 +1921,11 @@
         <f>IF(N(AC8)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC8&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC8&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN8" s="69" t="n"/>
+      <c r="AN8" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 10 d: YT 538 · IG 1342 (34% ret) · TT 83 (17% ret).</t>
+        </is>
+      </c>
       <c r="AO8" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -2926,19 +2946,33 @@
           <t>3390233992092010605</t>
         </is>
       </c>
-      <c r="S16" s="71" t="n"/>
+      <c r="S16" s="71" t="n">
+        <v>175</v>
+      </c>
       <c r="T16" s="69" t="n"/>
       <c r="U16" s="72">
         <f>IF(OR(T16="",N(O16)=0),"",T16/O16)</f>
         <v/>
       </c>
-      <c r="V16" s="69" t="n"/>
-      <c r="W16" s="69" t="n"/>
+      <c r="V16" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="W16" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X16" s="69" t="n"/>
-      <c r="Y16" s="71" t="n"/>
-      <c r="Z16" s="69" t="n"/>
-      <c r="AA16" s="71" t="n"/>
-      <c r="AB16" s="69" t="n"/>
+      <c r="Y16" s="71" t="n">
+        <v>33</v>
+      </c>
+      <c r="Z16" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="71" t="n">
+        <v>155</v>
+      </c>
+      <c r="AB16" s="69" t="n">
+        <v>7</v>
+      </c>
       <c r="AC16" s="73">
         <f>IF(COUNT(S16,Y16,AA16)=0,"",SUM(S16,Y16,AA16))</f>
         <v/>
@@ -2967,7 +3001,7 @@
       </c>
       <c r="AN16" s="69" t="inlineStr">
         <is>
-          <t>Metricool confirms published 2026-10-12 on YouTube, Instagram and TikTok (Status still Scheduled; left for the workflow/Shivam). Per-video stats not in Metricool yet.</t>
+          <t>Metricool confirms published 2026-10-12 on YouTube, Instagram and TikTok (Status still Scheduled; left for the workflow/Shivam). Per-video stats not in Metricool yet. 2026-10-25 review: d7 from Buffer at age 13 d: YT 175 · IG 33 (20% ret) · TT 155 (47% ret).</t>
         </is>
       </c>
       <c r="AO16" s="69" t="inlineStr">
@@ -3204,19 +3238,29 @@
           <t>buffer:youtube=6ad27dfc346e510ac44f4f11;tiktok=6ad27dfd5720e82b418e1add;instagram=6addab04bd33ce99c35d20e4</t>
         </is>
       </c>
-      <c r="S18" s="71" t="n"/>
+      <c r="S18" s="71" t="n">
+        <v>944</v>
+      </c>
       <c r="T18" s="69" t="n"/>
       <c r="U18" s="72">
         <f>IF(OR(T18="",N(O18)=0),"",T18/O18)</f>
         <v/>
       </c>
-      <c r="V18" s="69" t="n"/>
-      <c r="W18" s="69" t="n"/>
+      <c r="V18" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="W18" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X18" s="69" t="n"/>
       <c r="Y18" s="71" t="n"/>
       <c r="Z18" s="69" t="n"/>
-      <c r="AA18" s="71" t="n"/>
-      <c r="AB18" s="69" t="n"/>
+      <c r="AA18" s="71" t="n">
+        <v>49</v>
+      </c>
+      <c r="AB18" s="69" t="n">
+        <v>4</v>
+      </c>
       <c r="AC18" s="73">
         <f>IF(COUNT(S18,Y18,AA18)=0,"",SUM(S18,Y18,AA18))</f>
         <v/>
@@ -3243,7 +3287,11 @@
         <f>IF(N(AC18)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC18&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC18&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN18" s="69" t="n"/>
+      <c r="AN18" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 8 d: YT 944 · TT 49 (14% ret).</t>
+        </is>
+      </c>
       <c r="AO18" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -4405,19 +4453,29 @@
           <t>-7020071267758420690</t>
         </is>
       </c>
-      <c r="S27" s="71" t="n"/>
+      <c r="S27" s="71" t="n">
+        <v>11</v>
+      </c>
       <c r="T27" s="69" t="n"/>
       <c r="U27" s="72">
         <f>IF(OR(T27="",N(O27)=0),"",T27/O27)</f>
         <v/>
       </c>
-      <c r="V27" s="69" t="n"/>
-      <c r="W27" s="69" t="n"/>
+      <c r="V27" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="W27" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X27" s="69" t="n"/>
       <c r="Y27" s="71" t="n"/>
       <c r="Z27" s="69" t="n"/>
-      <c r="AA27" s="71" t="n"/>
-      <c r="AB27" s="69" t="n"/>
+      <c r="AA27" s="71" t="n">
+        <v>283</v>
+      </c>
+      <c r="AB27" s="69" t="n">
+        <v>5</v>
+      </c>
       <c r="AC27" s="73">
         <f>IF(COUNT(S27,Y27,AA27)=0,"",SUM(S27,Y27,AA27))</f>
         <v/>
@@ -4446,7 +4504,7 @@
       </c>
       <c r="AN27" s="69" t="inlineStr">
         <is>
-          <t>Metricool: published 2026-10-13 on YouTube + TikTok; Instagram ERROR (Unknown). Status still Scheduled. Per-video stats not in Metricool yet.</t>
+          <t>Metricool: published 2026-10-13 on YouTube + TikTok; Instagram ERROR (Unknown). Status still Scheduled. Per-video stats not in Metricool yet. 2026-10-25 review: d7 from Buffer at age 12 d: YT 11 · TT 283 (15% ret).</t>
         </is>
       </c>
       <c r="AO27" s="69" t="inlineStr">
@@ -4836,19 +4894,29 @@
           <t>buffer:youtube=6ad27dfe5720e82b418e1b51;tiktok=6ad27dfe346e510ac44f4f9b</t>
         </is>
       </c>
-      <c r="S30" s="71" t="n"/>
+      <c r="S30" s="71" t="n">
+        <v>1056</v>
+      </c>
       <c r="T30" s="69" t="n"/>
       <c r="U30" s="72">
         <f>IF(OR(T30="",N(O30)=0),"",T30/O30)</f>
         <v/>
       </c>
-      <c r="V30" s="69" t="n"/>
-      <c r="W30" s="69" t="n"/>
+      <c r="V30" s="69" t="n">
+        <v>27</v>
+      </c>
+      <c r="W30" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X30" s="69" t="n"/>
       <c r="Y30" s="71" t="n"/>
       <c r="Z30" s="69" t="n"/>
-      <c r="AA30" s="71" t="n"/>
-      <c r="AB30" s="69" t="n"/>
+      <c r="AA30" s="71" t="n">
+        <v>61</v>
+      </c>
+      <c r="AB30" s="69" t="n">
+        <v>10</v>
+      </c>
       <c r="AC30" s="73">
         <f>IF(COUNT(S30,Y30,AA30)=0,"",SUM(S30,Y30,AA30))</f>
         <v/>
@@ -4875,7 +4943,11 @@
         <f>IF(N(AC30)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC30&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC30&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN30" s="69" t="n"/>
+      <c r="AN30" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 8 d: YT 1056 · TT 61 (26% ret).</t>
+        </is>
+      </c>
       <c r="AO30" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -5707,19 +5779,33 @@
           <t>buffer:youtube=6ace86df1bdf729a2aa960ff;instagram=6ace86df4a3bafcd13007dde;tiktok=6ace86dfeaea728d3cae7f6c</t>
         </is>
       </c>
-      <c r="S37" s="71" t="n"/>
+      <c r="S37" s="71" t="n">
+        <v>12</v>
+      </c>
       <c r="T37" s="69" t="n"/>
       <c r="U37" s="72">
         <f>IF(OR(T37="",N(O37)=0),"",T37/O37)</f>
         <v/>
       </c>
-      <c r="V37" s="69" t="n"/>
-      <c r="W37" s="69" t="n"/>
+      <c r="V37" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X37" s="69" t="n"/>
-      <c r="Y37" s="71" t="n"/>
-      <c r="Z37" s="69" t="n"/>
-      <c r="AA37" s="71" t="n"/>
-      <c r="AB37" s="69" t="n"/>
+      <c r="Y37" s="71" t="n">
+        <v>11</v>
+      </c>
+      <c r="Z37" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="71" t="n">
+        <v>38</v>
+      </c>
+      <c r="AB37" s="69" t="n">
+        <v>1</v>
+      </c>
       <c r="AC37" s="73">
         <f>IF(COUNT(S37,Y37,AA37)=0,"",SUM(S37,Y37,AA37))</f>
         <v/>
@@ -5746,7 +5832,11 @@
         <f>IF(N(AC37)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC37&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC37&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN37" s="69" t="n"/>
+      <c r="AN37" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 11 d: YT 12 · IG 11 (15% ret) · TT 38 (18% ret).</t>
+        </is>
+      </c>
       <c r="AO37" s="69" t="inlineStr">
         <is>
           <t>whiteboard</t>
@@ -6074,19 +6164,33 @@
           <t>buffer:youtube=6ad131005063ce0336b55163;tiktok=6ad13101b4510d553d75dea0;instagram=6ad6884346c9e2453ba0b2bf</t>
         </is>
       </c>
-      <c r="S40" s="71" t="n"/>
+      <c r="S40" s="71" t="n">
+        <v>189</v>
+      </c>
       <c r="T40" s="69" t="n"/>
       <c r="U40" s="72">
         <f>IF(OR(T40="",N(O40)=0),"",T40/O40)</f>
         <v/>
       </c>
-      <c r="V40" s="69" t="n"/>
-      <c r="W40" s="69" t="n"/>
+      <c r="V40" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="W40" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X40" s="69" t="n"/>
-      <c r="Y40" s="71" t="n"/>
-      <c r="Z40" s="69" t="n"/>
-      <c r="AA40" s="71" t="n"/>
-      <c r="AB40" s="69" t="n"/>
+      <c r="Y40" s="71" t="n">
+        <v>140</v>
+      </c>
+      <c r="Z40" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA40" s="71" t="n">
+        <v>40</v>
+      </c>
+      <c r="AB40" s="69" t="n">
+        <v>2</v>
+      </c>
       <c r="AC40" s="73">
         <f>IF(COUNT(S40,Y40,AA40)=0,"",SUM(S40,Y40,AA40))</f>
         <v/>
@@ -6113,7 +6217,11 @@
         <f>IF(N(AC40)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC40&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC40&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN40" s="69" t="n"/>
+      <c r="AN40" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 9 d: YT 189 · IG 140 (13% ret) · TT 40 (11% ret).</t>
+        </is>
+      </c>
       <c r="AO40" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -6207,19 +6315,29 @@
           <t>buffer:youtube=6ad27e00346e510ac44f4fd1;tiktok=6ad27e005720e82b418e1bb9</t>
         </is>
       </c>
-      <c r="S41" s="71" t="n"/>
+      <c r="S41" s="71" t="n">
+        <v>261</v>
+      </c>
       <c r="T41" s="69" t="n"/>
       <c r="U41" s="72">
         <f>IF(OR(T41="",N(O41)=0),"",T41/O41)</f>
         <v/>
       </c>
-      <c r="V41" s="69" t="n"/>
-      <c r="W41" s="69" t="n"/>
+      <c r="V41" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="W41" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X41" s="69" t="n"/>
       <c r="Y41" s="71" t="n"/>
       <c r="Z41" s="69" t="n"/>
-      <c r="AA41" s="71" t="n"/>
-      <c r="AB41" s="69" t="n"/>
+      <c r="AA41" s="71" t="n">
+        <v>62</v>
+      </c>
+      <c r="AB41" s="69" t="n">
+        <v>18</v>
+      </c>
       <c r="AC41" s="73">
         <f>IF(COUNT(S41,Y41,AA41)=0,"",SUM(S41,Y41,AA41))</f>
         <v/>
@@ -6246,7 +6364,11 @@
         <f>IF(N(AC41)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC41&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC41&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN41" s="69" t="n"/>
+      <c r="AN41" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 8 d: YT 261 · TT 62 (15% ret).</t>
+        </is>
+      </c>
       <c r="AO41" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -6945,19 +7067,33 @@
           <t>buffer:youtube=6ace86e1eaea728d3cae7fdc;instagram=6ace86e11bdf729a2aa961ae;tiktok=6ace86e29abb1755a4728c48</t>
         </is>
       </c>
-      <c r="S47" s="71" t="n"/>
+      <c r="S47" s="71" t="n">
+        <v>40</v>
+      </c>
       <c r="T47" s="69" t="n"/>
       <c r="U47" s="72">
         <f>IF(OR(T47="",N(O47)=0),"",T47/O47)</f>
         <v/>
       </c>
-      <c r="V47" s="69" t="n"/>
-      <c r="W47" s="69" t="n"/>
+      <c r="V47" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W47" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X47" s="69" t="n"/>
-      <c r="Y47" s="71" t="n"/>
-      <c r="Z47" s="69" t="n"/>
-      <c r="AA47" s="71" t="n"/>
-      <c r="AB47" s="69" t="n"/>
+      <c r="Y47" s="71" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z47" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA47" s="71" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB47" s="69" t="n">
+        <v>1</v>
+      </c>
       <c r="AC47" s="73">
         <f>IF(COUNT(S47,Y47,AA47)=0,"",SUM(S47,Y47,AA47))</f>
         <v/>
@@ -6984,7 +7120,11 @@
         <f>IF(N(AC47)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC47&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC47&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN47" s="69" t="n"/>
+      <c r="AN47" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 11 d: YT 40 · IG 10 (8% ret) · TT 20 (11% ret).</t>
+        </is>
+      </c>
       <c r="AO47" s="69" t="inlineStr">
         <is>
           <t>one-line</t>
@@ -7078,19 +7218,33 @@
           <t>buffer:youtube=6ad04e620d0df6a75bc21aba;instagram=6ad04e6278f377d888aeff2b;tiktok=6ad04e63e09e6bdb27e11075</t>
         </is>
       </c>
-      <c r="S48" s="71" t="n"/>
+      <c r="S48" s="71" t="n">
+        <v>523</v>
+      </c>
       <c r="T48" s="69" t="n"/>
       <c r="U48" s="72">
         <f>IF(OR(T48="",N(O48)=0),"",T48/O48)</f>
         <v/>
       </c>
-      <c r="V48" s="69" t="n"/>
-      <c r="W48" s="69" t="n"/>
+      <c r="V48" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="W48" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X48" s="69" t="n"/>
-      <c r="Y48" s="71" t="n"/>
-      <c r="Z48" s="69" t="n"/>
-      <c r="AA48" s="71" t="n"/>
-      <c r="AB48" s="69" t="n"/>
+      <c r="Y48" s="71" t="n">
+        <v>123</v>
+      </c>
+      <c r="Z48" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA48" s="71" t="n">
+        <v>16</v>
+      </c>
+      <c r="AB48" s="69" t="n">
+        <v>2</v>
+      </c>
       <c r="AC48" s="73">
         <f>IF(COUNT(S48,Y48,AA48)=0,"",SUM(S48,Y48,AA48))</f>
         <v/>
@@ -7117,7 +7271,11 @@
         <f>IF(N(AC48)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC48&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC48&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN48" s="69" t="n"/>
+      <c r="AN48" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 11 d: YT 523 · IG 123 (22% ret) · TT 16 (11% ret).</t>
+        </is>
+      </c>
       <c r="AO48" s="69" t="inlineStr">
         <is>
           <t>ted1</t>
@@ -7562,19 +7720,29 @@
           <t>buffer:youtube=6ad3c111e272c4918f997f66;tiktok=6ad3c1120b0d72757aedb6ef</t>
         </is>
       </c>
-      <c r="S52" s="71" t="n"/>
+      <c r="S52" s="71" t="n">
+        <v>423</v>
+      </c>
       <c r="T52" s="69" t="n"/>
       <c r="U52" s="72">
         <f>IF(OR(T52="",N(O52)=0),"",T52/O52)</f>
         <v/>
       </c>
-      <c r="V52" s="69" t="n"/>
-      <c r="W52" s="69" t="n"/>
+      <c r="V52" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="W52" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X52" s="69" t="n"/>
       <c r="Y52" s="71" t="n"/>
       <c r="Z52" s="69" t="n"/>
-      <c r="AA52" s="71" t="n"/>
-      <c r="AB52" s="69" t="n"/>
+      <c r="AA52" s="71" t="n">
+        <v>30</v>
+      </c>
+      <c r="AB52" s="69" t="n">
+        <v>2</v>
+      </c>
       <c r="AC52" s="73">
         <f>IF(COUNT(S52,Y52,AA52)=0,"",SUM(S52,Y52,AA52))</f>
         <v/>
@@ -7601,7 +7769,11 @@
         <f>IF(N(AC52)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC52&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC52&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN52" s="69" t="n"/>
+      <c r="AN52" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 7 d: YT 423 · TT 30 (9% ret).</t>
+        </is>
+      </c>
       <c r="AO52" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -8869,19 +9041,33 @@
           <t>buffer:youtube=6ace86e34a3bafcd13007ef2;instagram=6ace86e49abb1755a4728ccf;tiktok=6ace86e4cb3665561f6351fe</t>
         </is>
       </c>
-      <c r="S63" s="71" t="n"/>
+      <c r="S63" s="71" t="n">
+        <v>42</v>
+      </c>
       <c r="T63" s="69" t="n"/>
       <c r="U63" s="72">
         <f>IF(OR(T63="",N(O63)=0),"",T63/O63)</f>
         <v/>
       </c>
-      <c r="V63" s="69" t="n"/>
-      <c r="W63" s="69" t="n"/>
+      <c r="V63" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W63" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X63" s="69" t="n"/>
-      <c r="Y63" s="71" t="n"/>
-      <c r="Z63" s="69" t="n"/>
-      <c r="AA63" s="71" t="n"/>
-      <c r="AB63" s="69" t="n"/>
+      <c r="Y63" s="71" t="n">
+        <v>43</v>
+      </c>
+      <c r="Z63" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA63" s="71" t="n">
+        <v>83</v>
+      </c>
+      <c r="AB63" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="AC63" s="73">
         <f>IF(COUNT(S63,Y63,AA63)=0,"",SUM(S63,Y63,AA63))</f>
         <v/>
@@ -8908,7 +9094,11 @@
         <f>IF(N(AC63)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC63&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC63&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN63" s="69" t="n"/>
+      <c r="AN63" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 11 d: YT 42 · IG 43 (13% ret) · TT 83 (9% ret).</t>
+        </is>
+      </c>
       <c r="AO63" s="69" t="inlineStr">
         <is>
           <t>game-show</t>
@@ -9002,19 +9192,33 @@
           <t>buffer:youtube=6ad131032aec0f0a6da4b49c;tiktok=6ad131044fd04e4eb3ab0df1;instagram=6ad7ca1b028de2f3133ebf78</t>
         </is>
       </c>
-      <c r="S64" s="71" t="n"/>
+      <c r="S64" s="71" t="n">
+        <v>182</v>
+      </c>
       <c r="T64" s="69" t="n"/>
       <c r="U64" s="72">
         <f>IF(OR(T64="",N(O64)=0),"",T64/O64)</f>
         <v/>
       </c>
-      <c r="V64" s="69" t="n"/>
-      <c r="W64" s="69" t="n"/>
+      <c r="V64" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="W64" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X64" s="69" t="n"/>
-      <c r="Y64" s="71" t="n"/>
-      <c r="Z64" s="69" t="n"/>
-      <c r="AA64" s="71" t="n"/>
-      <c r="AB64" s="69" t="n"/>
+      <c r="Y64" s="71" t="n">
+        <v>215</v>
+      </c>
+      <c r="Z64" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA64" s="71" t="n">
+        <v>34</v>
+      </c>
+      <c r="AB64" s="69" t="n">
+        <v>3</v>
+      </c>
       <c r="AC64" s="73">
         <f>IF(COUNT(S64,Y64,AA64)=0,"",SUM(S64,Y64,AA64))</f>
         <v/>
@@ -9041,7 +9245,11 @@
         <f>IF(N(AC64)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC64&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC64&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN64" s="69" t="n"/>
+      <c r="AN64" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 9 d: YT 182 · IG 215 (29% ret) · TT 34 (9% ret).</t>
+        </is>
+      </c>
       <c r="AO64" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -9256,19 +9464,33 @@
           <t>buffer:youtube=6acff9681cf1b660315c437a;instagram=6acff968fd7b73f9b827be52;tiktok=6acff96968bd56434b7c64ce</t>
         </is>
       </c>
-      <c r="S66" s="71" t="n"/>
+      <c r="S66" s="71" t="n">
+        <v>1238</v>
+      </c>
       <c r="T66" s="69" t="n"/>
       <c r="U66" s="72">
         <f>IF(OR(T66="",N(O66)=0),"",T66/O66)</f>
         <v/>
       </c>
-      <c r="V66" s="69" t="n"/>
-      <c r="W66" s="69" t="n"/>
+      <c r="V66" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="W66" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X66" s="69" t="n"/>
-      <c r="Y66" s="71" t="n"/>
-      <c r="Z66" s="69" t="n"/>
-      <c r="AA66" s="71" t="n"/>
-      <c r="AB66" s="69" t="n"/>
+      <c r="Y66" s="71" t="n">
+        <v>520</v>
+      </c>
+      <c r="Z66" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA66" s="71" t="n">
+        <v>94</v>
+      </c>
+      <c r="AB66" s="69" t="n">
+        <v>1</v>
+      </c>
       <c r="AC66" s="73">
         <f>IF(COUNT(S66,Y66,AA66)=0,"",SUM(S66,Y66,AA66))</f>
         <v/>
@@ -9295,7 +9517,11 @@
         <f>IF(N(AC66)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC66&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC66&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN66" s="69" t="n"/>
+      <c r="AN66" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 11 d: YT 1238 · IG 520 (37% ret) · TT 94 (13% ret).</t>
+        </is>
+      </c>
       <c r="AO66" s="69" t="inlineStr">
         <is>
           <t>dossier</t>
@@ -9389,19 +9615,33 @@
           <t>buffer:youtube=6ad1310584453eae6f32ec7f;tiktok=6ad131064fd04e4eb3ab0eb3;instagram=6ad91e75b945508d3f85a09d</t>
         </is>
       </c>
-      <c r="S67" s="71" t="n"/>
+      <c r="S67" s="71" t="n">
+        <v>160</v>
+      </c>
       <c r="T67" s="69" t="n"/>
       <c r="U67" s="72">
         <f>IF(OR(T67="",N(O67)=0),"",T67/O67)</f>
         <v/>
       </c>
-      <c r="V67" s="69" t="n"/>
-      <c r="W67" s="69" t="n"/>
+      <c r="V67" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="W67" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X67" s="69" t="n"/>
-      <c r="Y67" s="71" t="n"/>
-      <c r="Z67" s="69" t="n"/>
-      <c r="AA67" s="71" t="n"/>
-      <c r="AB67" s="69" t="n"/>
+      <c r="Y67" s="71" t="n">
+        <v>253</v>
+      </c>
+      <c r="Z67" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA67" s="71" t="n">
+        <v>13</v>
+      </c>
+      <c r="AB67" s="69" t="n">
+        <v>2</v>
+      </c>
       <c r="AC67" s="73">
         <f>IF(COUNT(S67,Y67,AA67)=0,"",SUM(S67,Y67,AA67))</f>
         <v/>
@@ -9428,7 +9668,11 @@
         <f>IF(N(AC67)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC67&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC67&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN67" s="69" t="n"/>
+      <c r="AN67" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 9 d: YT 160 · IG 253 (28% ret) · TT 13 (53% ret).</t>
+        </is>
+      </c>
       <c r="AO67" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -9522,19 +9766,29 @@
           <t>buffer:youtube=6ad3c114ae173d6e00cc5d2c;tiktok=6ad3c114938409f1d09b2e54</t>
         </is>
       </c>
-      <c r="S68" s="71" t="n"/>
+      <c r="S68" s="71" t="n">
+        <v>672</v>
+      </c>
       <c r="T68" s="69" t="n"/>
       <c r="U68" s="72">
         <f>IF(OR(T68="",N(O68)=0),"",T68/O68)</f>
         <v/>
       </c>
-      <c r="V68" s="69" t="n"/>
-      <c r="W68" s="69" t="n"/>
+      <c r="V68" s="69" t="n">
+        <v>7</v>
+      </c>
+      <c r="W68" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X68" s="69" t="n"/>
       <c r="Y68" s="71" t="n"/>
       <c r="Z68" s="69" t="n"/>
-      <c r="AA68" s="71" t="n"/>
-      <c r="AB68" s="69" t="n"/>
+      <c r="AA68" s="71" t="n">
+        <v>33</v>
+      </c>
+      <c r="AB68" s="69" t="n">
+        <v>1</v>
+      </c>
       <c r="AC68" s="73">
         <f>IF(COUNT(S68,Y68,AA68)=0,"",SUM(S68,Y68,AA68))</f>
         <v/>
@@ -9561,7 +9815,11 @@
         <f>IF(N(AC68)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC68&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC68&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN68" s="69" t="n"/>
+      <c r="AN68" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 7 d: YT 672 · TT 33 (8% ret).</t>
+        </is>
+      </c>
       <c r="AO68" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -10546,19 +10804,33 @@
           <t>buffer:youtube=6acff96a38b78c67c8fec2aa;instagram=6acff96b68bd56434b7c651d;tiktok=6acff96b90e61174bee1ea47</t>
         </is>
       </c>
-      <c r="S76" s="71" t="n"/>
+      <c r="S76" s="71" t="n">
+        <v>666</v>
+      </c>
       <c r="T76" s="69" t="n"/>
       <c r="U76" s="72">
         <f>IF(OR(T76="",N(O76)=0),"",T76/O76)</f>
         <v/>
       </c>
-      <c r="V76" s="69" t="n"/>
-      <c r="W76" s="69" t="n"/>
+      <c r="V76" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="W76" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X76" s="69" t="n"/>
-      <c r="Y76" s="71" t="n"/>
-      <c r="Z76" s="69" t="n"/>
-      <c r="AA76" s="71" t="n"/>
-      <c r="AB76" s="69" t="n"/>
+      <c r="Y76" s="71" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z76" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="71" t="n">
+        <v>75</v>
+      </c>
+      <c r="AB76" s="69" t="n">
+        <v>5</v>
+      </c>
       <c r="AC76" s="73">
         <f>IF(COUNT(S76,Y76,AA76)=0,"",SUM(S76,Y76,AA76))</f>
         <v/>
@@ -10585,7 +10857,11 @@
         <f>IF(N(AC76)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC76&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC76&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN76" s="69" t="n"/>
+      <c r="AN76" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 11 d: YT 666 · IG 14 (12% ret) · TT 75 (18% ret).</t>
+        </is>
+      </c>
       <c r="AO76" s="69" t="inlineStr">
         <is>
           <t>data-story</t>
@@ -10679,19 +10955,33 @@
           <t>buffer:youtube=6ad131084fd04e4eb3ab0f47;tiktok=6ad13108b4510d553d75e196;instagram=6ada6fa180b62e657504c588</t>
         </is>
       </c>
-      <c r="S77" s="71" t="n"/>
+      <c r="S77" s="71" t="n">
+        <v>804</v>
+      </c>
       <c r="T77" s="69" t="n"/>
       <c r="U77" s="72">
         <f>IF(OR(T77="",N(O77)=0),"",T77/O77)</f>
         <v/>
       </c>
-      <c r="V77" s="69" t="n"/>
-      <c r="W77" s="69" t="n"/>
+      <c r="V77" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="W77" s="69" t="n">
+        <v>4</v>
+      </c>
       <c r="X77" s="69" t="n"/>
-      <c r="Y77" s="71" t="n"/>
-      <c r="Z77" s="69" t="n"/>
-      <c r="AA77" s="71" t="n"/>
-      <c r="AB77" s="69" t="n"/>
+      <c r="Y77" s="71" t="n">
+        <v>1509</v>
+      </c>
+      <c r="Z77" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA77" s="71" t="n">
+        <v>9</v>
+      </c>
+      <c r="AB77" s="69" t="n">
+        <v>1</v>
+      </c>
       <c r="AC77" s="73">
         <f>IF(COUNT(S77,Y77,AA77)=0,"",SUM(S77,Y77,AA77))</f>
         <v/>
@@ -10718,7 +11008,11 @@
         <f>IF(N(AC77)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC77&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC77&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN77" s="69" t="n"/>
+      <c r="AN77" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 9 d: YT 804 · IG 1509 (48% ret) · TT 9 (14% ret).</t>
+        </is>
+      </c>
       <c r="AO77" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -10812,19 +11106,29 @@
           <t>buffer:youtube=6ad3c116938409f1d09b2eb1;tiktok=6ad3c117ae173d6e00cc5da0</t>
         </is>
       </c>
-      <c r="S78" s="71" t="n"/>
+      <c r="S78" s="71" t="n">
+        <v>119</v>
+      </c>
       <c r="T78" s="69" t="n"/>
       <c r="U78" s="72">
         <f>IF(OR(T78="",N(O78)=0),"",T78/O78)</f>
         <v/>
       </c>
-      <c r="V78" s="69" t="n"/>
-      <c r="W78" s="69" t="n"/>
+      <c r="V78" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="W78" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X78" s="69" t="n"/>
       <c r="Y78" s="71" t="n"/>
       <c r="Z78" s="69" t="n"/>
-      <c r="AA78" s="71" t="n"/>
-      <c r="AB78" s="69" t="n"/>
+      <c r="AA78" s="71" t="n">
+        <v>24</v>
+      </c>
+      <c r="AB78" s="69" t="n">
+        <v>3</v>
+      </c>
       <c r="AC78" s="73">
         <f>IF(COUNT(S78,Y78,AA78)=0,"",SUM(S78,Y78,AA78))</f>
         <v/>
@@ -10851,7 +11155,11 @@
         <f>IF(N(AC78)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC78&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC78&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN78" s="69" t="n"/>
+      <c r="AN78" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 7 d: YT 119 · TT 24 (16% ret).</t>
+        </is>
+      </c>
       <c r="AO78" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -11929,17 +12237,27 @@
           <t>buffer:youtube=6acfed2bd7ed7764890a8cb7;instagram=6acfed2b384901ac08409b26;tiktok=6acfed2cd7ed7764890a8d15</t>
         </is>
       </c>
-      <c r="S87" s="71" t="n"/>
+      <c r="S87" s="71" t="n">
+        <v>123</v>
+      </c>
       <c r="T87" s="69" t="n"/>
       <c r="U87" s="72">
         <f>IF(OR(T87="",N(O87)=0),"",T87/O87)</f>
         <v/>
       </c>
-      <c r="V87" s="69" t="n"/>
-      <c r="W87" s="69" t="n"/>
+      <c r="V87" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W87" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X87" s="69" t="n"/>
-      <c r="Y87" s="71" t="n"/>
-      <c r="Z87" s="69" t="n"/>
+      <c r="Y87" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z87" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="AA87" s="71" t="n"/>
       <c r="AB87" s="69" t="n"/>
       <c r="AC87" s="73">
@@ -11968,7 +12286,11 @@
         <f>IF(N(AC87)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC87&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC87&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN87" s="69" t="n"/>
+      <c r="AN87" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 10 d: YT 123 · IG 4 (4% ret).</t>
+        </is>
+      </c>
       <c r="AO87" s="69" t="inlineStr">
         <is>
           <t>game-show</t>
@@ -12062,19 +12384,33 @@
           <t>buffer:youtube=6ad1310ab4510d553d75e22a;tiktok=6ad1310b84453eae6f32edcf;instagram=6adbc6ad8b3d437ddc85eb35</t>
         </is>
       </c>
-      <c r="S88" s="71" t="n"/>
+      <c r="S88" s="71" t="n">
+        <v>295</v>
+      </c>
       <c r="T88" s="69" t="n"/>
       <c r="U88" s="72">
         <f>IF(OR(T88="",N(O88)=0),"",T88/O88)</f>
         <v/>
       </c>
-      <c r="V88" s="69" t="n"/>
-      <c r="W88" s="69" t="n"/>
+      <c r="V88" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="W88" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X88" s="69" t="n"/>
-      <c r="Y88" s="71" t="n"/>
-      <c r="Z88" s="69" t="n"/>
-      <c r="AA88" s="71" t="n"/>
-      <c r="AB88" s="69" t="n"/>
+      <c r="Y88" s="71" t="n">
+        <v>327</v>
+      </c>
+      <c r="Z88" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA88" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB88" s="69" t="n">
+        <v>1</v>
+      </c>
       <c r="AC88" s="73">
         <f>IF(COUNT(S88,Y88,AA88)=0,"",SUM(S88,Y88,AA88))</f>
         <v/>
@@ -12101,7 +12437,11 @@
         <f>IF(N(AC88)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC88&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC88&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN88" s="69" t="n"/>
+      <c r="AN88" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 9 d: YT 295 · IG 327 (25% ret) · TT 2 (4% ret).</t>
+        </is>
+      </c>
       <c r="AO88" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -13199,19 +13539,29 @@
           <t>buffer:youtube=6ad14ad97998c185a61ca9af;tiktok=6ad14ada5533140b41cadc08</t>
         </is>
       </c>
-      <c r="S97" s="71" t="n"/>
+      <c r="S97" s="71" t="n">
+        <v>251</v>
+      </c>
       <c r="T97" s="69" t="n"/>
       <c r="U97" s="72">
         <f>IF(OR(T97="",N(O97)=0),"",T97/O97)</f>
         <v/>
       </c>
-      <c r="V97" s="69" t="n"/>
-      <c r="W97" s="69" t="n"/>
+      <c r="V97" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="W97" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X97" s="69" t="n"/>
       <c r="Y97" s="71" t="n"/>
       <c r="Z97" s="69" t="n"/>
-      <c r="AA97" s="71" t="n"/>
-      <c r="AB97" s="69" t="n"/>
+      <c r="AA97" s="71" t="n">
+        <v>115</v>
+      </c>
+      <c r="AB97" s="69" t="n">
+        <v>12</v>
+      </c>
       <c r="AC97" s="73">
         <f>IF(COUNT(S97,Y97,AA97)=0,"",SUM(S97,Y97,AA97))</f>
         <v/>
@@ -13238,7 +13588,11 @@
         <f>IF(N(AC97)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC97&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC97&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN97" s="69" t="n"/>
+      <c r="AN97" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 10 d: YT 251 · TT 115 (19% ret).</t>
+        </is>
+      </c>
       <c r="AO97" s="69" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -14308,19 +14662,33 @@
           <t>buffer:youtube=6ad0715a8b6f374826e2018a;instagram=6ad0715b8886414c963c3815;tiktok=6ad0715b0ad4869c077e294a</t>
         </is>
       </c>
-      <c r="S106" s="71" t="n"/>
+      <c r="S106" s="71" t="n">
+        <v>3</v>
+      </c>
       <c r="T106" s="69" t="n"/>
       <c r="U106" s="72">
         <f>IF(OR(T106="",N(O106)=0),"",T106/O106)</f>
         <v/>
       </c>
-      <c r="V106" s="69" t="n"/>
-      <c r="W106" s="69" t="n"/>
+      <c r="V106" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W106" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X106" s="69" t="n"/>
-      <c r="Y106" s="71" t="n"/>
-      <c r="Z106" s="69" t="n"/>
-      <c r="AA106" s="71" t="n"/>
-      <c r="AB106" s="69" t="n"/>
+      <c r="Y106" s="71" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z106" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA106" s="71" t="n">
+        <v>24</v>
+      </c>
+      <c r="AB106" s="69" t="n">
+        <v>1</v>
+      </c>
       <c r="AC106" s="73">
         <f>IF(COUNT(S106,Y106,AA106)=0,"",SUM(S106,Y106,AA106))</f>
         <v/>
@@ -14347,7 +14715,11 @@
         <f>IF(N(AC106)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC106&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC106&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN106" s="69" t="n"/>
+      <c r="AN106" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 10 d: YT 3 · IG 21 (17% ret) · TT 24 (3% ret).</t>
+        </is>
+      </c>
       <c r="AO106" s="69" t="inlineStr">
         <is>
           <t>nova</t>
@@ -14433,19 +14805,29 @@
           <t>buffer:youtube=6ad1a654a82f34dbe1464882;tiktok=6ad1a654fb64fffcf1b41af2;instagram=6adcff3c3d5b27036b9ba0a4</t>
         </is>
       </c>
-      <c r="S107" s="71" t="n"/>
+      <c r="S107" s="71" t="n">
+        <v>107</v>
+      </c>
       <c r="T107" s="69" t="n"/>
       <c r="U107" s="72">
         <f>IF(OR(T107="",N(O107)=0),"",T107/O107)</f>
         <v/>
       </c>
-      <c r="V107" s="69" t="n"/>
-      <c r="W107" s="69" t="n"/>
+      <c r="V107" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="W107" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="X107" s="69" t="n"/>
       <c r="Y107" s="71" t="n"/>
       <c r="Z107" s="69" t="n"/>
-      <c r="AA107" s="71" t="n"/>
-      <c r="AB107" s="69" t="n"/>
+      <c r="AA107" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB107" s="69" t="n">
+        <v>0</v>
+      </c>
       <c r="AC107" s="73">
         <f>IF(COUNT(S107,Y107,AA107)=0,"",SUM(S107,Y107,AA107))</f>
         <v/>
@@ -14472,7 +14854,11 @@
         <f>IF(N(AC107)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC107&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC107&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN107" s="69" t="n"/>
+      <c r="AN107" s="69" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: d7 from Buffer at age 9 d: YT 107 · TT 1 (6% ret).</t>
+        </is>
+      </c>
       <c r="AO107" s="69" t="inlineStr">
         <is>
           <t>editorial</t>
@@ -14520,7 +14906,7 @@
       </c>
       <c r="H108" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="I108" s="124" t="n">
@@ -14601,7 +14987,11 @@
         <f>IF(N(AC108)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC108&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC108&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN108" s="124" t="n"/>
+      <c r="AN108" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: sent on all 3 per Buffer; early (~1 day) IG 1638 (52% ret) · TT 45 (13%) · YT 4. Pattern-test day 1.</t>
+        </is>
+      </c>
       <c r="AO108" s="124" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -14649,7 +15039,7 @@
       </c>
       <c r="H109" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="I109" s="124" t="n">
@@ -14730,7 +15120,11 @@
         <f>IF(N(AC109)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC109&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC109&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN109" s="124" t="n"/>
+      <c r="AN109" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: sent on all 3 per Buffer; early (~1 day) IG 226 (37% ret) · TT 54 (20%) · YT 0. Pattern-test day 1.</t>
+        </is>
+      </c>
       <c r="AO109" s="124" t="inlineStr">
         <is>
           <t>ted2</t>
@@ -14778,7 +15172,7 @@
       </c>
       <c r="H110" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="I110" s="124" t="n">
@@ -14859,7 +15253,11 @@
         <f>IF(N(AC110)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC110&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC110&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN110" s="124" t="n"/>
+      <c r="AN110" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-25 review: sent on all 3 per Buffer; early (~1 day) IG 1361 (42% ret) · TT 30 (13%) · YT 0. Pattern-test day 1.</t>
+        </is>
+      </c>
       <c r="AO110" s="124" t="inlineStr">
         <is>
           <t>ted2</t>

</xml_diff>

<commit_message>
Stop stick stories for psychology Shorts; queue the retro Short to post as built
- Tracker rows 112-114 (unbuilt stick scripts) -> Vetoed (Shivam 2026-10-26: stick format stopped;
  the Stick or Twist channel is separate and untouched)
- New row 136: arthur-the-critic (retro), Scripted, posted from the approved render
- build_short.sh: any slug with source/final.mp4 is posted as-is (plus platform music variants)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pD4wKEEfqXBEsy6kZEdFn
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -1141,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:AV140"/>
+  <dimension ref="A2:AV141"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="61" min="1" max="1"/>
@@ -16103,7 +16103,7 @@
       </c>
       <c r="H117" s="123" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I117" s="124" t="n">
@@ -16176,7 +16176,11 @@
         <f>IF(N(AC117)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC117&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC117&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN117" s="124" t="n"/>
+      <c r="AN117" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-26 Shivam: stick format stopped for psychology Shorts (replaced by the tedmg/retro style cycle); never built</t>
+        </is>
+      </c>
       <c r="AO117" s="124" t="inlineStr">
         <is>
           <t>stick</t>
@@ -16224,7 +16228,7 @@
       </c>
       <c r="H118" s="123" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I118" s="124" t="n">
@@ -16297,7 +16301,11 @@
         <f>IF(N(AC118)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC118&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC118&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN118" s="124" t="n"/>
+      <c r="AN118" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-26 Shivam: stick format stopped for psychology Shorts (replaced by the tedmg/retro style cycle); never built</t>
+        </is>
+      </c>
       <c r="AO118" s="124" t="inlineStr">
         <is>
           <t>stick</t>
@@ -16345,7 +16353,7 @@
       </c>
       <c r="H119" s="123" t="inlineStr">
         <is>
-          <t>Scripted</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I119" s="124" t="n">
@@ -16418,7 +16426,11 @@
         <f>IF(N(AC119)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC119&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC119&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
         <v/>
       </c>
-      <c r="AN119" s="124" t="n"/>
+      <c r="AN119" s="124" t="inlineStr">
+        <is>
+          <t>2026-10-26 Shivam: stick format stopped for psychology Shorts (replaced by the tedmg/retro style cycle); never built</t>
+        </is>
+      </c>
       <c r="AO119" s="124" t="inlineStr">
         <is>
           <t>stick</t>
@@ -18840,6 +18852,117 @@
       <c r="AT140" s="129" t="n"/>
       <c r="AU140" s="129" t="n"/>
       <c r="AV140" s="130" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="123" t="n">
+        <v>136</v>
+      </c>
+      <c r="B141" s="123" t="inlineStr">
+        <is>
+          <t>Character story</t>
+        </is>
+      </c>
+      <c r="C141" s="123" t="inlineStr">
+        <is>
+          <t>Arthur &amp; the Critic: one criticism beats ten compliments (negativity bias)</t>
+        </is>
+      </c>
+      <c r="D141" s="123" t="inlineStr">
+        <is>
+          <t>Arthur got ten compliments today. And one criticism.</t>
+        </is>
+      </c>
+      <c r="E141" s="123" t="inlineStr">
+        <is>
+          <t>Negativity bias: bad is stronger than good (Baumeister et al. 2001; Rozin &amp; Royzman 2001); the Critic is an old alarm</t>
+        </is>
+      </c>
+      <c r="F141" s="123" t="n"/>
+      <c r="G141" s="123" t="n"/>
+      <c r="H141" s="123" t="inlineStr">
+        <is>
+          <t>Scripted</t>
+        </is>
+      </c>
+      <c r="I141" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" s="124" t="n"/>
+      <c r="K141" s="124" t="inlineStr">
+        <is>
+          <t>arthur-the-critic</t>
+        </is>
+      </c>
+      <c r="L141" s="125" t="n"/>
+      <c r="M141" s="123">
+        <f>IF(L141="","",TEXT(L141,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="N141" s="124" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="O141" s="124" t="n"/>
+      <c r="P141" s="124" t="n"/>
+      <c r="Q141" s="124" t="inlineStr">
+        <is>
+          <t>Baumeister, Bratslavsky, Finkenauer &amp; Vohs 2001 (Rev Gen Psych); Rozin &amp; Royzman 2001 (PSPR)</t>
+        </is>
+      </c>
+      <c r="R141" s="124" t="n"/>
+      <c r="S141" s="126" t="n"/>
+      <c r="T141" s="124" t="n"/>
+      <c r="U141" s="127">
+        <f>IF(OR(T141="",N(O141)=0),"",T141/O141)</f>
+        <v/>
+      </c>
+      <c r="V141" s="124" t="n"/>
+      <c r="W141" s="124" t="n"/>
+      <c r="X141" s="124" t="n"/>
+      <c r="Y141" s="126" t="n"/>
+      <c r="Z141" s="124" t="n"/>
+      <c r="AA141" s="126" t="n"/>
+      <c r="AB141" s="124" t="n"/>
+      <c r="AC141" s="128">
+        <f>IF(COUNT(S141,Y141,AA141)=0,"",SUM(S141,Y141,AA141))</f>
+        <v/>
+      </c>
+      <c r="AD141" s="127">
+        <f>IF(N(AC141)=0,"",SUM(V141,W141,X141,Z141,AB141)/AC141)</f>
+        <v/>
+      </c>
+      <c r="AE141" s="126" t="n"/>
+      <c r="AF141" s="126" t="n"/>
+      <c r="AG141" s="126" t="n"/>
+      <c r="AH141" s="128">
+        <f>IF(COUNT(AE141,AF141,AG141)=0,"",SUM(AE141,AF141,AG141))</f>
+        <v/>
+      </c>
+      <c r="AI141" s="126" t="n"/>
+      <c r="AJ141" s="126" t="n"/>
+      <c r="AK141" s="126" t="n"/>
+      <c r="AL141" s="128">
+        <f>IF(COUNT(AI141,AJ141,AK141)=0,"",SUM(AI141,AJ141,AK141))</f>
+        <v/>
+      </c>
+      <c r="AM141" s="123">
+        <f>IF(N(AC141)=0,"",IF(COUNT($AC$6:$AC$105)&lt;5,"Too early",IF(AC141&gt;=1.5*MEDIAN($AC$6:$AC$105),"Top",IF(AC141&lt;=0.5*MEDIAN($AC$6:$AC$105),"Low","Average"))))</f>
+        <v/>
+      </c>
+      <c r="AN141" s="124" t="n"/>
+      <c r="AO141" s="124" t="inlineStr">
+        <is>
+          <t>retro</t>
+        </is>
+      </c>
+      <c r="AP141" s="129" t="n"/>
+      <c r="AQ141" s="129" t="n"/>
+      <c r="AR141" s="129" t="n"/>
+      <c r="AS141" s="129" t="n"/>
+      <c r="AT141" s="129" t="n"/>
+      <c r="AU141" s="129" t="n"/>
+      <c r="AV141" s="130" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="AM6:AM105">
@@ -18851,19 +18974,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="H6:H140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H6:H141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Idea,Researching,Scripted,Scheduled,Published,Vetoed,Failed,Filming,Editing"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="J6:J140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="J6:J141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Strong,Weak"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AO6:AO140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AO6:AO141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>Looks!$A$5:$A$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="AP6:AP140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="AP6:AP141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"ted2,story"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Tracker: rows 110-111 Vetoed (stick posts cancelled in Buffer, Shivam 2026-10-26)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pD4wKEEfqXBEsy6kZEdFn
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -15837,7 +15837,7 @@
       </c>
       <c r="H115" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I115" s="124" t="n">
@@ -15920,7 +15920,7 @@
       </c>
       <c r="AN115" s="124" t="inlineStr">
         <is>
-          <t>2026-10-25: explainer script shelved; rewrite as a stick character story (Shivam)</t>
+          <t>2026-10-26 Shivam: stick format stopped; scheduled Buffer posts deleted before they went out</t>
         </is>
       </c>
       <c r="AO115" s="124" t="inlineStr">
@@ -15970,7 +15970,7 @@
       </c>
       <c r="H116" s="123" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Vetoed</t>
         </is>
       </c>
       <c r="I116" s="124" t="n">
@@ -16053,7 +16053,7 @@
       </c>
       <c r="AN116" s="124" t="inlineStr">
         <is>
-          <t>2026-10-25: explainer script shelved; rewrite as a stick character story (Shivam)</t>
+          <t>2026-10-26 Shivam: stick format stopped; scheduled Buffer posts deleted before they went out</t>
         </is>
       </c>
       <c r="AO116" s="124" t="inlineStr">

</xml_diff>

<commit_message>
scripts: 3 new (doodlers tedmg, first-impressions tedmg, friend-question ted2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EKMmbo2dX24agYX8CfZocZ
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -16478,7 +16478,7 @@
       </c>
       <c r="H120" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I120" s="124" t="n">
@@ -16499,10 +16499,18 @@
         <f>IF(L120="","",TEXT(L120,"ddd"))</f>
         <v/>
       </c>
-      <c r="N120" s="124" t="n"/>
+      <c r="N120" s="124" t="inlineStr">
+        <is>
+          <t>character story: June doodles through the meeting</t>
+        </is>
+      </c>
       <c r="O120" s="124" t="n"/>
       <c r="P120" s="124" t="n"/>
-      <c r="Q120" s="124" t="n"/>
+      <c r="Q120" s="124" t="inlineStr">
+        <is>
+          <t>Andrade, Applied Cognitive Psychology 24(1) 2010 (online 2009): 40 adults, doodlers recalled 29% more (7.5 vs 5.81) — simplypsychology.org/andrade-doodling.html</t>
+        </is>
+      </c>
       <c r="R120" s="124" t="n"/>
       <c r="S120" s="126" t="n"/>
       <c r="T120" s="124" t="n"/>
@@ -16546,7 +16554,7 @@
       <c r="AN120" s="124" t="n"/>
       <c r="AO120" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>tedmg</t>
         </is>
       </c>
       <c r="AP120" s="129" t="n"/>
@@ -16591,7 +16599,7 @@
       </c>
       <c r="H121" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I121" s="124" t="n">
@@ -16612,10 +16620,18 @@
         <f>IF(L121="","",TEXT(L121,"ddd"))</f>
         <v/>
       </c>
-      <c r="N121" s="124" t="n"/>
+      <c r="N121" s="124" t="inlineStr">
+        <is>
+          <t>character story: Rosa rehearsed 40 answers (numbered facts)</t>
+        </is>
+      </c>
       <c r="O121" s="124" t="n"/>
       <c r="P121" s="124" t="n"/>
-      <c r="Q121" s="124" t="n"/>
+      <c r="Q121" s="124" t="inlineStr">
+        <is>
+          <t>Willis &amp; Todorov 2006 Psych Sci (PubMed 16866745): 100-ms judgments correlate highly with untimed, longer exposure mainly raises confidence; Nisbett &amp; Wilson 1977 JPSP halo (warm vs cold lecturer, 118 Michigan students)</t>
+        </is>
+      </c>
       <c r="R121" s="124" t="n"/>
       <c r="S121" s="126" t="n"/>
       <c r="T121" s="124" t="n"/>
@@ -16659,7 +16675,7 @@
       <c r="AN121" s="124" t="n"/>
       <c r="AO121" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>tedmg</t>
         </is>
       </c>
       <c r="AP121" s="129" t="n"/>
@@ -16704,7 +16720,7 @@
       </c>
       <c r="H122" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I122" s="124" t="n">
@@ -16725,10 +16741,18 @@
         <f>IF(L122="","",TEXT(L122,"ddd"))</f>
         <v/>
       </c>
-      <c r="N122" s="124" t="n"/>
+      <c r="N122" s="124" t="inlineStr">
+        <is>
+          <t>you callout: Stuck? Ask yourself one question</t>
+        </is>
+      </c>
       <c r="O122" s="124" t="n"/>
       <c r="P122" s="124" t="n"/>
-      <c r="Q122" s="124" t="n"/>
+      <c r="Q122" s="124" t="inlineStr">
+        <is>
+          <t>Grossmann &amp; Kross 2014 Psych Sci 'Exploring Solomon's paradox' (doi 10.1177/0956797614535400): wiser reasoning about a friend's problem; self-distancing eliminated the asymmetry</t>
+        </is>
+      </c>
       <c r="R122" s="124" t="n"/>
       <c r="S122" s="126" t="n"/>
       <c r="T122" s="124" t="n"/>

</xml_diff>

<commit_message>
scripts: 3 new (shaky-bridge tedmg, semantic-satiation ted2, stroop-test retro)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EKMmbo2dX24agYX8CfZocZ
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -16841,7 +16841,7 @@
       </c>
       <c r="H123" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I123" s="124" t="n">
@@ -16862,10 +16862,18 @@
         <f>IF(L123="","",TEXT(L123,"ddd"))</f>
         <v/>
       </c>
-      <c r="N123" s="124" t="n"/>
+      <c r="N123" s="124" t="inlineStr">
+        <is>
+          <t>character story: Theo says make the date scary</t>
+        </is>
+      </c>
       <c r="O123" s="124" t="n"/>
       <c r="P123" s="124" t="n"/>
-      <c r="Q123" s="124" t="n"/>
+      <c r="Q123" s="124" t="inlineStr">
+        <is>
+          <t>Dutton &amp; Aron 1974 JPSP (Capilano suspension bridge ~230 ft vs low solid bridge): ~50% vs 12.5% of men called the female interviewer — youarenotsosmart.com/2011/07/07/misattribution-of-arousal</t>
+        </is>
+      </c>
       <c r="R123" s="124" t="n"/>
       <c r="S123" s="126" t="n"/>
       <c r="T123" s="124" t="n"/>
@@ -16909,7 +16917,7 @@
       <c r="AN123" s="124" t="n"/>
       <c r="AO123" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>tedmg</t>
         </is>
       </c>
       <c r="AP123" s="129" t="n"/>
@@ -16954,7 +16962,7 @@
       </c>
       <c r="H124" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I124" s="124" t="n">
@@ -16975,10 +16983,18 @@
         <f>IF(L124="","",TEXT(L124,"ddd"))</f>
         <v/>
       </c>
-      <c r="N124" s="124" t="n"/>
+      <c r="N124" s="124" t="inlineStr">
+        <is>
+          <t>bold claim: say any word over and over</t>
+        </is>
+      </c>
       <c r="O124" s="124" t="n"/>
       <c r="P124" s="124" t="n"/>
-      <c r="Q124" s="124" t="n"/>
+      <c r="Q124" s="124" t="inlineStr">
+        <is>
+          <t>Severance &amp; Washburn 1907 (Am J Psych): 3-min fixation on a word → loss of meaning; term coined by Leon Jakobovits James, 1962 McGill dissertation (Wikipedia; Frontiers in Psychology 2019 10.3389/fpsyg.2019.02236). Hook's '30 times' dropped: no study gives a count</t>
+        </is>
+      </c>
       <c r="R124" s="124" t="n"/>
       <c r="S124" s="126" t="n"/>
       <c r="T124" s="124" t="n"/>
@@ -17067,7 +17083,7 @@
       </c>
       <c r="H125" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I125" s="124" t="n">
@@ -17088,10 +17104,18 @@
         <f>IF(L125="","",TEXT(L125,"ddd"))</f>
         <v/>
       </c>
-      <c r="N125" s="124" t="n"/>
+      <c r="N125" s="124" t="inlineStr">
+        <is>
+          <t>character story + viewer quiz: Otto says no test can trick him</t>
+        </is>
+      </c>
       <c r="O125" s="124" t="n"/>
       <c r="P125" s="124" t="n"/>
-      <c r="Q125" s="124" t="n"/>
+      <c r="Q125" s="124" t="inlineStr">
+        <is>
+          <t>Stroop 1935 J Exp Psych 'Studies of interference in serial verbal reactions': 100 undergraduates, naming ink of incongruent colour words took ~47 s (74.3%) longer than colour patches — simplypsychology.org/stroop-effect.html</t>
+        </is>
+      </c>
       <c r="R125" s="124" t="n"/>
       <c r="S125" s="126" t="n"/>
       <c r="T125" s="124" t="n"/>
@@ -17135,7 +17159,7 @@
       <c r="AN125" s="124" t="n"/>
       <c r="AO125" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>retro</t>
         </is>
       </c>
       <c r="AP125" s="129" t="n"/>

</xml_diff>

<commit_message>
scripts: 6 new (ted2 x2, retro x2, tedmg x2) + fix stroop-test negative-t crash
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EKMmbo67ryiMzz2ccuk36K
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -17123,7 +17123,7 @@
       </c>
       <c r="H125" s="123" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I125" s="124" t="n">
@@ -17198,7 +17198,7 @@
       </c>
       <c r="AN125" s="124" t="inlineStr">
         <is>
-          <t>CI 2026-10-28: build produced no video</t>
+          <t>CI 2026-10-28: build produced no video (art threw on negative t in STQuiz); fixed 2026-10-29 by the script writer, back to Scripted (once)</t>
         </is>
       </c>
       <c r="AO125" s="124" t="inlineStr">
@@ -17248,7 +17248,7 @@
       </c>
       <c r="H126" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I126" s="124" t="n">
@@ -17269,10 +17269,18 @@
         <f>IF(L126="","",TEXT(L126,"ddd"))</f>
         <v/>
       </c>
-      <c r="N126" s="124" t="n"/>
+      <c r="N126" s="124" t="inlineStr">
+        <is>
+          <t>character story: Leo cuts the copier line with because</t>
+        </is>
+      </c>
       <c r="O126" s="124" t="n"/>
       <c r="P126" s="124" t="n"/>
-      <c r="Q126" s="124" t="n"/>
+      <c r="Q126" s="124" t="inlineStr">
+        <is>
+          <t>Langer, Blank &amp; Chanowitz 1978 JPSP 36(6): library copier, 5 pages — no reason 60%, real reason 94%, empty reason ('I have to make copies') 93%; for 20 pages the empty 'because' stopped working — jamesclear.com/copy-machine-study</t>
+        </is>
+      </c>
       <c r="R126" s="124" t="n"/>
       <c r="S126" s="126" t="n"/>
       <c r="T126" s="124" t="n"/>
@@ -17361,7 +17369,7 @@
       </c>
       <c r="H127" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I127" s="124" t="n">
@@ -17382,10 +17390,18 @@
         <f>IF(L127="","",TEXT(L127,"ddd"))</f>
         <v/>
       </c>
-      <c r="N127" s="124" t="n"/>
+      <c r="N127" s="124" t="inlineStr">
+        <is>
+          <t>character story: Arthur's flight home gets cancelled after six perfect days</t>
+        </is>
+      </c>
       <c r="O127" s="124" t="n"/>
       <c r="P127" s="124" t="n"/>
-      <c r="Q127" s="124" t="n"/>
+      <c r="Q127" s="124" t="inlineStr">
+        <is>
+          <t>Kahneman, Fredrickson, Schreiber &amp; Redelmeier 1993 Psych Sci 'When more pain is preferred to less': 60 s at 14 °C vs same + 30 s warming to ~15 °C; nearly 70% chose to repeat the longer trial — mindhacks.com/2013/05/28/why-you-might-prefer-more-pain/, en.wikipedia.org/wiki/Duration_neglect</t>
+        </is>
+      </c>
       <c r="R127" s="124" t="n"/>
       <c r="S127" s="126" t="n"/>
       <c r="T127" s="124" t="n"/>
@@ -17429,7 +17445,7 @@
       <c r="AN127" s="124" t="n"/>
       <c r="AO127" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>retro</t>
         </is>
       </c>
       <c r="AP127" s="129" t="n"/>
@@ -17474,7 +17490,7 @@
       </c>
       <c r="H128" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I128" s="124" t="n">
@@ -17495,10 +17511,18 @@
         <f>IF(L128="","",TEXT(L128,"ddd"))</f>
         <v/>
       </c>
-      <c r="N128" s="124" t="n"/>
+      <c r="N128" s="124" t="inlineStr">
+        <is>
+          <t>result-first number: Two in three ordinary people went all the way to the highest SHOCK</t>
+        </is>
+      </c>
       <c r="O128" s="124" t="n"/>
       <c r="P128" s="124" t="n"/>
-      <c r="Q128" s="124" t="n"/>
+      <c r="Q128" s="124" t="inlineStr">
+        <is>
+          <t>Milgram 1963 J Abnormal &amp; Social Psych: 40 men, 26/40 (65%) to 450 V, all to 300 V; psychiatrists predicted ~0.1%; Milgram 1974 two-peers-refuse variation 4/40; caveat Perry 2012 — en.wikipedia.org/wiki/Milgram_experiment</t>
+        </is>
+      </c>
       <c r="R128" s="124" t="n"/>
       <c r="S128" s="126" t="n"/>
       <c r="T128" s="124" t="n"/>
@@ -17587,7 +17611,7 @@
       </c>
       <c r="H129" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I129" s="124" t="n">
@@ -17608,10 +17632,18 @@
         <f>IF(L129="","",TEXT(L129,"ddd"))</f>
         <v/>
       </c>
-      <c r="N129" s="124" t="n"/>
+      <c r="N129" s="124" t="inlineStr">
+        <is>
+          <t>character story: Lila sees an only-two-left sign</t>
+        </is>
+      </c>
       <c r="O129" s="124" t="n"/>
       <c r="P129" s="124" t="n"/>
-      <c r="Q129" s="124" t="n"/>
+      <c r="Q129" s="124" t="inlineStr">
+        <is>
+          <t>Worchel, Lee &amp; Adewole 1975 JPSP 'Effects of supply and demand on ratings of object value': 134 students, identical cookies from a jar of 2 rated more desirable/attractive than from a jar of 10; drop 10→2 by demand raised value most; price difference n.s. (no price claim) — uni-muenster.de PDF of the paper, coglode.com/nuggets/scarcity</t>
+        </is>
+      </c>
       <c r="R129" s="124" t="n"/>
       <c r="S129" s="126" t="n"/>
       <c r="T129" s="124" t="n"/>
@@ -17655,7 +17687,7 @@
       <c r="AN129" s="124" t="n"/>
       <c r="AO129" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>retro</t>
         </is>
       </c>
       <c r="AP129" s="129" t="n"/>
@@ -17700,7 +17732,7 @@
       </c>
       <c r="H130" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I130" s="124" t="n">
@@ -17721,10 +17753,18 @@
         <f>IF(L130="","",TEXT(L130,"ddd"))</f>
         <v/>
       </c>
-      <c r="N130" s="124" t="n"/>
+      <c r="N130" s="124" t="inlineStr">
+        <is>
+          <t>character story: Nia talks to herself by name, Milo thinks she's lost it</t>
+        </is>
+      </c>
       <c r="O130" s="124" t="n"/>
       <c r="P130" s="124" t="n"/>
-      <c r="Q130" s="124" t="n"/>
+      <c r="Q130" s="124" t="inlineStr">
+        <is>
+          <t>Kross, Bruehlman-Senecal, Park, Burson, Dougherty, Shablack, Bremner, Moser &amp; Ayduk 2014 JPSP 'Self-talk as a regulatory mechanism': Study 3, 89 students, 5-min speech prep; name/non-first-person group rated better by blind coders (p=.022), less shame and rumination; Study 4 less anticipatory anxiety — rascl.studentorg.berkeley.edu PDF, lsa.umich.edu 2014 news</t>
+        </is>
+      </c>
       <c r="R130" s="124" t="n"/>
       <c r="S130" s="126" t="n"/>
       <c r="T130" s="124" t="n"/>
@@ -17768,7 +17808,7 @@
       <c r="AN130" s="124" t="n"/>
       <c r="AO130" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>tedmg</t>
         </is>
       </c>
       <c r="AP130" s="129" t="n"/>
@@ -17813,7 +17853,7 @@
       </c>
       <c r="H131" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I131" s="124" t="n">
@@ -17834,10 +17874,18 @@
         <f>IF(L131="","",TEXT(L131,"ddd"))</f>
         <v/>
       </c>
-      <c r="N131" s="124" t="n"/>
+      <c r="N131" s="124" t="inlineStr">
+        <is>
+          <t>character story + numbered facts: Dev says nobody tells him what to choose</t>
+        </is>
+      </c>
       <c r="O131" s="124" t="n"/>
       <c r="P131" s="124" t="n"/>
-      <c r="Q131" s="124" t="n"/>
+      <c r="Q131" s="124" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Goldstein 2003 Science: online n=161, opt-in 42% / opt-out 82% / neutral 79% (journalofethics.ama-assn.org 2005-09); Iyengar &amp; Lepper 2000 jams 24 vs 6: ~3% vs ~30% of stoppers bought, Scheibehenne et al. 2010 meta-analysis ~zero average (said in script); Huber, Payne &amp; Puto 1982 decoy, qualitative only</t>
+        </is>
+      </c>
       <c r="R131" s="124" t="n"/>
       <c r="S131" s="126" t="n"/>
       <c r="T131" s="124" t="n"/>
@@ -17881,7 +17929,7 @@
       <c r="AN131" s="124" t="n"/>
       <c r="AO131" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>tedmg</t>
         </is>
       </c>
       <c r="AP131" s="129" t="n"/>

</xml_diff>

<commit_message>
scripts: 6 new (gratitude-visit, thirty-six-questions, lima-syndrome, maximizer-test, lower-voice, ikea-effect)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EKMmbmCx58zrbPUMeFSFSC
</commit_message>
<xml_diff>
--- a/shorts/Psychology_Shorts_Tracker.xlsx
+++ b/shorts/Psychology_Shorts_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Long form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Looks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shorts ideas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Act Scripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long form" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'3-Act Scripts'!$A$4:$J$718</definedName>
@@ -18022,7 +18022,7 @@
       </c>
       <c r="H132" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I132" s="124" t="n">
@@ -18043,10 +18043,18 @@
         <f>IF(L132="","",TEXT(L132,"ddd"))</f>
         <v/>
       </c>
-      <c r="N132" s="124" t="n"/>
+      <c r="N132" s="124" t="inlineStr">
+        <is>
+          <t>surprising claim: ONE letter made people happier for a month; Omar + Grace story</t>
+        </is>
+      </c>
       <c r="O132" s="124" t="n"/>
       <c r="P132" s="124" t="n"/>
-      <c r="Q132" s="124" t="n"/>
+      <c r="Q132" s="124" t="inlineStr">
+        <is>
+          <t>Seligman, Steen, Park &amp; Peterson 2005 Am Psychol 'Positive Psychology Progress': gratitude visit gave the greatest happiness benefit at one month, back to baseline by six months (Greater Good Science Center summary ggia.berkeley.edu/practice/gratitude_letter). No sample-size numbers used.</t>
+        </is>
+      </c>
       <c r="R132" s="124" t="n"/>
       <c r="S132" s="126" t="n"/>
       <c r="T132" s="124" t="n"/>
@@ -18135,7 +18143,7 @@
       </c>
       <c r="H133" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I133" s="124" t="n">
@@ -18156,10 +18164,18 @@
         <f>IF(L133="","",TEXT(L133,"ddd"))</f>
         <v/>
       </c>
-      <c r="N133" s="124" t="n"/>
+      <c r="N133" s="124" t="inlineStr">
+        <is>
+          <t>character story: Otto has sat next to Arthur for TEN years</t>
+        </is>
+      </c>
       <c r="O133" s="124" t="n"/>
       <c r="P133" s="124" t="n"/>
-      <c r="Q133" s="124" t="n"/>
+      <c r="Q133" s="124" t="inlineStr">
+        <is>
+          <t>Aron, Melinat, Aron, Vallone &amp; Bator 1997 PSPB abstract: 45-min escalating self-disclosure tasks gave greater post-interaction closeness than small-talk tasks (stafforini.com PDF abstract); 36 questions in three sets of 12 (ggia.berkeley.edu). No closeness numbers used.</t>
+        </is>
+      </c>
       <c r="R133" s="124" t="n"/>
       <c r="S133" s="126" t="n"/>
       <c r="T133" s="124" t="n"/>
@@ -18203,7 +18219,7 @@
       <c r="AN133" s="124" t="n"/>
       <c r="AO133" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>retro</t>
         </is>
       </c>
       <c r="AP133" s="129" t="n"/>
@@ -18248,7 +18264,7 @@
       </c>
       <c r="H134" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I134" s="124" t="n">
@@ -18269,10 +18285,18 @@
         <f>IF(L134="","",TEXT(L134,"ddd"))</f>
         <v/>
       </c>
-      <c r="N134" s="124" t="n"/>
+      <c r="N134" s="124" t="inlineStr">
+        <is>
+          <t>character story: Rosa must keep Milo and June LOCKED in</t>
+        </is>
+      </c>
       <c r="O134" s="124" t="n"/>
       <c r="P134" s="124" t="n"/>
-      <c r="Q134" s="124" t="n"/>
+      <c r="Q134" s="124" t="inlineStr">
+        <is>
+          <t>Japanese embassy hostage crisis (Wikipedia): began 17 Dec 1996, 600+ hostages, releases of 38/255/20 in the first 11 days, 72 held to 22 Apr 1997; Healthline: term named for captors growing sympathetic, research scarce. Script says one case, not lab studies.</t>
+        </is>
+      </c>
       <c r="R134" s="124" t="n"/>
       <c r="S134" s="126" t="n"/>
       <c r="T134" s="124" t="n"/>
@@ -18316,7 +18340,7 @@
       <c r="AN134" s="124" t="n"/>
       <c r="AO134" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>tedmg</t>
         </is>
       </c>
       <c r="AP134" s="129" t="n"/>
@@ -18361,7 +18385,7 @@
       </c>
       <c r="H135" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I135" s="124" t="n">
@@ -18382,10 +18406,18 @@
         <f>IF(L135="","",TEXT(L135,"ddd"))</f>
         <v/>
       </c>
-      <c r="N135" s="124" t="n"/>
+      <c r="N135" s="124" t="inlineStr">
+        <is>
+          <t>question to viewer: do you always hunt for the BEST option? Sam vs Leo</t>
+        </is>
+      </c>
       <c r="O135" s="124" t="n"/>
       <c r="P135" s="124" t="n"/>
-      <c r="Q135" s="124" t="n"/>
+      <c r="Q135" s="124" t="inlineStr">
+        <is>
+          <t>Schwartz, Ward, Monterosso, Lyubomirsky, White &amp; Lehman 2002 JPSP (works.swarthmore.edu/fac-psychology/101): maximizers report less happiness, optimism, self-esteem, life satisfaction; more depression, perfectionism, regret. Correlational; no numbers used.</t>
+        </is>
+      </c>
       <c r="R135" s="124" t="n"/>
       <c r="S135" s="126" t="n"/>
       <c r="T135" s="124" t="n"/>
@@ -18474,7 +18506,7 @@
       </c>
       <c r="H136" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I136" s="124" t="n">
@@ -18495,10 +18527,18 @@
         <f>IF(L136="","",TEXT(L136,"ddd"))</f>
         <v/>
       </c>
-      <c r="N136" s="124" t="n"/>
+      <c r="N136" s="124" t="inlineStr">
+        <is>
+          <t>surprising claim: same speech, only the PITCH changed; Priya + Grace</t>
+        </is>
+      </c>
       <c r="O136" s="124" t="n"/>
       <c r="P136" s="124" t="n"/>
-      <c r="Q136" s="124" t="n"/>
+      <c r="Q136" s="124" t="inlineStr">
+        <is>
+          <t>Klofstad, Anderson &amp; Peters 2012 Proc R Soc B (Duke Today 2012-03, ScienceDaily 2012-03-13): pitch-edited 'I urge you to vote for me this November'; men and women chose lower-pitched male and female candidates; lower female voices rated stronger/more competent/trustworthy by both sexes, lower male voices stronger/more competent by men. No % reported, none used; lab-only caveat in script.</t>
+        </is>
+      </c>
       <c r="R136" s="124" t="n"/>
       <c r="S136" s="126" t="n"/>
       <c r="T136" s="124" t="n"/>
@@ -18587,7 +18627,7 @@
       </c>
       <c r="H137" s="123" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Scripted</t>
         </is>
       </c>
       <c r="I137" s="124" t="n">
@@ -18608,10 +18648,18 @@
         <f>IF(L137="","",TEXT(L137,"ddd"))</f>
         <v/>
       </c>
-      <c r="N137" s="124" t="n"/>
+      <c r="N137" s="124" t="inlineStr">
+        <is>
+          <t>character story: Nia spent six hours building a SHELF</t>
+        </is>
+      </c>
       <c r="O137" s="124" t="n"/>
       <c r="P137" s="124" t="n"/>
-      <c r="Q137" s="124" t="n"/>
+      <c r="Q137" s="124" t="inlineStr">
+        <is>
+          <t>Norton, Mochon &amp; Ariely (HBS WP 2011; J Consumer Psychol 2012): IKEA box builders paid 63% more than for pre-assembled (Wikipedia IKEA effect; coglode); completion required for the effect (Colby CogBlog).</t>
+        </is>
+      </c>
       <c r="R137" s="124" t="n"/>
       <c r="S137" s="126" t="n"/>
       <c r="T137" s="124" t="n"/>
@@ -18655,7 +18703,7 @@
       <c r="AN137" s="124" t="n"/>
       <c r="AO137" s="124" t="inlineStr">
         <is>
-          <t>ted2</t>
+          <t>tedmg</t>
         </is>
       </c>
       <c r="AP137" s="129" t="n"/>

</xml_diff>